<commit_message>
Add benchmarking reports baselines
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6ED05F-2253-4F12-B152-806F968C9730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4934EBB0-5B46-4943-BCB8-F2406F249390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="M6" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Functions</t>
   </si>
@@ -33,15 +44,9 @@
     <t>Total_Requests</t>
   </si>
   <si>
-    <t>Baseline: Without Middleware</t>
-  </si>
-  <si>
     <t>Response_Time_Metric: milliseconds</t>
   </si>
   <si>
-    <t>Baseline_Response_Time</t>
-  </si>
-  <si>
     <t>M6: Middleware with 6 database servers</t>
   </si>
   <si>
@@ -54,18 +59,6 @@
     <t>M1: Middleware with 1 database server</t>
   </si>
   <si>
-    <t>M6</t>
-  </si>
-  <si>
-    <t>M4</t>
-  </si>
-  <si>
-    <t>M2</t>
-  </si>
-  <si>
-    <t>M1</t>
-  </si>
-  <si>
     <t>Get-Range</t>
   </si>
   <si>
@@ -90,19 +83,43 @@
     <t>Cool-Down_Time: 1 Minute</t>
   </si>
   <si>
-    <t>SetSingle</t>
-  </si>
-  <si>
-    <t>SetMultiples</t>
-  </si>
-  <si>
-    <t>GetSingle</t>
-  </si>
-  <si>
-    <t>GetMultiples</t>
-  </si>
-  <si>
     <t>Average_Response_Time_Per_Requests: M1-M6</t>
+  </si>
+  <si>
+    <t>Set</t>
+  </si>
+  <si>
+    <t>Get</t>
+  </si>
+  <si>
+    <t>Throughput</t>
+  </si>
+  <si>
+    <t>Baseline:Response_Time</t>
+  </si>
+  <si>
+    <t>Baseline:Requests_Per_Second(RPS)</t>
+  </si>
+  <si>
+    <t>Baseline:Client Connected to Single Redis Instance Without Middleware</t>
+  </si>
+  <si>
+    <t>M6-DB:Average_Response_Time</t>
+  </si>
+  <si>
+    <t>M6-DB:Total_Response_Time</t>
+  </si>
+  <si>
+    <t>M6:Requests_Per_Second(RPS)</t>
+  </si>
+  <si>
+    <t>Client-M6:Average_Response_Time</t>
+  </si>
+  <si>
+    <t>M6 Internal Processing Time</t>
+  </si>
+  <si>
+    <t>Client-Middleware Response Time (Base Communication)</t>
   </si>
 </sst>
 </file>
@@ -429,72 +446,80 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.5703125" customWidth="1"/>
-    <col min="2" max="2" width="31.42578125" customWidth="1"/>
+    <col min="1" max="1" width="52.28515625" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" customWidth="1"/>
+    <col min="4" max="4" width="34.5703125" customWidth="1"/>
     <col min="5" max="5" width="27.28515625" customWidth="1"/>
     <col min="6" max="6" width="30.28515625" customWidth="1"/>
-    <col min="7" max="7" width="20.5703125" customWidth="1"/>
+    <col min="7" max="7" width="35.7109375" customWidth="1"/>
+    <col min="8" max="8" width="37.85546875" customWidth="1"/>
+    <col min="9" max="9" width="31.28515625" customWidth="1"/>
+    <col min="10" max="10" width="56.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="C1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
         <v>18</v>
       </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -502,61 +527,124 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B11">
-        <v>6048</v>
+        <v>11942</v>
       </c>
       <c r="D11">
-        <v>10.384393271080899</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9196.4009272318253</v>
+      </c>
+      <c r="E11">
+        <v>1018360.3970850317</v>
+      </c>
+      <c r="F11">
+        <v>85.275531492633704</v>
+      </c>
+      <c r="G11">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="I11">
+        <f>F11-G11</f>
+        <v>81.85114489524743</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B12">
-        <v>5894</v>
+        <v>12491</v>
       </c>
       <c r="D12">
-        <v>74.891138221552794</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>9183.8560924287813</v>
+      </c>
+      <c r="E12">
+        <v>475452.95695960498</v>
+      </c>
+      <c r="F12">
+        <v>38.063642379281497</v>
+      </c>
+      <c r="G12">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="I12">
+        <f t="shared" ref="I12:I14" si="0">F12-G12</f>
+        <v>34.631419436413125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>9795</v>
+      </c>
+      <c r="D13">
+        <v>9183.9702836643701</v>
+      </c>
+      <c r="E13">
+        <v>567651.17784589506</v>
+      </c>
+      <c r="F13">
+        <v>57.953157513618699</v>
+      </c>
+      <c r="G13">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="0"/>
+        <v>54.549991659125141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>14</v>
+        <v>8</v>
+      </c>
+      <c r="B14">
+        <v>10671</v>
+      </c>
+      <c r="D14">
+        <v>9165.6664454259699</v>
+      </c>
+      <c r="E14">
+        <v>582540.25277588505</v>
+      </c>
+      <c r="F14">
+        <v>54.590971115723399</v>
+      </c>
+      <c r="G14">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="0"/>
+        <v>51.150896611061086</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 6 DBs configs for profiling
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4934EBB0-5B46-4943-BCB8-F2406F249390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B05B56-FCC5-4E7A-B686-241D1D656BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>Functions</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Baseline:Client Connected to Single Redis Instance Without Middleware</t>
   </si>
   <si>
-    <t>M6-DB:Average_Response_Time</t>
-  </si>
-  <si>
     <t>M6-DB:Total_Response_Time</t>
   </si>
   <si>
@@ -120,13 +117,31 @@
   </si>
   <si>
     <t>Client-Middleware Response Time (Base Communication)</t>
+  </si>
+  <si>
+    <t>M1:Requests_Per_Second(RPS)</t>
+  </si>
+  <si>
+    <t>Client-M1:Average_Response_Time</t>
+  </si>
+  <si>
+    <t>M1-DB:Total_Response_Time</t>
+  </si>
+  <si>
+    <t>M1-DB:Average_Response_Time_Per_Key_Value_Pair</t>
+  </si>
+  <si>
+    <t>M1 Internal Processing Time</t>
+  </si>
+  <si>
+    <t>M6-DB:Average_Response_Time_Per_Key_Value_Pair</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,16 +157,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -159,16 +187,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -446,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.28515625" customWidth="1"/>
@@ -454,7 +500,7 @@
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="34.5703125" customWidth="1"/>
     <col min="5" max="5" width="27.28515625" customWidth="1"/>
-    <col min="6" max="6" width="30.28515625" customWidth="1"/>
+    <col min="6" max="6" width="53" customWidth="1"/>
     <col min="7" max="7" width="35.7109375" customWidth="1"/>
     <col min="8" max="8" width="37.85546875" customWidth="1"/>
     <col min="9" max="9" width="31.28515625" customWidth="1"/>
@@ -527,28 +573,28 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E10" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" t="s">
-        <v>19</v>
-      </c>
-      <c r="H10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="J10" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -645,6 +691,118 @@
       <c r="I14">
         <f t="shared" si="0"/>
         <v>51.150896611061086</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>4475</v>
+      </c>
+      <c r="D18">
+        <v>8922.0126792951196</v>
+      </c>
+      <c r="E18">
+        <v>97660.997001454205</v>
+      </c>
+      <c r="F18">
+        <v>53.670286270020398</v>
+      </c>
+      <c r="G18">
+        <v>3.4243865973862802</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>4428</v>
+      </c>
+      <c r="D19">
+        <v>8905.3457502867641</v>
+      </c>
+      <c r="E19">
+        <v>86850.022056140006</v>
+      </c>
+      <c r="F19">
+        <v>19.613826119272801</v>
+      </c>
+      <c r="G19">
+        <v>3.4322229428683699</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20">
+        <v>2210</v>
+      </c>
+      <c r="D20">
+        <v>8917.6700800189392</v>
+      </c>
+      <c r="E20">
+        <v>54144.182988442401</v>
+      </c>
+      <c r="F20">
+        <v>24.499630311512401</v>
+      </c>
+      <c r="G20">
+        <v>3.4031658544935599</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21">
+        <v>2230</v>
+      </c>
+      <c r="D21">
+        <v>8905.8606007410399</v>
+      </c>
+      <c r="E21">
+        <v>50546.400175429801</v>
+      </c>
+      <c r="F21">
+        <v>22.6665471638699</v>
+      </c>
+      <c r="G21">
+        <v>3.4400745046623098</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize logs and reports
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8244B535-C10E-4BEC-B89F-D97E3F5807AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1143C2-5AE7-43E3-B107-3BE6637F0207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M6" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
   <si>
     <t>Functions</t>
   </si>
@@ -159,6 +160,45 @@
   </si>
   <si>
     <t>Average: 8913.04358205774</t>
+  </si>
+  <si>
+    <t>get_range</t>
+  </si>
+  <si>
+    <t>del_single</t>
+  </si>
+  <si>
+    <t>Client_Instances = 1</t>
+  </si>
+  <si>
+    <t>Baseline: Response_Time</t>
+  </si>
+  <si>
+    <t>Logs_Evaluation_Time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 minute </t>
+  </si>
+  <si>
+    <t>M1: Internal_Response_Time</t>
+  </si>
+  <si>
+    <t>M2:  Internal_Response_Time</t>
+  </si>
+  <si>
+    <t>M4: Internal_Response_Time</t>
+  </si>
+  <si>
+    <t>M6: Internal_Response_Time</t>
+  </si>
+  <si>
+    <t>set</t>
+  </si>
+  <si>
+    <t>get</t>
+  </si>
+  <si>
+    <t>del</t>
   </si>
 </sst>
 </file>
@@ -166,8 +206,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.00000000"/>
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -241,22 +281,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,10 +632,10 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="3"/>
+      <c r="G5" s="8"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -667,7 +708,7 @@
       <c r="G11">
         <v>85.275531492633704</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="3">
         <v>3.4243865973862802</v>
       </c>
       <c r="J11">
@@ -691,7 +732,7 @@
       <c r="G12">
         <v>38.063642379281497</v>
       </c>
-      <c r="H12" s="4">
+      <c r="H12" s="3">
         <v>3.4322229428683699</v>
       </c>
       <c r="J12">
@@ -715,7 +756,7 @@
       <c r="G13">
         <v>57.953157513618699</v>
       </c>
-      <c r="H13" s="4">
+      <c r="H13" s="3">
         <v>3.4031658544935599</v>
       </c>
       <c r="J13">
@@ -739,7 +780,7 @@
       <c r="G14">
         <v>54.590971115723399</v>
       </c>
-      <c r="H14" s="4">
+      <c r="H14" s="3">
         <v>3.4400745046623098</v>
       </c>
       <c r="J14">
@@ -797,13 +838,13 @@
         <f>D19/B19</f>
         <v>1.6594462344080945</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="5">
         <v>120887.90003769091</v>
       </c>
       <c r="G19">
         <v>53.670286270020398</v>
       </c>
-      <c r="H19" s="4">
+      <c r="H19" s="3">
         <v>3.4243865973862802</v>
       </c>
       <c r="J19">
@@ -818,7 +859,7 @@
       <c r="B20">
         <v>10743</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>35.806887798237</v>
       </c>
       <c r="D20">
@@ -834,7 +875,7 @@
       <c r="G20">
         <v>19.613826119272801</v>
       </c>
-      <c r="H20" s="4">
+      <c r="H20" s="3">
         <v>3.4322229428683699</v>
       </c>
       <c r="J20">
@@ -856,7 +897,7 @@
         <v>8917.6700800189392</v>
       </c>
       <c r="E21">
-        <f t="shared" ref="E20:E22" si="2">D21/B21</f>
+        <f t="shared" ref="E21:E22" si="2">D21/B21</f>
         <v>1.6778306829762821</v>
       </c>
       <c r="F21">
@@ -865,7 +906,7 @@
       <c r="G21">
         <v>24.499630311512401</v>
       </c>
-      <c r="H21" s="4">
+      <c r="H21" s="3">
         <v>3.4031658544935599</v>
       </c>
       <c r="J21">
@@ -896,7 +937,7 @@
       <c r="G22">
         <v>22.6665471638699</v>
       </c>
-      <c r="H22" s="4">
+      <c r="H22" s="3">
         <v>3.4400745046623098</v>
       </c>
       <c r="J22">
@@ -916,13 +957,13 @@
         <f>SUM(C19:C22)</f>
         <v>106.90737467452772</v>
       </c>
-      <c r="H23" s="4"/>
+      <c r="H23" s="3"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -984,7 +1025,7 @@
       <c r="G27">
         <v>89.672978634367993</v>
       </c>
-      <c r="H27" s="4">
+      <c r="H27" s="3">
         <v>3.4243865973862802</v>
       </c>
       <c r="J27">
@@ -1002,12 +1043,12 @@
       <c r="C28">
         <v>31.156985334915301</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="5">
         <f>SUM(D26:D27)</f>
         <v>20541.8354965254</v>
       </c>
       <c r="E28">
-        <f t="shared" ref="E28:E31" si="3">D28/B28</f>
+        <f t="shared" ref="E28:E30" si="3">D28/B28</f>
         <v>2.1979280437112561</v>
       </c>
       <c r="F28">
@@ -1016,7 +1057,7 @@
       <c r="G28">
         <v>38.506308392196701</v>
       </c>
-      <c r="H28" s="4">
+      <c r="H28" s="3">
         <v>3.4322229428683699</v>
       </c>
       <c r="J28">
@@ -1047,7 +1088,7 @@
       <c r="G29">
         <v>49.572030971004097</v>
       </c>
-      <c r="H29" s="4">
+      <c r="H29" s="3">
         <v>3.4031658544935599</v>
       </c>
       <c r="J29">
@@ -1078,7 +1119,7 @@
       <c r="G30">
         <v>50.046090764103504</v>
       </c>
-      <c r="H30" s="4">
+      <c r="H30" s="3">
         <v>3.4400745046623098</v>
       </c>
       <c r="J30">
@@ -1102,10 +1143,10 @@
       <c r="E31" s="1"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1116,10 +1157,10 @@
       <c r="C41" s="1"/>
     </row>
     <row r="44" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="G44" s="6"/>
+      <c r="G44" s="5"/>
     </row>
     <row r="49" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F49" s="6"/>
+      <c r="F49" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1128,4 +1169,183 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="6">
+        <v>17.337385863109212</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1018360.3970850317</v>
+      </c>
+      <c r="E11" s="6">
+        <v>85.275531492633704</v>
+      </c>
+      <c r="F11" s="9">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6">
+        <f>E11-(2*F11)</f>
+        <v>78.426758297861142</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="6">
+        <v>13.554599573799599</v>
+      </c>
+      <c r="D12" s="6">
+        <v>475452.95695960498</v>
+      </c>
+      <c r="E12" s="6">
+        <v>38.063642379281497</v>
+      </c>
+      <c r="F12" s="9">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6">
+        <f t="shared" ref="H12:H14" si="0">E12-(2*F12)</f>
+        <v>31.199196493544758</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="6">
+        <v>3.5198966997507801</v>
+      </c>
+      <c r="D13" s="6">
+        <v>567651.17784589506</v>
+      </c>
+      <c r="E13" s="6">
+        <v>57.953157513618699</v>
+      </c>
+      <c r="F13" s="9">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6">
+        <f t="shared" si="0"/>
+        <v>51.146825804631575</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14">
+        <v>1.9306251285782701</v>
+      </c>
+      <c r="D14" s="6">
+        <v>582540.25277588505</v>
+      </c>
+      <c r="E14" s="6">
+        <v>54.590971115723399</v>
+      </c>
+      <c r="F14" s="9">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6">
+        <f t="shared" si="0"/>
+        <v>47.71082210639878</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C28" s="6">
+        <v>0.54063046130762304</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C29" s="6">
+        <v>34.134141264910802</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <f>(C28+C29)/2</f>
+        <v>17.337385863109212</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add execution time m_ware
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1143C2-5AE7-43E3-B107-3BE6637F0207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D937AA64-4D6A-4127-92F5-498C61B73ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="29040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="M6" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="96">
   <si>
     <t>Functions</t>
   </si>
@@ -192,13 +192,139 @@
     <t>M6: Internal_Response_Time</t>
   </si>
   <si>
-    <t>set</t>
-  </si>
-  <si>
-    <t>get</t>
-  </si>
-  <si>
-    <t>del</t>
+    <t>set_single</t>
+  </si>
+  <si>
+    <t>set_multiple</t>
+  </si>
+  <si>
+    <t>get_single</t>
+  </si>
+  <si>
+    <t>get_multiple</t>
+  </si>
+  <si>
+    <t>del_multiple</t>
+  </si>
+  <si>
+    <t>Communication_Time_gRPC</t>
+  </si>
+  <si>
+    <t>Client_Instances = 10</t>
+  </si>
+  <si>
+    <t>Client_Instances = 100</t>
+  </si>
+  <si>
+    <t>M1: Processing Time</t>
+  </si>
+  <si>
+    <t>M2: Processing Time</t>
+  </si>
+  <si>
+    <t>M4: Processing Time</t>
+  </si>
+  <si>
+    <t>M6: Processing Time</t>
+  </si>
+  <si>
+    <t>C1-M1</t>
+  </si>
+  <si>
+    <t>C1-M2</t>
+  </si>
+  <si>
+    <t>C1-M4</t>
+  </si>
+  <si>
+    <t>C1-M6</t>
+  </si>
+  <si>
+    <t>Baseline=Without Middleware</t>
+  </si>
+  <si>
+    <t>Constant Workload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Response Time Evaluation </t>
+  </si>
+  <si>
+    <t>3 minute</t>
+  </si>
+  <si>
+    <t>Warmup = 10 seconds</t>
+  </si>
+  <si>
+    <t>Cooldown = 20 seconds</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average_Response_Time_Metric: </t>
+  </si>
+  <si>
+    <t>milliseconds</t>
+  </si>
+  <si>
+    <t>C10-M1</t>
+  </si>
+  <si>
+    <t>C10-M2</t>
+  </si>
+  <si>
+    <t>C10-M4</t>
+  </si>
+  <si>
+    <t>C10-M6</t>
+  </si>
+  <si>
+    <t>C100-M1</t>
+  </si>
+  <si>
+    <t>C100-M2</t>
+  </si>
+  <si>
+    <t>C100-M4</t>
+  </si>
+  <si>
+    <t>C100-M6</t>
+  </si>
+  <si>
+    <t>Average Middleware Processing Time</t>
+  </si>
+  <si>
+    <t>Asynchronous Calls</t>
+  </si>
+  <si>
+    <t>Synchronous Calls(Execution_Times)</t>
+  </si>
+  <si>
+    <t>10_Clients</t>
+  </si>
+  <si>
+    <t>100_Clients</t>
+  </si>
+  <si>
+    <t>Processing_Time</t>
+  </si>
+  <si>
+    <t>M-DB (M6)</t>
+  </si>
+  <si>
+    <t>Total Response Time</t>
+  </si>
+  <si>
+    <t>Calculated</t>
+  </si>
+  <si>
+    <t>Total Waiting Time</t>
+  </si>
+  <si>
+    <t>Client-M(gRPC)</t>
+  </si>
+  <si>
+    <t>Overhead</t>
   </si>
 </sst>
 </file>
@@ -209,7 +335,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.00000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,8 +359,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -250,6 +383,11 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -277,11 +415,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
@@ -294,12 +433,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="4" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
   </cellStyles>
@@ -623,34 +765,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
+      <c r="G5" s="11"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
@@ -1173,19 +1292,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="34.28515625" customWidth="1"/>
+    <col min="12" max="15" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1193,155 +1314,1733 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="G11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="6">
-        <v>17.337385863109212</v>
-      </c>
-      <c r="D11" s="6">
-        <v>1018360.3970850317</v>
-      </c>
-      <c r="E11" s="6">
-        <v>85.275531492633704</v>
-      </c>
-      <c r="F11" s="9">
+      <c r="B12">
+        <v>1.7484884995680501</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.52516379831418403</v>
+      </c>
+      <c r="D12">
+        <v>0.55217083894890695</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.56642264724104496</v>
+      </c>
+      <c r="F12">
+        <v>0.53922044867672203</v>
+      </c>
+      <c r="G12" s="8">
         <v>3.4243865973862802</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6">
-        <f>E11-(2*F11)</f>
-        <v>78.426758297861142</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="H12">
+        <v>3.9895902707595199</v>
+      </c>
+      <c r="I12">
+        <v>4.02605646143118</v>
+      </c>
+      <c r="J12">
+        <v>4.0353076186722596</v>
+      </c>
+      <c r="K12">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="L12" s="6">
+        <f>(H12-C12-G12)</f>
+        <v>4.0039875059055596E-2</v>
+      </c>
+      <c r="M12" s="6">
+        <f>(I12-D12-G12)</f>
+        <v>4.9499025095992799E-2</v>
+      </c>
+      <c r="N12" s="6">
+        <f>(J12-E12-G12)</f>
+        <v>4.4498374044934508E-2</v>
+      </c>
+      <c r="O12" s="6">
+        <f>(K12-F12-G12)</f>
+        <v>4.1486054322107613E-2</v>
+      </c>
+      <c r="P12" s="9">
+        <f>(L12+M12+N12+O12)/4</f>
+        <v>4.3880832130522629E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="6">
-        <v>13.554599573799599</v>
-      </c>
-      <c r="D12" s="6">
-        <v>475452.95695960498</v>
-      </c>
-      <c r="E12" s="6">
-        <v>38.063642379281497</v>
-      </c>
-      <c r="F12" s="9">
-        <v>3.4322229428683699</v>
-      </c>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6">
-        <f t="shared" ref="H12:H14" si="0">E12-(2*F12)</f>
-        <v>31.199196493544758</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="6">
-        <v>3.5198966997507801</v>
+      <c r="B13">
+        <v>6683.5777209355201</v>
+      </c>
+      <c r="C13">
+        <v>32.977948012191398</v>
       </c>
       <c r="D13" s="6">
-        <v>567651.17784589506</v>
+        <v>37.627384497258902</v>
       </c>
       <c r="E13" s="6">
-        <v>57.953157513618699</v>
-      </c>
-      <c r="F13" s="9">
-        <v>3.4031658544935599</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6">
-        <f t="shared" si="0"/>
-        <v>51.146825804631575</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>40.476617648566901</v>
+      </c>
+      <c r="F13">
+        <v>45.082622893090097</v>
+      </c>
+      <c r="G13" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="H13">
+        <v>41.8466371823881</v>
+      </c>
+      <c r="I13">
+        <v>45.799138335569502</v>
+      </c>
+      <c r="J13">
+        <v>48.675797406364801</v>
+      </c>
+      <c r="K13">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="L13" s="6">
+        <f t="shared" ref="L13:L18" si="0">(H13-C13-G13)</f>
+        <v>5.4443025728104226</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" ref="M13:M18" si="1">(I13-D13-G13)</f>
+        <v>4.7473672409243202</v>
+      </c>
+      <c r="N13" s="6">
+        <f t="shared" ref="N13:N18" si="2">(J13-E13-G13)</f>
+        <v>4.7747931604116198</v>
+      </c>
+      <c r="O13" s="6">
+        <f t="shared" ref="O13:O18" si="3">(K13-F13-G13)</f>
+        <v>6.0045148916153233</v>
+      </c>
+      <c r="P13" s="9">
+        <f t="shared" ref="P13:P18" si="4">(L13+M13+N13+O13)/4</f>
+        <v>5.2427444664404215</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>53</v>
       </c>
+      <c r="B14">
+        <v>7.7534715334574296</v>
+      </c>
       <c r="C14">
-        <v>1.9306251285782701</v>
+        <v>0.49840760395546102</v>
       </c>
       <c r="D14" s="6">
-        <v>582540.25277588505</v>
+        <v>0.42816291537031098</v>
       </c>
       <c r="E14" s="6">
-        <v>54.590971115723399</v>
-      </c>
-      <c r="F14" s="9">
+        <v>0.53777458074084705</v>
+      </c>
+      <c r="F14">
+        <v>0.54917054483667005</v>
+      </c>
+      <c r="G14" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H14">
+        <v>4.0147860416504804</v>
+      </c>
+      <c r="I14">
+        <v>4.1628384834501704</v>
+      </c>
+      <c r="J14">
+        <v>4.1707241313894299</v>
+      </c>
+      <c r="K14">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="L14" s="6">
+        <f t="shared" si="0"/>
+        <v>8.4155494826649413E-2</v>
+      </c>
+      <c r="M14" s="6">
+        <f t="shared" si="1"/>
+        <v>0.30245262521148941</v>
+      </c>
+      <c r="N14" s="6">
+        <f t="shared" si="2"/>
+        <v>0.20072660778021278</v>
+      </c>
+      <c r="O14" s="6">
+        <f t="shared" si="3"/>
+        <v>9.6146269678780261E-2</v>
+      </c>
+      <c r="P14" s="9">
+        <f t="shared" si="4"/>
+        <v>0.17087024937428297</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15">
+        <v>5248.1240630149796</v>
+      </c>
+      <c r="C15">
+        <v>25.759887776849901</v>
+      </c>
+      <c r="D15" s="6">
+        <v>27.827213474541299</v>
+      </c>
+      <c r="E15" s="6">
+        <v>32.509592705689798</v>
+      </c>
+      <c r="F15">
+        <v>34.394685960258002</v>
+      </c>
+      <c r="G15" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H15">
+        <v>38.3633321341607</v>
+      </c>
+      <c r="I15">
+        <v>42.259016332980003</v>
+      </c>
+      <c r="J15">
+        <v>44.808815805147901</v>
+      </c>
+      <c r="K15">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="L15" s="6">
+        <f t="shared" si="0"/>
+        <v>9.1712214144424298</v>
+      </c>
+      <c r="M15" s="6">
+        <f t="shared" si="1"/>
+        <v>10.999579915570335</v>
+      </c>
+      <c r="N15" s="6">
+        <f t="shared" si="2"/>
+        <v>8.8670001565897341</v>
+      </c>
+      <c r="O15" s="6">
+        <f t="shared" si="3"/>
+        <v>9.3623754654125282</v>
+      </c>
+      <c r="P15" s="9">
+        <f t="shared" si="4"/>
+        <v>9.6000442380037558</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16">
+        <v>526.84138371394204</v>
+      </c>
+      <c r="C16">
+        <v>3.52255095970304</v>
+      </c>
+      <c r="D16" s="6">
+        <v>4.2291533285572704</v>
+      </c>
+      <c r="E16" s="6">
+        <v>5.3097894837627804</v>
+      </c>
+      <c r="F16">
+        <v>6.2376752522495398</v>
+      </c>
+      <c r="G16" s="8">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="H16">
+        <v>7.9163517599320397</v>
+      </c>
+      <c r="I16">
+        <v>8.8410975673074592</v>
+      </c>
+      <c r="J16">
+        <v>9.8086684739508598</v>
+      </c>
+      <c r="K16">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="L16" s="6">
+        <f t="shared" si="0"/>
+        <v>0.9906349457354402</v>
+      </c>
+      <c r="M16" s="6">
+        <f t="shared" si="1"/>
+        <v>1.2087783842566289</v>
+      </c>
+      <c r="N16" s="6">
+        <f t="shared" si="2"/>
+        <v>1.0957131356945196</v>
+      </c>
+      <c r="O16" s="6">
+        <f t="shared" si="3"/>
+        <v>1.567547813893901</v>
+      </c>
+      <c r="P16" s="9">
+        <f t="shared" si="4"/>
+        <v>1.2156685698951224</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17">
+        <v>1.6942660013834601</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.49062787411620901</v>
+      </c>
+      <c r="D17" s="6">
+        <v>0.42316263608524202</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0.53834092805300005</v>
+      </c>
+      <c r="F17">
+        <v>0.54279469219126897</v>
+      </c>
+      <c r="G17" s="8">
         <v>3.4400745046623098</v>
       </c>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6">
+      <c r="H17">
+        <v>4.0209035037549397</v>
+      </c>
+      <c r="I17">
+        <v>4.1352269590162702</v>
+      </c>
+      <c r="J17">
+        <v>4.0890994634011797</v>
+      </c>
+      <c r="K17">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="L17" s="6">
         <f t="shared" si="0"/>
-        <v>47.71082210639878</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+        <v>9.0201124976420743E-2</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="1"/>
+        <v>0.2719898182687186</v>
+      </c>
+      <c r="N17" s="6">
+        <f t="shared" si="2"/>
+        <v>0.11068403068586985</v>
+      </c>
+      <c r="O17" s="6">
+        <f t="shared" si="3"/>
+        <v>0.12456650453927143</v>
+      </c>
+      <c r="P17" s="9">
+        <f t="shared" si="4"/>
+        <v>0.14936036961757015</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18">
+        <v>2.2942038143382302</v>
+      </c>
+      <c r="C18">
+        <v>3.1790446098824598</v>
+      </c>
+      <c r="D18">
+        <v>3.5695951125117098</v>
+      </c>
+      <c r="E18">
+        <v>4.99549014023889</v>
+      </c>
+      <c r="F18">
+        <v>5.9257052455949104</v>
+      </c>
+      <c r="G18" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="H18">
+        <v>6.9167933755607498</v>
+      </c>
+      <c r="I18">
+        <v>7.6918990911074498</v>
+      </c>
+      <c r="J18">
+        <v>8.6418529562595499</v>
+      </c>
+      <c r="K18">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="L18" s="6">
+        <f t="shared" si="0"/>
+        <v>0.29767426101598016</v>
+      </c>
+      <c r="M18" s="6">
+        <f t="shared" si="1"/>
+        <v>0.68222947393343025</v>
+      </c>
+      <c r="N18" s="6">
+        <f t="shared" si="2"/>
+        <v>0.20628831135835002</v>
+      </c>
+      <c r="O18" s="6">
+        <f t="shared" si="3"/>
+        <v>0.47330379379092902</v>
+      </c>
+      <c r="P18" s="9">
+        <f t="shared" si="4"/>
+        <v>0.41487396002467236</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O25" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26">
+        <v>95.74904649154</v>
+      </c>
+      <c r="C26" s="6">
+        <v>11.847161237319201</v>
+      </c>
+      <c r="D26">
+        <v>11.823772956803801</v>
+      </c>
+      <c r="E26" s="6">
+        <v>10.2693631465152</v>
+      </c>
+      <c r="F26">
+        <v>10.8891134198832</v>
+      </c>
+      <c r="G26" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="H26">
+        <v>104.206596222385</v>
+      </c>
+      <c r="I26">
+        <v>103.825935221908</v>
+      </c>
+      <c r="J26">
+        <v>100.11177985049</v>
+      </c>
+      <c r="K26">
+        <v>93.901651246207095</v>
+      </c>
+      <c r="L26" s="6">
+        <f>(H26-C26-G26)</f>
+        <v>88.935048387679529</v>
+      </c>
+      <c r="M26" s="6">
+        <f>(I26-D26-G26)</f>
+        <v>88.57777566771793</v>
+      </c>
+      <c r="N26" s="6">
+        <f>(J26-E26-G26)</f>
+        <v>86.418030106588517</v>
+      </c>
+      <c r="O26" s="6">
+        <f>(K26-F26-G26)</f>
+        <v>79.588151228937619</v>
+      </c>
+      <c r="P26" s="9">
+        <f>(L26+M26+N26+O26)/4</f>
+        <v>85.879751347730888</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27">
+        <v>19995.0293793397</v>
+      </c>
+      <c r="C27">
+        <v>106.746648747265</v>
+      </c>
+      <c r="D27" s="6">
+        <v>106.067911051753</v>
+      </c>
+      <c r="E27" s="6">
+        <v>117.862013085952</v>
+      </c>
+      <c r="F27">
+        <v>123.020812843901</v>
+      </c>
+      <c r="G27" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="H27">
+        <v>198.878516435623</v>
+      </c>
+      <c r="I27">
+        <v>193.56502606161001</v>
+      </c>
+      <c r="J27">
+        <v>204.52682309183899</v>
+      </c>
+      <c r="K27">
+        <v>207.255575950614</v>
+      </c>
+      <c r="L27" s="6">
+        <f t="shared" ref="L27:L32" si="5">(H27-C27-G27)</f>
+        <v>88.707481090971726</v>
+      </c>
+      <c r="M27" s="6">
+        <f t="shared" ref="M27:M32" si="6">(I27-D27-G27)</f>
+        <v>84.072728412470738</v>
+      </c>
+      <c r="N27" s="6">
+        <f t="shared" ref="N27:N32" si="7">(J27-E27-G27)</f>
+        <v>83.240423408500718</v>
+      </c>
+      <c r="O27" s="6">
+        <f t="shared" ref="O27:O32" si="8">(K27-F27-G27)</f>
+        <v>80.81037650932673</v>
+      </c>
+      <c r="P27" s="9">
+        <f t="shared" ref="P27:P32" si="9">(L27+M27+N27+O27)/4</f>
+        <v>84.207752355317467</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28">
+        <v>138.138762226811</v>
+      </c>
+      <c r="C28">
+        <v>11.2682738745265</v>
+      </c>
+      <c r="D28" s="6">
+        <v>11.1841406676281</v>
+      </c>
+      <c r="E28" s="6">
+        <v>11.0258072177275</v>
+      </c>
+      <c r="F28">
+        <v>11.0649394160403</v>
+      </c>
+      <c r="G28" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H28">
+        <v>104.699721246761</v>
+      </c>
+      <c r="I28">
+        <v>103.176413636536</v>
+      </c>
+      <c r="J28">
+        <v>100.929154780147</v>
+      </c>
+      <c r="K28">
+        <v>95.117645530865104</v>
+      </c>
+      <c r="L28" s="6">
+        <f t="shared" si="5"/>
+        <v>89.999224429366137</v>
+      </c>
+      <c r="M28" s="6">
+        <f t="shared" si="6"/>
+        <v>88.560050026039534</v>
+      </c>
+      <c r="N28" s="6">
+        <f t="shared" si="7"/>
+        <v>86.471124619551134</v>
+      </c>
+      <c r="O28" s="6">
+        <f t="shared" si="8"/>
+        <v>80.620483171956437</v>
+      </c>
+      <c r="P28" s="9">
+        <f t="shared" si="9"/>
+        <v>86.412720561728307</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29">
+        <v>54800.687812623502</v>
+      </c>
+      <c r="C29">
+        <v>64.767009309883903</v>
+      </c>
+      <c r="D29" s="6">
+        <v>72.4037472078886</v>
+      </c>
+      <c r="E29" s="6">
+        <v>78.781588723359107</v>
+      </c>
+      <c r="F29">
+        <v>88.852265229373302</v>
+      </c>
+      <c r="G29" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H29">
+        <v>164.52485036118699</v>
+      </c>
+      <c r="I29">
+        <v>172.540658884236</v>
+      </c>
+      <c r="J29">
+        <v>183.230999074528</v>
+      </c>
+      <c r="K29">
+        <v>182.358312283896</v>
+      </c>
+      <c r="L29" s="6">
+        <f t="shared" si="5"/>
+        <v>96.325618108434725</v>
+      </c>
+      <c r="M29" s="6">
+        <f t="shared" si="6"/>
+        <v>96.704688733479031</v>
+      </c>
+      <c r="N29" s="6">
+        <f t="shared" si="7"/>
+        <v>101.01718740830053</v>
+      </c>
+      <c r="O29" s="6">
+        <f t="shared" si="8"/>
+        <v>90.073824111654332</v>
+      </c>
+      <c r="P29" s="9">
+        <f t="shared" si="9"/>
+        <v>96.030329590467161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30">
+        <v>6011.8293762207004</v>
+      </c>
+      <c r="C30">
+        <v>13.7873021123293</v>
+      </c>
+      <c r="D30" s="6">
+        <v>22.490014621644601</v>
+      </c>
+      <c r="E30" s="6">
+        <v>37.305102812492102</v>
+      </c>
+      <c r="F30">
+        <v>54.420109575413903</v>
+      </c>
+      <c r="G30" s="8">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="H30">
+        <v>103.10741371392299</v>
+      </c>
+      <c r="I30">
+        <v>113.343025767809</v>
+      </c>
+      <c r="J30">
+        <v>128.083347378882</v>
+      </c>
+      <c r="K30">
+        <v>139.43136468744001</v>
+      </c>
+      <c r="L30" s="6">
+        <f t="shared" si="5"/>
+        <v>85.916945747100129</v>
+      </c>
+      <c r="M30" s="6">
+        <f t="shared" si="6"/>
+        <v>87.449845291670826</v>
+      </c>
+      <c r="N30" s="6">
+        <f t="shared" si="7"/>
+        <v>87.375078711896336</v>
+      </c>
+      <c r="O30" s="6">
+        <f t="shared" si="8"/>
+        <v>81.608089257532541</v>
+      </c>
+      <c r="P30" s="9">
+        <f t="shared" si="9"/>
+        <v>85.587489752049947</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="28" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C28" s="6">
-        <v>0.54063046130762304</v>
-      </c>
-    </row>
-    <row r="29" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C29" s="6">
-        <v>34.134141264910802</v>
-      </c>
-    </row>
-    <row r="30" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C30">
-        <f>(C28+C29)/2</f>
-        <v>17.337385863109212</v>
+      <c r="B31">
+        <v>47.943197763883099</v>
+      </c>
+      <c r="C31" s="6">
+        <v>11.4811841212213</v>
+      </c>
+      <c r="D31" s="6">
+        <v>10.6480205078108</v>
+      </c>
+      <c r="E31" s="6">
+        <v>10.915173121256901</v>
+      </c>
+      <c r="F31">
+        <v>11.0722959164007</v>
+      </c>
+      <c r="G31" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="H31">
+        <v>103.38036423672099</v>
+      </c>
+      <c r="I31">
+        <v>103.99572480142</v>
+      </c>
+      <c r="J31">
+        <v>99.234147304171998</v>
+      </c>
+      <c r="K31">
+        <v>94.367099788090897</v>
+      </c>
+      <c r="L31" s="6">
+        <f t="shared" si="5"/>
+        <v>88.459105610837383</v>
+      </c>
+      <c r="M31" s="6">
+        <f t="shared" si="6"/>
+        <v>89.907629788946892</v>
+      </c>
+      <c r="N31" s="6">
+        <f t="shared" si="7"/>
+        <v>84.878899678252793</v>
+      </c>
+      <c r="O31" s="6">
+        <f t="shared" si="8"/>
+        <v>79.854729367027886</v>
+      </c>
+      <c r="P31" s="9">
+        <f t="shared" si="9"/>
+        <v>85.775091111266221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32">
+        <v>54.362399237496497</v>
+      </c>
+      <c r="C32">
+        <v>12.9621852923768</v>
+      </c>
+      <c r="D32">
+        <v>15.323743060902</v>
+      </c>
+      <c r="E32">
+        <v>37.042560603958101</v>
+      </c>
+      <c r="F32">
+        <v>53.041429329361399</v>
+      </c>
+      <c r="G32" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="H32">
+        <v>101.70695238601699</v>
+      </c>
+      <c r="I32">
+        <v>110.026416640646</v>
+      </c>
+      <c r="J32">
+        <v>122.731095552444</v>
+      </c>
+      <c r="K32">
+        <v>138.09521327147601</v>
+      </c>
+      <c r="L32" s="6">
+        <f t="shared" si="5"/>
+        <v>85.304692588977886</v>
+      </c>
+      <c r="M32" s="6">
+        <f t="shared" si="6"/>
+        <v>91.262599075081695</v>
+      </c>
+      <c r="N32" s="6">
+        <f t="shared" si="7"/>
+        <v>82.248460443823603</v>
+      </c>
+      <c r="O32" s="6">
+        <f t="shared" si="8"/>
+        <v>81.613709437452314</v>
+      </c>
+      <c r="P32" s="9">
+        <f t="shared" si="9"/>
+        <v>85.107365386333882</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="O40" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41">
+        <v>3144.16048723623</v>
+      </c>
+      <c r="C41" s="6">
+        <v>16.172406414180401</v>
+      </c>
+      <c r="D41">
+        <v>16.584852244704901</v>
+      </c>
+      <c r="E41" s="6">
+        <v>15.076120185435499</v>
+      </c>
+      <c r="F41">
+        <v>15.3296778046866</v>
+      </c>
+      <c r="G41" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="H41">
+        <v>1266.3802028626401</v>
+      </c>
+      <c r="I41">
+        <v>1239.2457168881199</v>
+      </c>
+      <c r="J41">
+        <v>1312.1272076882999</v>
+      </c>
+      <c r="K41">
+        <v>1330.2754645709399</v>
+      </c>
+      <c r="L41" s="6">
+        <f>(H41-C41-G41)</f>
+        <v>1246.7834098510734</v>
+      </c>
+      <c r="M41" s="6">
+        <f>(I41-D41-G41)</f>
+        <v>1219.2364780460287</v>
+      </c>
+      <c r="N41" s="6">
+        <f>(J41-E41-G41)</f>
+        <v>1293.6267009054782</v>
+      </c>
+      <c r="O41" s="6">
+        <f>(K41-F41-G41)</f>
+        <v>1311.5214001688671</v>
+      </c>
+      <c r="P41" s="9">
+        <f>(L41+M41+N41+O41)/4</f>
+        <v>1267.791997242862</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>52</v>
+      </c>
+      <c r="B42">
+        <v>137100.715637207</v>
+      </c>
+      <c r="C42" s="6">
+        <v>152.29655436061199</v>
+      </c>
+      <c r="D42" s="6">
+        <v>144.29762564570601</v>
+      </c>
+      <c r="E42" s="6">
+        <v>160.05635477709001</v>
+      </c>
+      <c r="F42">
+        <v>173.15498055168001</v>
+      </c>
+      <c r="G42" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="H42">
+        <v>1398.5665355409801</v>
+      </c>
+      <c r="I42">
+        <v>1381.67841990958</v>
+      </c>
+      <c r="J42">
+        <v>1465.4698619411599</v>
+      </c>
+      <c r="K42">
+        <v>1479.3596455648601</v>
+      </c>
+      <c r="L42" s="6">
+        <f t="shared" ref="L42:L47" si="10">(H42-C42-G42)</f>
+        <v>1242.8455945829819</v>
+      </c>
+      <c r="M42" s="6">
+        <f t="shared" ref="M42:M47" si="11">(I42-D42-G42)</f>
+        <v>1233.9564076664878</v>
+      </c>
+      <c r="N42" s="6">
+        <f t="shared" ref="N42:N47" si="12">(J42-E42-G42)</f>
+        <v>1301.9891205666836</v>
+      </c>
+      <c r="O42" s="6">
+        <f t="shared" ref="O42:O47" si="13">(K42-F42-G42)</f>
+        <v>1302.7802784157939</v>
+      </c>
+      <c r="P42" s="9">
+        <f t="shared" ref="P42:P47" si="14">(L42+M42+N42+O42)/4</f>
+        <v>1270.3928503079869</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+      <c r="B43">
+        <v>3125.5087894675999</v>
+      </c>
+      <c r="C43" s="6">
+        <v>15.7964597682774</v>
+      </c>
+      <c r="D43" s="6">
+        <v>15.5367968936068</v>
+      </c>
+      <c r="E43" s="6">
+        <v>15.848920827399199</v>
+      </c>
+      <c r="F43">
+        <v>16.407635592953898</v>
+      </c>
+      <c r="G43" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H43">
+        <v>1270.54629717892</v>
+      </c>
+      <c r="I43">
+        <v>1241.23775242325</v>
+      </c>
+      <c r="J43">
+        <v>1301.87346783812</v>
+      </c>
+      <c r="K43">
+        <v>1312.7505429759001</v>
+      </c>
+      <c r="L43" s="6">
+        <f t="shared" si="10"/>
+        <v>1251.3176144677743</v>
+      </c>
+      <c r="M43" s="6">
+        <f t="shared" si="11"/>
+        <v>1222.2687325867748</v>
+      </c>
+      <c r="N43" s="6">
+        <f t="shared" si="12"/>
+        <v>1282.5923240678524</v>
+      </c>
+      <c r="O43" s="6">
+        <f t="shared" si="13"/>
+        <v>1292.9106844400778</v>
+      </c>
+      <c r="P43" s="9">
+        <f t="shared" si="14"/>
+        <v>1262.2723388906197</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44">
+        <v>3642.0171727304801</v>
+      </c>
+      <c r="C44" s="6">
+        <v>91.448995502374501</v>
+      </c>
+      <c r="D44" s="6">
+        <v>99.246079891339605</v>
+      </c>
+      <c r="E44" s="6">
+        <v>119.293467306038</v>
+      </c>
+      <c r="F44">
+        <v>117.303567854397</v>
+      </c>
+      <c r="G44" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="H44">
+        <v>1353.1058268342799</v>
+      </c>
+      <c r="I44">
+        <v>1340.8253010552301</v>
+      </c>
+      <c r="J44">
+        <v>1432.73518285777</v>
+      </c>
+      <c r="K44">
+        <v>1428.9955440608901</v>
+      </c>
+      <c r="L44" s="6">
+        <f t="shared" si="10"/>
+        <v>1258.224608389037</v>
+      </c>
+      <c r="M44" s="6">
+        <f t="shared" si="11"/>
+        <v>1238.1469982210222</v>
+      </c>
+      <c r="N44" s="6">
+        <f t="shared" si="12"/>
+        <v>1310.0094926088639</v>
+      </c>
+      <c r="O44" s="6">
+        <f t="shared" si="13"/>
+        <v>1308.2597532636248</v>
+      </c>
+      <c r="P44" s="9">
+        <f t="shared" si="14"/>
+        <v>1278.6602131206369</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45">
+        <v>3232.9062776467199</v>
+      </c>
+      <c r="C45" s="6">
+        <v>17.691985893020401</v>
+      </c>
+      <c r="D45" s="6">
+        <v>30.922681124659299</v>
+      </c>
+      <c r="E45" s="6">
+        <v>53.687758967397997</v>
+      </c>
+      <c r="F45">
+        <v>76.816073135976595</v>
+      </c>
+      <c r="G45" s="8">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="H45">
+        <v>1258.5168948821799</v>
+      </c>
+      <c r="I45">
+        <v>1262.7569204172701</v>
+      </c>
+      <c r="J45">
+        <v>1337.6830662981699</v>
+      </c>
+      <c r="K45">
+        <v>1377.28891171451</v>
+      </c>
+      <c r="L45" s="6">
+        <f t="shared" si="10"/>
+        <v>1237.4217431346658</v>
+      </c>
+      <c r="M45" s="6">
+        <f t="shared" si="11"/>
+        <v>1228.4310734381172</v>
+      </c>
+      <c r="N45" s="6">
+        <f t="shared" si="12"/>
+        <v>1280.5921414762784</v>
+      </c>
+      <c r="O45" s="6">
+        <f t="shared" si="13"/>
+        <v>1297.0696727240397</v>
+      </c>
+      <c r="P45" s="9">
+        <f t="shared" si="14"/>
+        <v>1260.8786576932753</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B46">
+        <v>2798.6146199334498</v>
+      </c>
+      <c r="C46" s="6">
+        <v>15.552245469805801</v>
+      </c>
+      <c r="D46" s="6">
+        <v>15.6987551942034</v>
+      </c>
+      <c r="E46" s="6">
+        <v>15.9379273775171</v>
+      </c>
+      <c r="F46">
+        <v>14.6978477089423</v>
+      </c>
+      <c r="G46" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="H46">
+        <v>1262.12741147269</v>
+      </c>
+      <c r="I46">
+        <v>1247.39613110657</v>
+      </c>
+      <c r="J46">
+        <v>1312.9196750561</v>
+      </c>
+      <c r="K46">
+        <v>1309.10656011622</v>
+      </c>
+      <c r="L46" s="6">
+        <f t="shared" si="10"/>
+        <v>1243.135091498222</v>
+      </c>
+      <c r="M46" s="6">
+        <f t="shared" si="11"/>
+        <v>1228.2573014077043</v>
+      </c>
+      <c r="N46" s="6">
+        <f t="shared" si="12"/>
+        <v>1293.5416731739206</v>
+      </c>
+      <c r="O46" s="6">
+        <f t="shared" si="13"/>
+        <v>1290.9686379026152</v>
+      </c>
+      <c r="P46" s="9">
+        <f t="shared" si="14"/>
+        <v>1263.9756759956156</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>55</v>
+      </c>
+      <c r="B47">
+        <v>3012.9789593293399</v>
+      </c>
+      <c r="C47" s="6">
+        <v>15.354518245541801</v>
+      </c>
+      <c r="D47">
+        <v>26.029806109409702</v>
+      </c>
+      <c r="E47">
+        <v>52.645299658298597</v>
+      </c>
+      <c r="F47">
+        <v>73.765081063023601</v>
+      </c>
+      <c r="G47" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="H47">
+        <v>1269.7002746903299</v>
+      </c>
+      <c r="I47">
+        <v>1271.2879097467801</v>
+      </c>
+      <c r="J47">
+        <v>1357.9602965453701</v>
+      </c>
+      <c r="K47">
+        <v>1372.6979691172101</v>
+      </c>
+      <c r="L47" s="6">
+        <f t="shared" si="10"/>
+        <v>1250.9056819401258</v>
+      </c>
+      <c r="M47" s="6">
+        <f t="shared" si="11"/>
+        <v>1241.818029132708</v>
+      </c>
+      <c r="N47" s="6">
+        <f t="shared" si="12"/>
+        <v>1301.8749223824091</v>
+      </c>
+      <c r="O47" s="6">
+        <f t="shared" si="13"/>
+        <v>1295.492813549524</v>
+      </c>
+      <c r="P47" s="9">
+        <f t="shared" si="14"/>
+        <v>1272.5228617511916</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="J53" t="s">
+        <v>94</v>
+      </c>
+      <c r="K53" t="s">
+        <v>89</v>
+      </c>
+      <c r="L53" t="s">
+        <v>90</v>
+      </c>
+      <c r="M53" t="s">
+        <v>95</v>
+      </c>
+      <c r="N53" t="s">
+        <v>93</v>
+      </c>
+      <c r="O53" t="s">
+        <v>92</v>
+      </c>
+      <c r="P53" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>85</v>
+      </c>
+      <c r="D54" t="s">
+        <v>86</v>
+      </c>
+      <c r="F54" t="s">
+        <v>87</v>
+      </c>
+      <c r="G54" t="s">
+        <v>88</v>
+      </c>
+      <c r="J54" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="K54" s="10">
+        <v>5.5212200000823898E-5</v>
+      </c>
+      <c r="L54">
+        <v>0.53922044867672203</v>
+      </c>
+      <c r="M54">
+        <v>4.3880832130522629E-2</v>
+      </c>
+      <c r="N54" s="6">
+        <f>M54-K54</f>
+        <v>4.3825619930521802E-2</v>
+      </c>
+      <c r="O54" s="10">
+        <f>J54+K54+N54+L54</f>
+        <v>4.0074878781935244</v>
+      </c>
+      <c r="P54">
+        <v>4.0050931003851096</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>51</v>
+      </c>
+      <c r="D55" s="10">
+        <f>0.0000552122000008239*1000</f>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F55" s="10">
+        <f>D55*10</f>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G55" s="10">
+        <f>D55*100</f>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J55" s="8">
+        <v>3.4243865973862802</v>
+      </c>
+      <c r="K55" s="10">
+        <v>5.9445500002766401E-5</v>
+      </c>
+      <c r="L55">
+        <v>45.082622893090097</v>
+      </c>
+      <c r="M55">
+        <v>5.2427444664404215</v>
+      </c>
+      <c r="N55" s="6">
+        <f t="shared" ref="N55:N60" si="15">M55-K55</f>
+        <v>5.242685020940419</v>
+      </c>
+      <c r="O55" s="10">
+        <f t="shared" ref="O55:O60" si="16">J55+K55+N55+L55</f>
+        <v>53.749753956916798</v>
+      </c>
+      <c r="P55">
+        <v>54.5115243820917</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>52</v>
+      </c>
+      <c r="B56" s="10">
+        <v>1.2000018614344299E-7</v>
+      </c>
+      <c r="D56" s="10">
+        <f t="shared" ref="D56:D61" si="17">0.0000552122000008239*1000</f>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F56" s="10">
+        <f t="shared" ref="F56:F61" si="18">D56*10</f>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G56" s="10">
+        <f t="shared" ref="G56:G61" si="19">D56*100</f>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J56" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="K56" s="10">
+        <v>5.4939699999522401E-5</v>
+      </c>
+      <c r="L56">
+        <v>0.54917054483667005</v>
+      </c>
+      <c r="M56">
+        <v>0.17087024937428297</v>
+      </c>
+      <c r="N56" s="6">
+        <f t="shared" si="15"/>
+        <v>0.17081530967428343</v>
+      </c>
+      <c r="O56" s="10">
+        <f t="shared" si="16"/>
+        <v>4.1522637370793225</v>
+      </c>
+      <c r="P56">
+        <v>4.0775397573838204</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>53</v>
+      </c>
+      <c r="D57" s="10">
+        <f t="shared" si="17"/>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F57" s="10">
+        <f t="shared" si="18"/>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G57" s="10">
+        <f t="shared" si="19"/>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J57" s="8">
+        <v>3.4322229428683699</v>
+      </c>
+      <c r="K57" s="10">
+        <v>5.8752400000230403E-5</v>
+      </c>
+      <c r="L57">
+        <v>34.394685960258002</v>
+      </c>
+      <c r="M57">
+        <v>9.6000442380037558</v>
+      </c>
+      <c r="N57" s="6">
+        <f t="shared" si="15"/>
+        <v>9.5999854856037548</v>
+      </c>
+      <c r="O57" s="10">
+        <f t="shared" si="16"/>
+        <v>47.426953141130127</v>
+      </c>
+      <c r="P57">
+        <v>47.1892843685389</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>54</v>
+      </c>
+      <c r="D58" s="10">
+        <f t="shared" si="17"/>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F58" s="10">
+        <f t="shared" si="18"/>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G58" s="10">
+        <f t="shared" si="19"/>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J58" s="8">
+        <v>3.4031658544935599</v>
+      </c>
+      <c r="K58" s="10">
+        <v>5.9051499999535699E-5</v>
+      </c>
+      <c r="L58">
+        <v>6.2376752522495398</v>
+      </c>
+      <c r="M58">
+        <v>1.2156685698951224</v>
+      </c>
+      <c r="N58" s="6">
+        <f t="shared" si="15"/>
+        <v>1.2156095183951228</v>
+      </c>
+      <c r="O58" s="10">
+        <f t="shared" si="16"/>
+        <v>10.856509676638222</v>
+      </c>
+      <c r="P58">
+        <v>11.208388920637001</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>41</v>
+      </c>
+      <c r="D59" s="10">
+        <f t="shared" si="17"/>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F59" s="10">
+        <f t="shared" si="18"/>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G59" s="10">
+        <f t="shared" si="19"/>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J59" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="K59" s="10">
+        <v>5.64270999966538E-5</v>
+      </c>
+      <c r="L59">
+        <v>0.54279469219126897</v>
+      </c>
+      <c r="M59">
+        <v>0.14936036961757015</v>
+      </c>
+      <c r="N59" s="6">
+        <f t="shared" si="15"/>
+        <v>0.14930394251757351</v>
+      </c>
+      <c r="O59" s="10">
+        <f t="shared" si="16"/>
+        <v>4.1322295664711488</v>
+      </c>
+      <c r="P59">
+        <v>4.1074357013928502</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>42</v>
+      </c>
+      <c r="D60" s="10">
+        <f t="shared" si="17"/>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F60" s="10">
+        <f t="shared" si="18"/>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G60" s="10">
+        <f t="shared" si="19"/>
+        <v>5.5212200000823897</v>
+      </c>
+      <c r="J60" s="8">
+        <v>3.4400745046623098</v>
+      </c>
+      <c r="K60" s="10">
+        <v>5.7626800002472003E-5</v>
+      </c>
+      <c r="L60">
+        <v>5.9257052455949104</v>
+      </c>
+      <c r="M60">
+        <v>0.41487396002467236</v>
+      </c>
+      <c r="N60" s="6">
+        <f t="shared" si="15"/>
+        <v>0.41481633322466988</v>
+      </c>
+      <c r="O60" s="10">
+        <f t="shared" si="16"/>
+        <v>9.7806537102818929</v>
+      </c>
+      <c r="P60">
+        <v>9.8390835440481492</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61" s="10">
+        <f t="shared" si="17"/>
+        <v>5.5212200000823899E-2</v>
+      </c>
+      <c r="F61" s="10">
+        <f t="shared" si="18"/>
+        <v>0.55212200000823897</v>
+      </c>
+      <c r="G61" s="10">
+        <f t="shared" si="19"/>
+        <v>5.5212200000823897</v>
+      </c>
+    </row>
+    <row r="67" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O67" s="10">
+        <v>4.0074878781935244</v>
+      </c>
+    </row>
+    <row r="68" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O68" s="10">
+        <v>53.749753956916798</v>
+      </c>
+    </row>
+    <row r="69" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O69" s="10">
+        <v>4.1522637370793225</v>
+      </c>
+    </row>
+    <row r="70" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O70" s="10">
+        <v>47.426953141130127</v>
+      </c>
+    </row>
+    <row r="71" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O71" s="10">
+        <v>10.856509676638222</v>
+      </c>
+    </row>
+    <row r="72" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O72" s="10">
+        <v>4.1322295664711488</v>
+      </c>
+    </row>
+    <row r="73" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O73" s="10">
+        <v>9.7806537102818929</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add sharding execution time
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2A78FD-96CE-4E66-B1A4-6DA98FB2A389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF25CA8-89C0-4C94-83FA-5008D62007C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="102">
   <si>
     <t>Functions</t>
   </si>
@@ -330,13 +330,19 @@
     <t>Internal Processing Time</t>
   </si>
   <si>
-    <t>Total Internal Response Time</t>
-  </si>
-  <si>
     <t>Internal Waiting Time</t>
   </si>
   <si>
     <t>Internal Round Trip Latency</t>
+  </si>
+  <si>
+    <t>M6: Total Internal Response Time</t>
+  </si>
+  <si>
+    <t>M6: Internal Round-trip Latency</t>
+  </si>
+  <si>
+    <t>C1-M6:</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
-  <dimension ref="A1:P76"/>
+  <dimension ref="A1:P89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
@@ -2948,16 +2954,16 @@
         <v>66</v>
       </c>
       <c r="I69" t="s">
+        <v>98</v>
+      </c>
+      <c r="J69" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="J69" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="K69" t="s">
         <v>96</v>
       </c>
       <c r="L69" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P69" s="10"/>
     </row>
@@ -3230,6 +3236,115 @@
       <c r="L76">
         <f t="shared" si="19"/>
         <v>3.1220483790606308</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" t="s">
+        <v>101</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>51</v>
+      </c>
+      <c r="B83">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="C83">
+        <v>0.55838740154120903</v>
+      </c>
+      <c r="F83" s="2">
+        <v>1.80840492248535</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>52</v>
+      </c>
+      <c r="B84">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="C84">
+        <v>44.2128236796663</v>
+      </c>
+      <c r="F84" s="2">
+        <v>25.537014007568299</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>53</v>
+      </c>
+      <c r="B85">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="C85">
+        <v>0.55610468315723705</v>
+      </c>
+      <c r="F85" s="2">
+        <v>0.39505958557128901</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>54</v>
+      </c>
+      <c r="B86">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="C86">
+        <v>33.915199203098602</v>
+      </c>
+      <c r="F86" s="2">
+        <v>15.4211521148681</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>41</v>
+      </c>
+      <c r="B87">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="C87">
+        <v>6.26711183921228</v>
+      </c>
+      <c r="F87" s="2">
+        <v>3.9656162261962802</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>42</v>
+      </c>
+      <c r="B88">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="C88">
+        <v>0.53144267035855097</v>
+      </c>
+      <c r="F88" s="2">
+        <v>0.38695335388183499</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>55</v>
+      </c>
+      <c r="B89">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="C89">
+        <v>5.8418899377243996</v>
+      </c>
+      <c r="F89" s="2">
+        <v>3.5953521728515598</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add sharding execution time all
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF25CA8-89C0-4C94-83FA-5008D62007C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D71B3D2-8077-4D4D-8D76-D1DDB1387FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="103">
   <si>
     <t>Functions</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>C1-M6:</t>
+  </si>
+  <si>
+    <t>S</t>
   </si>
 </sst>
 </file>
@@ -3238,7 +3241,7 @@
         <v>3.1220483790606308</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>0</v>
       </c>
@@ -3248,8 +3251,11 @@
       <c r="F82" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H82" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>51</v>
       </c>
@@ -3263,7 +3269,7 @@
         <v>1.80840492248535</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>52</v>
       </c>
@@ -3277,7 +3283,7 @@
         <v>25.537014007568299</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>53</v>
       </c>
@@ -3291,7 +3297,7 @@
         <v>0.39505958557128901</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>54</v>
       </c>
@@ -3305,7 +3311,7 @@
         <v>15.4211521148681</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>41</v>
       </c>
@@ -3319,7 +3325,7 @@
         <v>3.9656162261962802</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>42</v>
       </c>
@@ -3333,7 +3339,7 @@
         <v>0.38695335388183499</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Logging for redis functions
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D71B3D2-8077-4D4D-8D76-D1DDB1387FAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904C84A0-69F6-4FEE-985A-ECE37AE8F277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="104">
   <si>
     <t>Functions</t>
   </si>
@@ -342,10 +342,13 @@
     <t>M6: Internal Round-trip Latency</t>
   </si>
   <si>
-    <t>C1-M6:</t>
-  </si>
-  <si>
-    <t>S</t>
+    <t>Sharding_Execution_Time</t>
+  </si>
+  <si>
+    <t>Number of Key-Value Pair</t>
+  </si>
+  <si>
+    <t>C1-M6: Total Response Time</t>
   </si>
 </sst>
 </file>
@@ -3246,13 +3249,16 @@
         <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>101</v>
+        <v>103</v>
+      </c>
+      <c r="E82" t="s">
+        <v>102</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H82" t="s">
-        <v>102</v>
+      <c r="G82" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -3265,8 +3271,18 @@
       <c r="C83">
         <v>0.55838740154120903</v>
       </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
       <c r="F83" s="2">
         <v>1.80840492248535</v>
+      </c>
+      <c r="G83">
+        <v>4.5504420995712202E-3</v>
+      </c>
+      <c r="H83">
+        <f>F83-G83</f>
+        <v>1.8038544803857788</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -3279,8 +3295,18 @@
       <c r="C84">
         <v>44.2128236796663</v>
       </c>
+      <c r="E84">
+        <v>1000</v>
+      </c>
       <c r="F84" s="2">
         <v>25.537014007568299</v>
+      </c>
+      <c r="G84">
+        <v>1.76797062158584</v>
+      </c>
+      <c r="H84">
+        <f t="shared" ref="H84:H89" si="20">F84-G84</f>
+        <v>23.76904338598246</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -3293,8 +3319,18 @@
       <c r="C85">
         <v>0.55610468315723705</v>
       </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
       <c r="F85" s="2">
         <v>0.39505958557128901</v>
+      </c>
+      <c r="G85">
+        <v>4.5504420995712202E-3</v>
+      </c>
+      <c r="H85">
+        <f t="shared" si="20"/>
+        <v>0.39050914347171778</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -3307,8 +3343,18 @@
       <c r="C86">
         <v>33.915199203098602</v>
       </c>
+      <c r="E86">
+        <v>1000</v>
+      </c>
       <c r="F86" s="2">
         <v>15.4211521148681</v>
+      </c>
+      <c r="G86">
+        <v>1.76797062158584</v>
+      </c>
+      <c r="H86">
+        <f t="shared" si="20"/>
+        <v>13.653181493282259</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -3321,8 +3367,18 @@
       <c r="C87">
         <v>6.26711183921228</v>
       </c>
+      <c r="E87">
+        <v>100</v>
+      </c>
       <c r="F87" s="2">
         <v>3.9656162261962802</v>
+      </c>
+      <c r="G87">
+        <v>0.18550083041191101</v>
+      </c>
+      <c r="H87">
+        <f t="shared" si="20"/>
+        <v>3.7801153957843692</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
@@ -3335,8 +3391,18 @@
       <c r="C88">
         <v>0.53144267035855097</v>
       </c>
+      <c r="E88">
+        <v>1</v>
+      </c>
       <c r="F88" s="2">
         <v>0.38695335388183499</v>
+      </c>
+      <c r="G88">
+        <v>4.5504420995712202E-3</v>
+      </c>
+      <c r="H88">
+        <f t="shared" si="20"/>
+        <v>0.38240291178226377</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -3349,8 +3415,18 @@
       <c r="C89">
         <v>5.8418899377243996</v>
       </c>
+      <c r="E89">
+        <v>100</v>
+      </c>
       <c r="F89" s="2">
         <v>3.5953521728515598</v>
+      </c>
+      <c r="G89">
+        <v>0.18550083041191101</v>
+      </c>
+      <c r="H89">
+        <f t="shared" si="20"/>
+        <v>3.4098513424396488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add reports fine tune
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1466689-ACC4-4D10-9107-34DE0FECB5B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434DB9E3-D3E6-4BCC-89E2-47EB3AD1752B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="72">
   <si>
     <t>Functions</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t>Difference: C10-C1 (M:6)</t>
+  </si>
+  <si>
+    <t>baseline :C1</t>
   </si>
 </sst>
 </file>
@@ -396,7 +399,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -508,6 +511,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -518,7 +532,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
@@ -539,6 +553,9 @@
     <xf numFmtId="164" fontId="7" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="6" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -572,9 +589,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="20% - Accent5" xfId="5" builtinId="46"/>
@@ -878,83 +893,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="24"/>
-      <c r="F1" s="22" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="25"/>
+      <c r="F1" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="24"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="26"/>
-      <c r="F2" s="25" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="27"/>
+      <c r="F2" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="26"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="26"/>
-      <c r="F3" s="25" t="s">
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="27"/>
+      <c r="F3" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="26"/>
+      <c r="G3" s="27"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="26"/>
-      <c r="F4" s="25" t="s">
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="27"/>
+      <c r="F4" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="26"/>
+      <c r="G4" s="27"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="26"/>
-      <c r="F5" s="25" t="s">
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="27"/>
+      <c r="F5" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="26"/>
+      <c r="G5" s="27"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="28"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="28"/>
+      <c r="B6" s="31"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="29"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="29"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="31" t="s">
+      <c r="A11" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="31"/>
+      <c r="B11" s="20"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -1422,10 +1437,10 @@
       <c r="P20" s="18"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="31" t="s">
+      <c r="A25" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="31"/>
+      <c r="B25" s="20"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -1893,10 +1908,10 @@
       <c r="P34" s="18"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
+      <c r="A40" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="31"/>
+      <c r="B40" s="20"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -2364,10 +2379,10 @@
       <c r="P49" s="18"/>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="20" t="s">
+      <c r="A51" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="B51" s="20"/>
+      <c r="B51" s="21"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D56" s="5"/>
@@ -2381,20 +2396,30 @@
       <c r="G57" s="5"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="21" t="s">
+      <c r="A58" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B58" s="21"/>
-      <c r="C58" s="21"/>
-      <c r="D58" s="21"/>
-      <c r="E58" s="21"/>
-      <c r="F58" s="21"/>
+      <c r="B58" s="22"/>
+      <c r="C58" s="22"/>
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
       <c r="G58" s="5"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D59" s="5"/>
       <c r="F59" s="5"/>
       <c r="G59" s="5"/>
+      <c r="K59" t="s">
+        <v>9</v>
+      </c>
+      <c r="N59" s="3">
+        <v>0.52516379831418403</v>
+      </c>
+      <c r="O59" s="3">
+        <f>N59-G91</f>
+        <v>0.19962707040891103</v>
+      </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
@@ -2415,6 +2440,16 @@
       <c r="F60" s="6" t="s">
         <v>37</v>
       </c>
+      <c r="K60" t="s">
+        <v>10</v>
+      </c>
+      <c r="N60">
+        <v>32.977948012191398</v>
+      </c>
+      <c r="O60" s="3">
+        <f>N60-G92</f>
+        <v>19.1043947361294</v>
+      </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
@@ -2435,6 +2470,16 @@
       <c r="F61" s="7">
         <v>1.68681144714355</v>
       </c>
+      <c r="K61" t="s">
+        <v>11</v>
+      </c>
+      <c r="N61">
+        <v>0.49840760395546102</v>
+      </c>
+      <c r="O61" s="3">
+        <f>N61-G93</f>
+        <v>0.33232522175331303</v>
+      </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -2455,6 +2500,16 @@
       <c r="F62" s="7">
         <v>18.5704231262207</v>
       </c>
+      <c r="K62" t="s">
+        <v>12</v>
+      </c>
+      <c r="N62">
+        <v>25.759887776849901</v>
+      </c>
+      <c r="O62" s="3">
+        <f>N62-G94</f>
+        <v>16.615271649835741</v>
+      </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
@@ -2475,6 +2530,16 @@
       <c r="F63" s="7">
         <v>0.40674209594726501</v>
       </c>
+      <c r="K63" t="s">
+        <v>1</v>
+      </c>
+      <c r="N63">
+        <v>3.52255095970304</v>
+      </c>
+      <c r="O63" s="3">
+        <f>N63-G95</f>
+        <v>2.1187900496688701</v>
+      </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -2495,8 +2560,18 @@
       <c r="F64" s="7">
         <v>12.6996040344238</v>
       </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K64" t="s">
+        <v>2</v>
+      </c>
+      <c r="N64" s="3">
+        <v>0.49062787411620901</v>
+      </c>
+      <c r="O64" s="3">
+        <f>N64-G96</f>
+        <v>0.36078511593749901</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>1</v>
       </c>
@@ -2515,8 +2590,18 @@
       <c r="F65" s="7">
         <v>3.41200828552246</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K65" t="s">
+        <v>13</v>
+      </c>
+      <c r="N65">
+        <v>3.1790446098824598</v>
+      </c>
+      <c r="O65" s="3">
+        <f>N65-G97</f>
+        <v>1.89718711934291</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2536,7 +2621,7 @@
         <v>0.13566017150878901</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>13</v>
       </c>
@@ -2556,13 +2641,13 @@
         <v>3.5090446472167902</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="I68" s="5"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="I69" s="5"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>0</v>
       </c>
@@ -2582,7 +2667,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -2602,7 +2687,7 @@
         <v>1.6944408416748</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>10</v>
       </c>
@@ -2622,7 +2707,7 @@
         <v>16.4527893066406</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>11</v>
       </c>
@@ -2642,7 +2727,7 @@
         <v>0.37431716918945301</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>12</v>
       </c>
@@ -2662,7 +2747,7 @@
         <v>11.4581584930419</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>1</v>
       </c>
@@ -2682,7 +2767,7 @@
         <v>3.2749176025390598</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>2</v>
       </c>
@@ -2702,7 +2787,7 @@
         <v>0.24819374084472601</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>13</v>
       </c>
@@ -2722,7 +2807,7 @@
         <v>2.8343200683593701</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>0</v>
       </c>
@@ -2742,7 +2827,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>9</v>
       </c>
@@ -2762,7 +2847,7 @@
         <v>1.66249275207519</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>10</v>
       </c>
@@ -2782,7 +2867,7 @@
         <v>14.9691104888916</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>11</v>
       </c>
@@ -2802,7 +2887,7 @@
         <v>0.39219856262206998</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>12</v>
       </c>
@@ -2822,7 +2907,7 @@
         <v>9.6678733825683594</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>1</v>
       </c>
@@ -2842,7 +2927,7 @@
         <v>2.42781639099121</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>2</v>
       </c>
@@ -2862,7 +2947,7 @@
         <v>0.32162666320800698</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>13</v>
       </c>
@@ -2882,7 +2967,7 @@
         <v>1.79862976074218</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>0</v>
       </c>
@@ -2901,8 +2986,11 @@
       <c r="F90" s="6" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G90" s="32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>9</v>
       </c>
@@ -2921,8 +3009,11 @@
       <c r="F91" s="7">
         <v>1.6837120056152299</v>
       </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G91">
+        <v>0.32553672790527299</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>10</v>
       </c>
@@ -2941,8 +3032,11 @@
       <c r="F92" s="7">
         <v>12.8097534179687</v>
       </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G92">
+        <v>13.873553276061999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>11</v>
       </c>
@@ -2961,8 +3055,11 @@
       <c r="F93" s="7">
         <v>0.47087669372558499</v>
       </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G93">
+        <v>0.16608238220214799</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>12</v>
       </c>
@@ -2981,8 +3078,11 @@
       <c r="F94" s="7">
         <v>8.54420661926269</v>
       </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G94">
+        <v>9.1446161270141602</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>1</v>
       </c>
@@ -3001,8 +3101,11 @@
       <c r="F95" s="7">
         <v>1.3589859008789</v>
       </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G95">
+        <v>1.4037609100341699</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>2</v>
       </c>
@@ -3020,6 +3123,9 @@
       </c>
       <c r="F96" s="7">
         <v>0.25033950805664001</v>
+      </c>
+      <c r="G96">
+        <v>0.12984275817870999</v>
       </c>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.25">
@@ -3041,6 +3147,9 @@
       <c r="F97" s="7">
         <v>1.34897232055664</v>
       </c>
+      <c r="G97">
+        <v>1.2818574905395499</v>
+      </c>
     </row>
     <row r="110" spans="1:19" x14ac:dyDescent="0.25">
       <c r="G110" s="2" t="s">
@@ -3400,6 +3509,7 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="A58:F58"/>
@@ -3416,7 +3526,6 @@
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A25:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add data distributions analysis
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434DB9E3-D3E6-4BCC-89E2-47EB3AD1752B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4C3AB1-3950-41EB-8B79-F89D670EBEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="73">
   <si>
     <t>Functions</t>
   </si>
@@ -194,9 +194,6 @@
     <t>Middleware Configurations:</t>
   </si>
   <si>
-    <t>Baseline_Failed_Execution: set_multiple</t>
-  </si>
-  <si>
     <t>Average</t>
   </si>
   <si>
@@ -252,6 +249,12 @@
   </si>
   <si>
     <t>baseline :C1</t>
+  </si>
+  <si>
+    <t>Response Time direct</t>
+  </si>
+  <si>
+    <t>Baseline: 1</t>
   </si>
 </sst>
 </file>
@@ -261,7 +264,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -302,14 +305,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -532,7 +527,7 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
@@ -542,21 +537,16 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="4" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="5" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="5"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="7" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="12" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="6" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
@@ -589,7 +579,6 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="20% - Accent5" xfId="5" builtinId="46"/>
@@ -876,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
-  <dimension ref="A1:S117"/>
+  <dimension ref="A1:S116"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -893,83 +882,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
-      <c r="F1" s="23" t="s">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="22"/>
+      <c r="F1" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="25"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="27"/>
-      <c r="F2" s="26" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="24"/>
+      <c r="F2" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" s="24"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="24"/>
+      <c r="F3" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="27"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="27"/>
-      <c r="F3" s="26" t="s">
+      <c r="G3" s="24"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="24"/>
+      <c r="F4" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="G3" s="27"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="27"/>
-      <c r="F4" s="26" t="s">
+      <c r="G4" s="24"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="24"/>
+      <c r="F5" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="27"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="27"/>
-      <c r="F5" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="27"/>
+      <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="31"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="29"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="29"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="26"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="26"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="20"/>
+      <c r="B11" s="18"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -993,16 +982,16 @@
       <c r="G12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J12" s="10" t="s">
+      <c r="J12" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="K12" s="10" t="s">
+      <c r="K12" s="9" t="s">
         <v>24</v>
       </c>
       <c r="L12" s="2" t="s">
@@ -1025,8 +1014,8 @@
       <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="9">
-        <v>1.7484884995680501</v>
+      <c r="B13">
+        <v>0.32553672790527299</v>
       </c>
       <c r="C13" s="3">
         <v>0.52516379831418403</v>
@@ -1043,16 +1032,16 @@
       <c r="G13" s="3">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="10">
         <v>3.9895902707595199</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <v>4.02605646143118</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="10">
         <v>4.0353076186722596</v>
       </c>
-      <c r="K13" s="11">
+      <c r="K13" s="10">
         <v>4.0050931003851096</v>
       </c>
       <c r="L13" s="3">
@@ -1071,7 +1060,7 @@
         <f>(K13-F13-G13)</f>
         <v>4.1486054322107613E-2</v>
       </c>
-      <c r="P13" s="19">
+      <c r="P13" s="16">
         <f>(L13+M13+N13+O13)/4</f>
         <v>4.3880832130522629E-2</v>
       </c>
@@ -1080,8 +1069,8 @@
       <c r="A14" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="9">
-        <v>6683.5777209355201</v>
+      <c r="B14">
+        <v>13.873553276061999</v>
       </c>
       <c r="C14">
         <v>32.977948012191398</v>
@@ -1098,16 +1087,16 @@
       <c r="G14" s="3">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <v>41.8466371823881</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="10">
         <v>45.799138335569502</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="10">
         <v>48.675797406364801</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="10">
         <v>54.5115243820917</v>
       </c>
       <c r="L14" s="3">
@@ -1126,7 +1115,7 @@
         <f t="shared" ref="O14:O19" si="3">(K14-F14-G14)</f>
         <v>6.0045148916153233</v>
       </c>
-      <c r="P14" s="19">
+      <c r="P14" s="16">
         <f t="shared" ref="P14:P19" si="4">(L14+M14+N14+O14)/4</f>
         <v>5.2427444664404215</v>
       </c>
@@ -1135,8 +1124,8 @@
       <c r="A15" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="9">
-        <v>7.7534715334574296</v>
+      <c r="B15">
+        <v>0.16608238220214799</v>
       </c>
       <c r="C15">
         <v>0.49840760395546102</v>
@@ -1153,16 +1142,16 @@
       <c r="G15" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="10">
         <v>4.0147860416504804</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="10">
         <v>4.1628384834501704</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="10">
         <v>4.1707241313894299</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K15" s="10">
         <v>4.0775397573838204</v>
       </c>
       <c r="L15" s="3">
@@ -1181,7 +1170,7 @@
         <f t="shared" si="3"/>
         <v>9.6146269678780261E-2</v>
       </c>
-      <c r="P15" s="19">
+      <c r="P15" s="16">
         <f t="shared" si="4"/>
         <v>0.17087024937428297</v>
       </c>
@@ -1190,8 +1179,8 @@
       <c r="A16" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="9">
-        <v>5248.1240630149796</v>
+      <c r="B16">
+        <v>9.1446161270141602</v>
       </c>
       <c r="C16">
         <v>25.759887776849901</v>
@@ -1208,16 +1197,16 @@
       <c r="G16" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H16" s="11">
+      <c r="H16" s="10">
         <v>38.3633321341607</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="10">
         <v>42.259016332980003</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="10">
         <v>44.808815805147901</v>
       </c>
-      <c r="K16" s="11">
+      <c r="K16" s="10">
         <v>47.1892843685389</v>
       </c>
       <c r="L16" s="3">
@@ -1236,7 +1225,7 @@
         <f t="shared" si="3"/>
         <v>9.3623754654125282</v>
       </c>
-      <c r="P16" s="19">
+      <c r="P16" s="16">
         <f t="shared" si="4"/>
         <v>9.6000442380037558</v>
       </c>
@@ -1245,8 +1234,8 @@
       <c r="A17" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="9">
-        <v>526.84138371394204</v>
+      <c r="B17">
+        <v>1.4037609100341699</v>
       </c>
       <c r="C17">
         <v>3.52255095970304</v>
@@ -1263,16 +1252,16 @@
       <c r="G17" s="3">
         <v>3.4031658544935599</v>
       </c>
-      <c r="H17" s="11">
+      <c r="H17" s="10">
         <v>7.9163517599320397</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="10">
         <v>8.8410975673074592</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="10">
         <v>9.8086684739508598</v>
       </c>
-      <c r="K17" s="11">
+      <c r="K17" s="10">
         <v>11.208388920637001</v>
       </c>
       <c r="L17" s="3">
@@ -1291,7 +1280,7 @@
         <f t="shared" si="3"/>
         <v>1.567547813893901</v>
       </c>
-      <c r="P17" s="19">
+      <c r="P17" s="16">
         <f t="shared" si="4"/>
         <v>1.2156685698951224</v>
       </c>
@@ -1300,8 +1289,8 @@
       <c r="A18" t="s">
         <v>2</v>
       </c>
-      <c r="B18" s="9">
-        <v>1.6942660013834601</v>
+      <c r="B18">
+        <v>0.12984275817870999</v>
       </c>
       <c r="C18" s="3">
         <v>0.49062787411620901</v>
@@ -1318,16 +1307,16 @@
       <c r="G18" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H18" s="11">
+      <c r="H18" s="10">
         <v>4.0209035037549397</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="10">
         <v>4.1352269590162702</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="10">
         <v>4.0890994634011797</v>
       </c>
-      <c r="K18" s="11">
+      <c r="K18" s="10">
         <v>4.1074357013928502</v>
       </c>
       <c r="L18" s="3">
@@ -1346,7 +1335,7 @@
         <f t="shared" si="3"/>
         <v>0.12456650453927143</v>
       </c>
-      <c r="P18" s="19">
+      <c r="P18" s="16">
         <f t="shared" si="4"/>
         <v>0.14936036961757015</v>
       </c>
@@ -1355,8 +1344,8 @@
       <c r="A19" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="9">
-        <v>2.2942038143382302</v>
+      <c r="B19">
+        <v>1.2818574905395499</v>
       </c>
       <c r="C19">
         <v>3.1790446098824598</v>
@@ -1373,16 +1362,16 @@
       <c r="G19" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H19" s="11">
+      <c r="H19" s="10">
         <v>6.9167933755607498</v>
       </c>
-      <c r="I19" s="11">
+      <c r="I19" s="10">
         <v>7.6918990911074498</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="10">
         <v>8.6418529562595499</v>
       </c>
-      <c r="K19" s="11">
+      <c r="K19" s="10">
         <v>9.8390835440481492</v>
       </c>
       <c r="L19" s="3">
@@ -1401,46 +1390,47 @@
         <f t="shared" si="3"/>
         <v>0.47330379379092902</v>
       </c>
-      <c r="P19" s="19">
+      <c r="P19" s="16">
         <f t="shared" si="4"/>
         <v>0.41487396002467236</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="18">
-        <v>1796.8244529999999</v>
-      </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18">
+      <c r="A20" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="15">
+        <f>SUM(B13:B19)/7</f>
+        <v>3.7607499531337156</v>
+      </c>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15">
         <v>15.1045682929261</v>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="15">
         <v>16.466972683078801</v>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="15">
         <v>17.623530680131701</v>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="15">
         <v>18.626433459035201</v>
       </c>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="18"/>
-      <c r="P20" s="18"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="20"/>
+      <c r="B25" s="18"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -1464,16 +1454,16 @@
       <c r="G26" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H26" s="10" t="s">
+      <c r="H26" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I26" s="10" t="s">
+      <c r="I26" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="J26" s="10" t="s">
+      <c r="J26" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="K26" s="10" t="s">
+      <c r="K26" s="9" t="s">
         <v>28</v>
       </c>
       <c r="L26" s="2" t="s">
@@ -1496,8 +1486,8 @@
       <c r="A27" t="s">
         <v>9</v>
       </c>
-      <c r="B27" s="9">
-        <v>95.74904649154</v>
+      <c r="B27">
+        <v>33.394912081043202</v>
       </c>
       <c r="C27" s="3">
         <v>11.847161237319201</v>
@@ -1514,16 +1504,16 @@
       <c r="G27" s="3">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H27" s="11">
+      <c r="H27" s="10">
         <v>104.206596222385</v>
       </c>
-      <c r="I27" s="11">
+      <c r="I27" s="10">
         <v>103.825935221908</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27" s="10">
         <v>100.11177985049</v>
       </c>
-      <c r="K27" s="11">
+      <c r="K27" s="10">
         <v>93.901651246207095</v>
       </c>
       <c r="L27" s="3">
@@ -1542,7 +1532,7 @@
         <f>(K27-F27-G27)</f>
         <v>79.588151228937619</v>
       </c>
-      <c r="P27" s="19">
+      <c r="P27" s="16">
         <f>(L27+M27+N27+O27)/4</f>
         <v>85.879751347730888</v>
       </c>
@@ -1551,8 +1541,8 @@
       <c r="A28" t="s">
         <v>10</v>
       </c>
-      <c r="B28" s="9">
-        <v>19995.0293793397</v>
+      <c r="B28">
+        <v>48.978336830402398</v>
       </c>
       <c r="C28">
         <v>106.746648747265</v>
@@ -1569,16 +1559,16 @@
       <c r="G28" s="3">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H28" s="11">
+      <c r="H28" s="10">
         <v>198.878516435623</v>
       </c>
-      <c r="I28" s="11">
+      <c r="I28" s="10">
         <v>193.56502606161001</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28" s="10">
         <v>204.52682309183899</v>
       </c>
-      <c r="K28" s="11">
+      <c r="K28" s="10">
         <v>207.255575950614</v>
       </c>
       <c r="L28" s="3">
@@ -1597,7 +1587,7 @@
         <f t="shared" ref="O28:O33" si="8">(K28-F28-G28)</f>
         <v>80.81037650932673</v>
       </c>
-      <c r="P28" s="19">
+      <c r="P28" s="16">
         <f t="shared" ref="P28:P33" si="9">(L28+M28+N28+O28)/4</f>
         <v>84.207752355317467</v>
       </c>
@@ -1606,8 +1596,8 @@
       <c r="A29" t="s">
         <v>11</v>
       </c>
-      <c r="B29" s="9">
-        <v>138.138762226811</v>
+      <c r="B29">
+        <v>34.905319895629297</v>
       </c>
       <c r="C29">
         <v>11.2682738745265</v>
@@ -1624,16 +1614,16 @@
       <c r="G29" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H29" s="11">
+      <c r="H29" s="10">
         <v>104.699721246761</v>
       </c>
-      <c r="I29" s="11">
+      <c r="I29" s="10">
         <v>103.176413636536</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="10">
         <v>100.929154780147</v>
       </c>
-      <c r="K29" s="11">
+      <c r="K29" s="10">
         <v>95.117645530865104</v>
       </c>
       <c r="L29" s="3">
@@ -1652,7 +1642,7 @@
         <f t="shared" si="8"/>
         <v>80.620483171956437</v>
       </c>
-      <c r="P29" s="19">
+      <c r="P29" s="16">
         <f t="shared" si="9"/>
         <v>86.412720561728307</v>
       </c>
@@ -1661,8 +1651,8 @@
       <c r="A30" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="9">
-        <v>54800.687812623502</v>
+      <c r="B30">
+        <v>52.326840627060598</v>
       </c>
       <c r="C30">
         <v>64.767009309883903</v>
@@ -1679,16 +1669,16 @@
       <c r="G30" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="10">
         <v>164.52485036118699</v>
       </c>
-      <c r="I30" s="11">
+      <c r="I30" s="10">
         <v>172.540658884236</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="10">
         <v>183.230999074528</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30" s="10">
         <v>182.358312283896</v>
       </c>
       <c r="L30" s="3">
@@ -1707,7 +1697,7 @@
         <f t="shared" si="8"/>
         <v>90.073824111654332</v>
       </c>
-      <c r="P30" s="19">
+      <c r="P30" s="16">
         <f t="shared" si="9"/>
         <v>96.030329590467161</v>
       </c>
@@ -1716,8 +1706,8 @@
       <c r="A31" t="s">
         <v>1</v>
       </c>
-      <c r="B31" s="9">
-        <v>6011.8293762207004</v>
+      <c r="B31">
+        <v>35.575733653136602</v>
       </c>
       <c r="C31">
         <v>13.7873021123293</v>
@@ -1734,16 +1724,16 @@
       <c r="G31" s="3">
         <v>3.4031658544935599</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="10">
         <v>103.10741371392299</v>
       </c>
-      <c r="I31" s="11">
+      <c r="I31" s="10">
         <v>113.343025767809</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="10">
         <v>128.083347378882</v>
       </c>
-      <c r="K31" s="11">
+      <c r="K31" s="10">
         <v>139.43136468744001</v>
       </c>
       <c r="L31" s="3">
@@ -1762,7 +1752,7 @@
         <f t="shared" si="8"/>
         <v>81.608089257532541</v>
       </c>
-      <c r="P31" s="19">
+      <c r="P31" s="16">
         <f t="shared" si="9"/>
         <v>85.587489752049947</v>
       </c>
@@ -1771,8 +1761,8 @@
       <c r="A32" t="s">
         <v>2</v>
       </c>
-      <c r="B32" s="9">
-        <v>47.943197763883099</v>
+      <c r="B32">
+        <v>33.100447415879003</v>
       </c>
       <c r="C32" s="3">
         <v>11.4811841212213</v>
@@ -1789,16 +1779,16 @@
       <c r="G32" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="10">
         <v>103.38036423672099</v>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="10">
         <v>103.99572480142</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="10">
         <v>99.234147304171998</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32" s="10">
         <v>94.367099788090897</v>
       </c>
       <c r="L32" s="3">
@@ -1817,7 +1807,7 @@
         <f t="shared" si="8"/>
         <v>79.854729367027886</v>
       </c>
-      <c r="P32" s="19">
+      <c r="P32" s="16">
         <f t="shared" si="9"/>
         <v>85.775091111266221</v>
       </c>
@@ -1826,8 +1816,8 @@
       <c r="A33" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="9">
-        <v>54.362399237496497</v>
+      <c r="B33">
+        <v>34.768972609870602</v>
       </c>
       <c r="C33">
         <v>12.9621852923768</v>
@@ -1844,16 +1834,16 @@
       <c r="G33" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H33" s="11">
+      <c r="H33" s="10">
         <v>101.70695238601699</v>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="10">
         <v>110.026416640646</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="10">
         <v>122.731095552444</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="10">
         <v>138.09521327147601</v>
       </c>
       <c r="L33" s="3">
@@ -1872,46 +1862,47 @@
         <f t="shared" si="8"/>
         <v>81.613709437452314</v>
       </c>
-      <c r="P33" s="19">
+      <c r="P33" s="16">
         <f t="shared" si="9"/>
         <v>85.107365386333882</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B34" s="18">
-        <v>10720.412156353201</v>
-      </c>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="18">
+      <c r="A34" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="15">
+        <f>SUM(B27:B33)/7</f>
+        <v>39.007223301860243</v>
+      </c>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15">
         <v>125.7497103</v>
       </c>
-      <c r="I34" s="18">
+      <c r="I34" s="15">
         <v>128.573508482931</v>
       </c>
-      <c r="J34" s="18">
+      <c r="J34" s="15">
         <v>134.417065435768</v>
       </c>
-      <c r="K34" s="18">
+      <c r="K34" s="15">
         <v>135.633717420675</v>
       </c>
-      <c r="L34" s="18"/>
-      <c r="M34" s="18"/>
-      <c r="N34" s="18"/>
-      <c r="O34" s="18"/>
-      <c r="P34" s="18"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+      <c r="O34" s="15"/>
+      <c r="P34" s="15"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="20" t="s">
+      <c r="A40" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="20"/>
+      <c r="B40" s="18"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -1935,16 +1926,16 @@
       <c r="G41" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="10" t="s">
+      <c r="H41" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="I41" s="10" t="s">
+      <c r="I41" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="J41" s="10" t="s">
+      <c r="J41" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="K41" s="10" t="s">
+      <c r="K41" s="9" t="s">
         <v>32</v>
       </c>
       <c r="L41" s="2" t="s">
@@ -1967,8 +1958,8 @@
       <c r="A42" t="s">
         <v>9</v>
       </c>
-      <c r="B42" s="9">
-        <v>3144.16048723623</v>
+      <c r="B42">
+        <v>309.75627683317703</v>
       </c>
       <c r="C42" s="3">
         <v>16.172406414180401</v>
@@ -1985,16 +1976,16 @@
       <c r="G42" s="3">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H42" s="11">
+      <c r="H42" s="10">
         <v>1266.3802028626401</v>
       </c>
-      <c r="I42" s="11">
+      <c r="I42" s="10">
         <v>1239.2457168881199</v>
       </c>
-      <c r="J42" s="11">
+      <c r="J42" s="10">
         <v>1312.1272076882999</v>
       </c>
-      <c r="K42" s="11">
+      <c r="K42" s="10">
         <v>1330.2754645709399</v>
       </c>
       <c r="L42" s="3">
@@ -2019,56 +2010,56 @@
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
+      <c r="A43" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="13">
-        <v>137100.715637207</v>
-      </c>
-      <c r="C43" s="15">
+      <c r="B43">
+        <v>385.85945187496498</v>
+      </c>
+      <c r="C43" s="12">
         <v>152.29655436061199</v>
       </c>
-      <c r="D43" s="14">
+      <c r="D43" s="11">
         <v>144.29762564570601</v>
       </c>
-      <c r="E43" s="14">
+      <c r="E43" s="11">
         <v>160.05635477709001</v>
       </c>
-      <c r="F43" s="16">
+      <c r="F43" s="13">
         <v>173.15498055168001</v>
       </c>
-      <c r="G43" s="14">
+      <c r="G43" s="11">
         <v>3.4243865973862802</v>
       </c>
-      <c r="H43" s="11">
+      <c r="H43" s="10">
         <v>1398.5665355409801</v>
       </c>
-      <c r="I43" s="11">
+      <c r="I43" s="10">
         <v>1381.67841990958</v>
       </c>
-      <c r="J43" s="11">
+      <c r="J43" s="10">
         <v>1465.4698619411599</v>
       </c>
-      <c r="K43" s="11">
+      <c r="K43" s="10">
         <v>1479.3596455648601</v>
       </c>
-      <c r="L43" s="14">
+      <c r="L43" s="11">
         <f t="shared" si="10"/>
         <v>1242.8455945829819</v>
       </c>
-      <c r="M43" s="14">
+      <c r="M43" s="11">
         <f t="shared" si="11"/>
         <v>1233.9564076664878</v>
       </c>
-      <c r="N43" s="14">
+      <c r="N43" s="11">
         <f t="shared" ref="N43:N48" si="12">(J43-E43-G43)</f>
         <v>1301.9891205666836</v>
       </c>
-      <c r="O43" s="14">
+      <c r="O43" s="11">
         <f t="shared" ref="O43:O48" si="13">(K43-F43-G43)</f>
         <v>1302.7802784157939</v>
       </c>
-      <c r="P43" s="17">
+      <c r="P43" s="14">
         <f t="shared" ref="P43:P48" si="14">(L43+M43+N43+O43)/4</f>
         <v>1270.3928503079869</v>
       </c>
@@ -2077,8 +2068,8 @@
       <c r="A44" t="s">
         <v>11</v>
       </c>
-      <c r="B44" s="9">
-        <v>3125.5087894675999</v>
+      <c r="B44">
+        <v>302.57200193169399</v>
       </c>
       <c r="C44" s="3">
         <v>15.7964597682774</v>
@@ -2095,16 +2086,16 @@
       <c r="G44" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H44" s="11">
+      <c r="H44" s="10">
         <v>1270.54629717892</v>
       </c>
-      <c r="I44" s="11">
+      <c r="I44" s="10">
         <v>1241.23775242325</v>
       </c>
-      <c r="J44" s="11">
+      <c r="J44" s="10">
         <v>1301.87346783812</v>
       </c>
-      <c r="K44" s="11">
+      <c r="K44" s="10">
         <v>1312.7505429759001</v>
       </c>
       <c r="L44" s="3">
@@ -2132,8 +2123,8 @@
       <c r="A45" t="s">
         <v>12</v>
       </c>
-      <c r="B45" s="9">
-        <v>3642.0171727304801</v>
+      <c r="B45">
+        <v>320.56131679487402</v>
       </c>
       <c r="C45" s="3">
         <v>91.448995502374501</v>
@@ -2150,16 +2141,16 @@
       <c r="G45" s="3">
         <v>3.4322229428683699</v>
       </c>
-      <c r="H45" s="11">
+      <c r="H45" s="10">
         <v>1353.1058268342799</v>
       </c>
-      <c r="I45" s="11">
+      <c r="I45" s="10">
         <v>1340.8253010552301</v>
       </c>
-      <c r="J45" s="11">
+      <c r="J45" s="10">
         <v>1432.73518285777</v>
       </c>
-      <c r="K45" s="11">
+      <c r="K45" s="10">
         <v>1428.9955440608901</v>
       </c>
       <c r="L45" s="3">
@@ -2187,8 +2178,8 @@
       <c r="A46" t="s">
         <v>1</v>
       </c>
-      <c r="B46" s="9">
-        <v>3232.9062776467199</v>
+      <c r="B46">
+        <v>308.79380874664997</v>
       </c>
       <c r="C46" s="3">
         <v>17.691985893020401</v>
@@ -2205,16 +2196,16 @@
       <c r="G46" s="3">
         <v>3.4031658544935599</v>
       </c>
-      <c r="H46" s="11">
+      <c r="H46" s="10">
         <v>1258.5168948821799</v>
       </c>
-      <c r="I46" s="11">
+      <c r="I46" s="10">
         <v>1262.7569204172701</v>
       </c>
-      <c r="J46" s="11">
+      <c r="J46" s="10">
         <v>1337.6830662981699</v>
       </c>
-      <c r="K46" s="11">
+      <c r="K46" s="10">
         <v>1377.28891171451</v>
       </c>
       <c r="L46" s="3">
@@ -2242,8 +2233,8 @@
       <c r="A47" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="9">
-        <v>2798.6146199334498</v>
+      <c r="B47">
+        <v>307.16703915205102</v>
       </c>
       <c r="C47" s="3">
         <v>15.552245469805801</v>
@@ -2260,16 +2251,16 @@
       <c r="G47" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H47" s="11">
+      <c r="H47" s="10">
         <v>1262.12741147269</v>
       </c>
-      <c r="I47" s="11">
+      <c r="I47" s="10">
         <v>1247.39613110657</v>
       </c>
-      <c r="J47" s="11">
+      <c r="J47" s="10">
         <v>1312.9196750561</v>
       </c>
-      <c r="K47" s="11">
+      <c r="K47" s="10">
         <v>1309.10656011622</v>
       </c>
       <c r="L47" s="3">
@@ -2297,8 +2288,8 @@
       <c r="A48" t="s">
         <v>13</v>
       </c>
-      <c r="B48" s="9">
-        <v>3012.9789593293399</v>
+      <c r="B48">
+        <v>301.47144548476598</v>
       </c>
       <c r="C48" s="3">
         <v>15.354518245541801</v>
@@ -2315,16 +2306,16 @@
       <c r="G48" s="3">
         <v>3.4400745046623098</v>
       </c>
-      <c r="H48" s="11">
+      <c r="H48" s="10">
         <v>1269.7002746903299</v>
       </c>
-      <c r="I48" s="11">
+      <c r="I48" s="10">
         <v>1271.2879097467801</v>
       </c>
-      <c r="J48" s="11">
+      <c r="J48" s="10">
         <v>1357.9602965453701</v>
       </c>
-      <c r="K48" s="11">
+      <c r="K48" s="10">
         <v>1372.6979691172101</v>
       </c>
       <c r="L48" s="3">
@@ -2349,1170 +2340,1261 @@
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B49" s="18">
-        <v>3375.2124883947499</v>
-      </c>
-      <c r="C49" s="18"/>
-      <c r="D49" s="18"/>
-      <c r="E49" s="18"/>
-      <c r="F49" s="18"/>
-      <c r="G49" s="18"/>
-      <c r="H49" s="18">
+      <c r="A49" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B49" s="15">
+        <f>SUM(B42:B48)/7</f>
+        <v>319.45447725973958</v>
+      </c>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15">
         <v>1297.3683296223201</v>
       </c>
-      <c r="I49" s="18">
+      <c r="I49" s="15">
         <v>1282.61406826794</v>
       </c>
-      <c r="J49" s="18">
+      <c r="J49" s="15">
         <v>1360.455627</v>
       </c>
-      <c r="K49" s="18">
+      <c r="K49" s="15">
         <v>1372.5491509999999</v>
       </c>
-      <c r="L49" s="18"/>
-      <c r="M49" s="18"/>
-      <c r="N49" s="18"/>
-      <c r="O49" s="18"/>
-      <c r="P49" s="18"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="21"/>
+      <c r="L49" s="15"/>
+      <c r="M49" s="15"/>
+      <c r="N49" s="15"/>
+      <c r="O49" s="15"/>
+      <c r="P49" s="15"/>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="D55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="G55" s="5"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B56" s="5"/>
       <c r="D56" s="5"/>
       <c r="F56" s="5"/>
       <c r="G56" s="5"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B57" s="5"/>
-      <c r="D57" s="5"/>
-      <c r="F57" s="5"/>
+      <c r="A57" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B57" s="19"/>
+      <c r="C57" s="19"/>
+      <c r="D57" s="19"/>
+      <c r="E57" s="19"/>
+      <c r="F57" s="19"/>
       <c r="G57" s="5"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B58" s="22"/>
-      <c r="C58" s="22"/>
-      <c r="D58" s="22"/>
-      <c r="E58" s="22"/>
-      <c r="F58" s="22"/>
+      <c r="D58" s="5"/>
+      <c r="F58" s="5"/>
       <c r="G58" s="5"/>
+      <c r="K58" t="s">
+        <v>9</v>
+      </c>
+      <c r="N58" s="3">
+        <v>0.52516379831418403</v>
+      </c>
+      <c r="O58" s="3">
+        <f t="shared" ref="O58:O64" si="15">N58-G90</f>
+        <v>0.19962707040891103</v>
+      </c>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="D59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
+      <c r="A59" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G59" s="17" t="s">
+        <v>72</v>
+      </c>
       <c r="K59" t="s">
+        <v>10</v>
+      </c>
+      <c r="N59">
+        <v>32.977948012191398</v>
+      </c>
+      <c r="O59" s="3">
+        <f t="shared" si="15"/>
+        <v>19.1043947361294</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>9</v>
       </c>
-      <c r="N59" s="3">
-        <v>0.52516379831418403</v>
-      </c>
-      <c r="O59" s="3">
-        <f>N59-G91</f>
-        <v>0.19962707040891103</v>
-      </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F60" s="6" t="s">
-        <v>37</v>
+      <c r="B60">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="C60">
+        <v>1</v>
+      </c>
+      <c r="D60">
+        <v>1.7750263214111299</v>
+      </c>
+      <c r="E60" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F60" s="7">
+        <v>1.68681144714355</v>
+      </c>
+      <c r="G60">
+        <v>0.32553672790527299</v>
       </c>
       <c r="K60" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N60">
-        <v>32.977948012191398</v>
+        <v>0.49840760395546102</v>
       </c>
       <c r="O60" s="3">
-        <f>N60-G92</f>
-        <v>19.1043947361294</v>
+        <f t="shared" si="15"/>
+        <v>0.33232522175331303</v>
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B61">
-        <v>4.0050931003851096</v>
+        <v>54.5115243820917</v>
       </c>
       <c r="C61">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="D61">
-        <v>1.7750263214111299</v>
+        <v>22.880792617797798</v>
       </c>
       <c r="E61" s="1">
-        <v>4.3846666812896702E-3</v>
+        <v>1.77403353154659</v>
       </c>
       <c r="F61" s="7">
-        <v>1.68681144714355</v>
+        <v>18.5704231262207</v>
+      </c>
+      <c r="G61">
+        <v>13.873553276061999</v>
       </c>
       <c r="K61" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N61">
-        <v>0.49840760395546102</v>
+        <v>25.759887776849901</v>
       </c>
       <c r="O61" s="3">
-        <f>N61-G93</f>
-        <v>0.33232522175331303</v>
+        <f t="shared" si="15"/>
+        <v>16.615271649835741</v>
       </c>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B62">
-        <v>54.5115243820917</v>
+        <v>4.0775397573838204</v>
       </c>
       <c r="C62">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="D62">
-        <v>22.880792617797798</v>
+        <v>0.46491622924804599</v>
       </c>
       <c r="E62" s="1">
-        <v>1.77403353154659</v>
+        <v>4.3846666812896702E-3</v>
       </c>
       <c r="F62" s="7">
-        <v>18.5704231262207</v>
+        <v>0.40674209594726501</v>
+      </c>
+      <c r="G62">
+        <v>0.16608238220214799</v>
       </c>
       <c r="K62" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="N62">
-        <v>25.759887776849901</v>
+        <v>3.52255095970304</v>
       </c>
       <c r="O62" s="3">
-        <f>N62-G94</f>
-        <v>16.615271649835741</v>
+        <f t="shared" si="15"/>
+        <v>2.1187900496688701</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B63">
-        <v>4.0775397573838204</v>
+        <v>47.1892843685389</v>
       </c>
       <c r="C63">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="D63">
-        <v>0.46491622924804599</v>
+        <v>15.479326248168899</v>
       </c>
       <c r="E63" s="1">
-        <v>4.3846666812896702E-3</v>
+        <v>1.77403353154659</v>
       </c>
       <c r="F63" s="7">
-        <v>0.40674209594726501</v>
+        <v>12.6996040344238</v>
+      </c>
+      <c r="G63">
+        <v>9.1446161270141602</v>
       </c>
       <c r="K63" t="s">
-        <v>1</v>
-      </c>
-      <c r="N63">
-        <v>3.52255095970304</v>
+        <v>2</v>
+      </c>
+      <c r="N63" s="3">
+        <v>0.49062787411620901</v>
       </c>
       <c r="O63" s="3">
-        <f>N63-G95</f>
-        <v>2.1187900496688701</v>
+        <f t="shared" si="15"/>
+        <v>0.36078511593749901</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>1</v>
+      </c>
+      <c r="B64">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="C64">
+        <v>100</v>
+      </c>
+      <c r="D64">
+        <v>3.7736892700195299</v>
+      </c>
+      <c r="E64" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F64" s="7">
+        <v>3.41200828552246</v>
+      </c>
+      <c r="G64">
+        <v>1.4037609100341699</v>
+      </c>
+      <c r="K64" t="s">
+        <v>13</v>
+      </c>
+      <c r="N64">
+        <v>3.1790446098824598</v>
+      </c>
+      <c r="O64" s="3">
+        <f t="shared" si="15"/>
+        <v>1.89718711934291</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>2</v>
+      </c>
+      <c r="B65">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="D65">
+        <v>0.19145011901855399</v>
+      </c>
+      <c r="E65" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F65" s="7">
+        <v>0.13566017150878901</v>
+      </c>
+      <c r="G65">
+        <v>0.12984275817870999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>13</v>
+      </c>
+      <c r="B66">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="C66">
+        <v>100</v>
+      </c>
+      <c r="D66">
+        <v>3.9923191070556601</v>
+      </c>
+      <c r="E66" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F66" s="7">
+        <v>3.5090446472167902</v>
+      </c>
+      <c r="G66">
+        <v>1.2818574905395499</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I67" s="5"/>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I68" s="5"/>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G69" s="17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>9</v>
+      </c>
+      <c r="B70">
+        <v>4.0353076186722596</v>
+      </c>
+      <c r="C70">
+        <v>1</v>
+      </c>
+      <c r="D70">
+        <v>1.78432464599609</v>
+      </c>
+      <c r="E70" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F70" s="7">
+        <v>1.6944408416748</v>
+      </c>
+      <c r="G70">
+        <v>0.32553672790527299</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>10</v>
+      </c>
+      <c r="B71">
+        <v>48.675797406364801</v>
+      </c>
+      <c r="C71">
+        <v>1000</v>
+      </c>
+      <c r="D71">
+        <v>20.764112472534102</v>
+      </c>
+      <c r="E71" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F71" s="7">
+        <v>16.4527893066406</v>
+      </c>
+      <c r="G71">
+        <v>13.873553276061999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>11</v>
+      </c>
+      <c r="B72">
+        <v>4.1707241313894299</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72">
+        <v>0.43320655822753901</v>
+      </c>
+      <c r="E72" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F72" s="7">
+        <v>0.37431716918945301</v>
+      </c>
+      <c r="G72">
+        <v>0.16608238220214799</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>12</v>
       </c>
-      <c r="B64">
-        <v>47.1892843685389</v>
-      </c>
-      <c r="C64">
+      <c r="B73">
+        <v>44.808815805147901</v>
+      </c>
+      <c r="C73">
         <v>1000</v>
       </c>
-      <c r="D64">
-        <v>15.479326248168899</v>
-      </c>
-      <c r="E64" s="1">
-        <v>1.77403353154659</v>
-      </c>
-      <c r="F64" s="7">
-        <v>12.6996040344238</v>
-      </c>
-      <c r="K64" t="s">
+      <c r="D73">
+        <v>14.152050018310501</v>
+      </c>
+      <c r="E73" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F73" s="7">
+        <v>11.4581584930419</v>
+      </c>
+      <c r="G73">
+        <v>9.1446161270141602</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>1</v>
+      </c>
+      <c r="B74">
+        <v>9.8086684739508598</v>
+      </c>
+      <c r="C74">
+        <v>100</v>
+      </c>
+      <c r="D74">
+        <v>3.6182403564453098</v>
+      </c>
+      <c r="E74" s="1">
+        <v>0.170979648828506</v>
+      </c>
+      <c r="F74" s="7">
+        <v>3.2749176025390598</v>
+      </c>
+      <c r="G74">
+        <v>1.4037609100341699</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>2</v>
       </c>
-      <c r="N64" s="3">
-        <v>0.49062787411620901</v>
-      </c>
-      <c r="O64" s="3">
-        <f>N64-G96</f>
-        <v>0.36078511593749901</v>
-      </c>
-    </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+      <c r="B75">
+        <v>4.0890994634011797</v>
+      </c>
+      <c r="C75">
         <v>1</v>
       </c>
-      <c r="B65">
-        <v>11.208388920637001</v>
-      </c>
-      <c r="C65">
+      <c r="D75">
+        <v>0.30469894409179599</v>
+      </c>
+      <c r="E75" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F75" s="7">
+        <v>0.24819374084472601</v>
+      </c>
+      <c r="G75">
+        <v>0.12984275817870999</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>13</v>
+      </c>
+      <c r="B76">
+        <v>8.6418529562595499</v>
+      </c>
+      <c r="C76">
         <v>100</v>
       </c>
-      <c r="D65">
-        <v>3.7736892700195299</v>
-      </c>
-      <c r="E65" s="1">
-        <v>0.20086206495761799</v>
-      </c>
-      <c r="F65" s="7">
-        <v>3.41200828552246</v>
-      </c>
-      <c r="K65" t="s">
+      <c r="D76">
+        <v>3.2210350036621</v>
+      </c>
+      <c r="E76" s="1">
+        <v>0.170979648828506</v>
+      </c>
+      <c r="F76" s="7">
+        <v>2.8343200683593701</v>
+      </c>
+      <c r="G76">
+        <v>1.2818574905395499</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G79" s="17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>9</v>
+      </c>
+      <c r="B80">
+        <v>4.02605646143118</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80">
+        <v>1.7490386962890601</v>
+      </c>
+      <c r="E80" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F80" s="7">
+        <v>1.66249275207519</v>
+      </c>
+      <c r="G80">
+        <v>0.32553672790527299</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>10</v>
+      </c>
+      <c r="B81">
+        <v>45.799138335569502</v>
+      </c>
+      <c r="C81">
+        <v>1000</v>
+      </c>
+      <c r="D81">
+        <v>19.1633701324462</v>
+      </c>
+      <c r="E81" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F81" s="7">
+        <v>14.9691104888916</v>
+      </c>
+      <c r="G81">
+        <v>13.873553276061999</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82">
+        <v>4.1628384834501704</v>
+      </c>
+      <c r="C82">
+        <v>1</v>
+      </c>
+      <c r="D82">
+        <v>0.53834915161132801</v>
+      </c>
+      <c r="E82" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F82" s="7">
+        <v>0.39219856262206998</v>
+      </c>
+      <c r="G82">
+        <v>0.16608238220214799</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>12</v>
+      </c>
+      <c r="B83">
+        <v>42.259016332980003</v>
+      </c>
+      <c r="C83">
+        <v>1000</v>
+      </c>
+      <c r="D83">
+        <v>12.4282836914062</v>
+      </c>
+      <c r="E83" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F83" s="7">
+        <v>9.6678733825683594</v>
+      </c>
+      <c r="G83">
+        <v>9.1446161270141602</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>1</v>
+      </c>
+      <c r="B84">
+        <v>8.8410975673074592</v>
+      </c>
+      <c r="C84">
+        <v>100</v>
+      </c>
+      <c r="D84">
+        <v>2.7823448181152299</v>
+      </c>
+      <c r="E84" s="1">
+        <v>0.16103312373161299</v>
+      </c>
+      <c r="F84" s="7">
+        <v>2.42781639099121</v>
+      </c>
+      <c r="G84">
+        <v>1.4037609100341699</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>2</v>
+      </c>
+      <c r="B85">
+        <v>4.1352269590162702</v>
+      </c>
+      <c r="C85">
+        <v>1</v>
+      </c>
+      <c r="D85">
+        <v>0.392913818359375</v>
+      </c>
+      <c r="E85" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F85" s="7">
+        <v>0.32162666320800698</v>
+      </c>
+      <c r="G85">
+        <v>0.12984275817870999</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>13</v>
       </c>
-      <c r="N65">
-        <v>3.1790446098824598</v>
-      </c>
-      <c r="O65" s="3">
-        <f>N65-G97</f>
-        <v>1.89718711934291</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+      <c r="B86">
+        <v>7.6918990911074498</v>
+      </c>
+      <c r="C86">
+        <v>100</v>
+      </c>
+      <c r="D86">
+        <v>2.16484069824218</v>
+      </c>
+      <c r="E86" s="1">
+        <v>0.16103312373161299</v>
+      </c>
+      <c r="F86" s="7">
+        <v>1.79862976074218</v>
+      </c>
+      <c r="G86">
+        <v>1.2818574905395499</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E89" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G89" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="H89" s="17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>9</v>
+      </c>
+      <c r="B90">
+        <v>3.9895902707595199</v>
+      </c>
+      <c r="C90">
+        <v>1</v>
+      </c>
+      <c r="D90">
+        <v>1.77168846130371</v>
+      </c>
+      <c r="E90" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F90" s="7">
+        <v>1.6837120056152299</v>
+      </c>
+      <c r="G90">
+        <v>0.32553672790527299</v>
+      </c>
+      <c r="H90">
+        <v>0.48804283142089799</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>10</v>
+      </c>
+      <c r="B91">
+        <v>41.8466371823881</v>
+      </c>
+      <c r="C91">
+        <v>1000</v>
+      </c>
+      <c r="D91">
+        <v>16.952753067016602</v>
+      </c>
+      <c r="E91" s="1">
+        <v>1.54353864490985</v>
+      </c>
+      <c r="F91" s="7">
+        <v>12.8097534179687</v>
+      </c>
+      <c r="G91">
+        <v>13.873553276061999</v>
+      </c>
+      <c r="H91">
+        <v>24.1720676422119</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>11</v>
+      </c>
+      <c r="B92">
+        <v>4.0147860416504804</v>
+      </c>
+      <c r="C92">
+        <v>1</v>
+      </c>
+      <c r="D92">
+        <v>0.55480003356933505</v>
+      </c>
+      <c r="E92" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F92" s="7">
+        <v>0.47087669372558499</v>
+      </c>
+      <c r="G92">
+        <v>0.16608238220214799</v>
+      </c>
+      <c r="H92">
+        <v>0.47612190246581998</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>12</v>
+      </c>
+      <c r="B93">
+        <v>38.3633321341607</v>
+      </c>
+      <c r="C93">
+        <v>1000</v>
+      </c>
+      <c r="D93">
+        <v>11.2018585205078</v>
+      </c>
+      <c r="E93" s="1">
+        <v>1.54353864490985</v>
+      </c>
+      <c r="F93" s="7">
+        <v>8.54420661926269</v>
+      </c>
+      <c r="G93">
+        <v>9.1446161270141602</v>
+      </c>
+      <c r="H93">
+        <v>20.414829254150298</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>1</v>
+      </c>
+      <c r="B94">
+        <v>7.9163517599320397</v>
+      </c>
+      <c r="C94">
+        <v>100</v>
+      </c>
+      <c r="D94">
+        <v>1.68442726135253</v>
+      </c>
+      <c r="E94" s="1">
+        <v>0.159744173288345</v>
+      </c>
+      <c r="F94" s="7">
+        <v>1.3589859008789</v>
+      </c>
+      <c r="G94">
+        <v>1.4037609100341699</v>
+      </c>
+      <c r="H94">
+        <v>2.92348861694335</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>2</v>
       </c>
-      <c r="B66">
-        <v>4.1074357013928502</v>
-      </c>
-      <c r="C66">
+      <c r="B95">
+        <v>4.0209035037549397</v>
+      </c>
+      <c r="C95">
         <v>1</v>
       </c>
-      <c r="D66">
-        <v>0.19145011901855399</v>
-      </c>
-      <c r="E66" s="1">
-        <v>4.3846666812896702E-3</v>
-      </c>
-      <c r="F66" s="7">
-        <v>0.13566017150878901</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+      <c r="D95">
+        <v>0.32210350036620999</v>
+      </c>
+      <c r="E95" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F95" s="7">
+        <v>0.25033950805664001</v>
+      </c>
+      <c r="G95">
+        <v>0.12984275817870999</v>
+      </c>
+      <c r="H95">
+        <v>0.42486190795898399</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>13</v>
       </c>
-      <c r="B67">
-        <v>9.8390835440481492</v>
-      </c>
-      <c r="C67">
+      <c r="B96">
+        <v>6.9167933755607498</v>
+      </c>
+      <c r="C96">
         <v>100</v>
       </c>
-      <c r="D67">
-        <v>3.9923191070556601</v>
-      </c>
-      <c r="E67" s="1">
-        <v>0.20086206495761799</v>
-      </c>
-      <c r="F67" s="7">
-        <v>3.5090446472167902</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="I68" s="5"/>
-    </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="I69" s="5"/>
-    </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A70" s="2" t="s">
+      <c r="D96">
+        <v>1.6908645629882799</v>
+      </c>
+      <c r="E96" s="1">
+        <v>0.159744173288345</v>
+      </c>
+      <c r="F96" s="7">
+        <v>1.34897232055664</v>
+      </c>
+      <c r="G96">
+        <v>1.2818574905395499</v>
+      </c>
+      <c r="H96">
+        <v>2.4752616882324201</v>
+      </c>
+    </row>
+    <row r="109" spans="7:19" x14ac:dyDescent="0.25">
+      <c r="G109" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F70" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="H109" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="I109" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="J109" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="K109" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="L109" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="M109" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N109" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="O109" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="P109" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q109" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R109" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="S109" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="110" spans="7:19" x14ac:dyDescent="0.25">
+      <c r="G110" t="s">
         <v>9</v>
       </c>
-      <c r="B71">
+      <c r="H110" s="10">
+        <v>3.9895902707595199</v>
+      </c>
+      <c r="I110" s="10">
+        <v>4.02605646143118</v>
+      </c>
+      <c r="J110" s="10">
         <v>4.0353076186722596</v>
       </c>
-      <c r="C71">
-        <v>1</v>
-      </c>
-      <c r="D71">
-        <v>1.78432464599609</v>
-      </c>
-      <c r="E71" s="1">
-        <v>4.3548643589019697E-3</v>
-      </c>
-      <c r="F71" s="7">
-        <v>1.6944408416748</v>
-      </c>
-    </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="K110" s="10">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="L110" s="10">
+        <v>104.206596222385</v>
+      </c>
+      <c r="M110" s="10">
+        <v>103.825935221908</v>
+      </c>
+      <c r="N110" s="10">
+        <v>100.11177985049</v>
+      </c>
+      <c r="O110" s="10">
+        <v>93.901651246207095</v>
+      </c>
+      <c r="P110">
+        <f>L110-H110</f>
+        <v>100.21700595162548</v>
+      </c>
+      <c r="Q110">
+        <f>M110-I110</f>
+        <v>99.799878760476815</v>
+      </c>
+      <c r="R110">
+        <f>N110-J110</f>
+        <v>96.076472231817732</v>
+      </c>
+      <c r="S110">
+        <f>O110-K110</f>
+        <v>89.896558145821984</v>
+      </c>
+    </row>
+    <row r="111" spans="7:19" x14ac:dyDescent="0.25">
+      <c r="G111" t="s">
         <v>10</v>
       </c>
-      <c r="B72">
+      <c r="H111" s="10">
+        <v>41.8466371823881</v>
+      </c>
+      <c r="I111" s="10">
+        <v>45.799138335569502</v>
+      </c>
+      <c r="J111" s="10">
         <v>48.675797406364801</v>
       </c>
-      <c r="C72">
-        <v>1000</v>
-      </c>
-      <c r="D72">
-        <v>20.764112472534102</v>
-      </c>
-      <c r="E72" s="1">
-        <v>1.6100797802209801</v>
-      </c>
-      <c r="F72" s="7">
-        <v>16.4527893066406</v>
-      </c>
-    </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="K111" s="10">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="L111" s="10">
+        <v>198.878516435623</v>
+      </c>
+      <c r="M111" s="10">
+        <v>193.56502606161001</v>
+      </c>
+      <c r="N111" s="10">
+        <v>204.52682309183899</v>
+      </c>
+      <c r="O111" s="10">
+        <v>207.255575950614</v>
+      </c>
+      <c r="P111">
+        <f t="shared" ref="P111:P116" si="16">L111-H111</f>
+        <v>157.03187925323491</v>
+      </c>
+      <c r="Q111">
+        <f t="shared" ref="Q111:Q116" si="17">M111-I111</f>
+        <v>147.76588772604052</v>
+      </c>
+      <c r="R111">
+        <f t="shared" ref="R111:R116" si="18">N111-J111</f>
+        <v>155.85102568547418</v>
+      </c>
+      <c r="S111">
+        <f t="shared" ref="S111:S116" si="19">O111-K111</f>
+        <v>152.74405156852231</v>
+      </c>
+    </row>
+    <row r="112" spans="7:19" x14ac:dyDescent="0.25">
+      <c r="G112" t="s">
         <v>11</v>
       </c>
-      <c r="B73">
+      <c r="H112" s="10">
+        <v>4.0147860416504804</v>
+      </c>
+      <c r="I112" s="10">
+        <v>4.1628384834501704</v>
+      </c>
+      <c r="J112" s="10">
         <v>4.1707241313894299</v>
       </c>
-      <c r="C73">
-        <v>1</v>
-      </c>
-      <c r="D73">
-        <v>0.43320655822753901</v>
-      </c>
-      <c r="E73" s="1">
-        <v>4.3548643589019697E-3</v>
-      </c>
-      <c r="F73" s="7">
-        <v>0.37431716918945301</v>
-      </c>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>12</v>
-      </c>
-      <c r="B74">
-        <v>44.808815805147901</v>
-      </c>
-      <c r="C74">
-        <v>1000</v>
-      </c>
-      <c r="D74">
-        <v>14.152050018310501</v>
-      </c>
-      <c r="E74" s="1">
-        <v>1.6100797802209801</v>
-      </c>
-      <c r="F74" s="7">
-        <v>11.4581584930419</v>
-      </c>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>1</v>
-      </c>
-      <c r="B75">
-        <v>9.8086684739508598</v>
-      </c>
-      <c r="C75">
-        <v>100</v>
-      </c>
-      <c r="D75">
-        <v>3.6182403564453098</v>
-      </c>
-      <c r="E75" s="1">
-        <v>0.170979648828506</v>
-      </c>
-      <c r="F75" s="7">
-        <v>3.2749176025390598</v>
-      </c>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>2</v>
-      </c>
-      <c r="B76">
-        <v>4.0890994634011797</v>
-      </c>
-      <c r="C76">
-        <v>1</v>
-      </c>
-      <c r="D76">
-        <v>0.30469894409179599</v>
-      </c>
-      <c r="E76" s="1">
-        <v>4.3548643589019697E-3</v>
-      </c>
-      <c r="F76" s="7">
-        <v>0.24819374084472601</v>
-      </c>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
-        <v>13</v>
-      </c>
-      <c r="B77">
-        <v>8.6418529562595499</v>
-      </c>
-      <c r="C77">
-        <v>100</v>
-      </c>
-      <c r="D77">
-        <v>3.2210350036621</v>
-      </c>
-      <c r="E77" s="1">
-        <v>0.170979648828506</v>
-      </c>
-      <c r="F77" s="7">
-        <v>2.8343200683593701</v>
-      </c>
-    </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A80" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F80" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
-        <v>9</v>
-      </c>
-      <c r="B81">
-        <v>4.02605646143118</v>
-      </c>
-      <c r="C81">
-        <v>1</v>
-      </c>
-      <c r="D81">
-        <v>1.7490386962890601</v>
-      </c>
-      <c r="E81" s="1">
-        <v>3.89851629734039E-3</v>
-      </c>
-      <c r="F81" s="7">
-        <v>1.66249275207519</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>10</v>
-      </c>
-      <c r="B82">
-        <v>45.799138335569502</v>
-      </c>
-      <c r="C82">
-        <v>1000</v>
-      </c>
-      <c r="D82">
-        <v>19.1633701324462</v>
-      </c>
-      <c r="E82" s="1">
-        <v>1.62918865680694</v>
-      </c>
-      <c r="F82" s="7">
-        <v>14.9691104888916</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>11</v>
-      </c>
-      <c r="B83">
-        <v>4.1628384834501704</v>
-      </c>
-      <c r="C83">
-        <v>1</v>
-      </c>
-      <c r="D83">
-        <v>0.53834915161132801</v>
-      </c>
-      <c r="E83" s="1">
-        <v>3.89851629734039E-3</v>
-      </c>
-      <c r="F83" s="7">
-        <v>0.39219856262206998</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>12</v>
-      </c>
-      <c r="B84">
-        <v>42.259016332980003</v>
-      </c>
-      <c r="C84">
-        <v>1000</v>
-      </c>
-      <c r="D84">
-        <v>12.4282836914062</v>
-      </c>
-      <c r="E84" s="1">
-        <v>1.62918865680694</v>
-      </c>
-      <c r="F84" s="7">
-        <v>9.6678733825683594</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>1</v>
-      </c>
-      <c r="B85">
-        <v>8.8410975673074592</v>
-      </c>
-      <c r="C85">
-        <v>100</v>
-      </c>
-      <c r="D85">
-        <v>2.7823448181152299</v>
-      </c>
-      <c r="E85" s="1">
-        <v>0.16103312373161299</v>
-      </c>
-      <c r="F85" s="7">
-        <v>2.42781639099121</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>2</v>
-      </c>
-      <c r="B86">
-        <v>4.1352269590162702</v>
-      </c>
-      <c r="C86">
-        <v>1</v>
-      </c>
-      <c r="D86">
-        <v>0.392913818359375</v>
-      </c>
-      <c r="E86" s="1">
-        <v>3.89851629734039E-3</v>
-      </c>
-      <c r="F86" s="7">
-        <v>0.32162666320800698</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>13</v>
-      </c>
-      <c r="B87">
-        <v>7.6918990911074498</v>
-      </c>
-      <c r="C87">
-        <v>100</v>
-      </c>
-      <c r="D87">
-        <v>2.16484069824218</v>
-      </c>
-      <c r="E87" s="1">
-        <v>0.16103312373161299</v>
-      </c>
-      <c r="F87" s="7">
-        <v>1.79862976074218</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F90" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G90" s="32" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>9</v>
-      </c>
-      <c r="B91">
-        <v>3.9895902707595199</v>
-      </c>
-      <c r="C91">
-        <v>1</v>
-      </c>
-      <c r="D91">
-        <v>1.77168846130371</v>
-      </c>
-      <c r="E91" s="1">
-        <v>4.3399631977081299E-3</v>
-      </c>
-      <c r="F91" s="7">
-        <v>1.6837120056152299</v>
-      </c>
-      <c r="G91">
-        <v>0.32553672790527299</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>10</v>
-      </c>
-      <c r="B92">
-        <v>41.8466371823881</v>
-      </c>
-      <c r="C92">
-        <v>1000</v>
-      </c>
-      <c r="D92">
-        <v>16.952753067016602</v>
-      </c>
-      <c r="E92" s="1">
-        <v>1.54353864490985</v>
-      </c>
-      <c r="F92" s="7">
-        <v>12.8097534179687</v>
-      </c>
-      <c r="G92">
-        <v>13.873553276061999</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>11</v>
-      </c>
-      <c r="B93">
-        <v>4.0147860416504804</v>
-      </c>
-      <c r="C93">
-        <v>1</v>
-      </c>
-      <c r="D93">
-        <v>0.55480003356933505</v>
-      </c>
-      <c r="E93" s="1">
-        <v>4.3399631977081299E-3</v>
-      </c>
-      <c r="F93" s="7">
-        <v>0.47087669372558499</v>
-      </c>
-      <c r="G93">
-        <v>0.16608238220214799</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>12</v>
-      </c>
-      <c r="B94">
-        <v>38.3633321341607</v>
-      </c>
-      <c r="C94">
-        <v>1000</v>
-      </c>
-      <c r="D94">
-        <v>11.2018585205078</v>
-      </c>
-      <c r="E94" s="1">
-        <v>1.54353864490985</v>
-      </c>
-      <c r="F94" s="7">
-        <v>8.54420661926269</v>
-      </c>
-      <c r="G94">
-        <v>9.1446161270141602</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>1</v>
-      </c>
-      <c r="B95">
-        <v>7.9163517599320397</v>
-      </c>
-      <c r="C95">
-        <v>100</v>
-      </c>
-      <c r="D95">
-        <v>1.68442726135253</v>
-      </c>
-      <c r="E95" s="1">
-        <v>0.159744173288345</v>
-      </c>
-      <c r="F95" s="7">
-        <v>1.3589859008789</v>
-      </c>
-      <c r="G95">
-        <v>1.4037609100341699</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>2</v>
-      </c>
-      <c r="B96">
-        <v>4.0209035037549397</v>
-      </c>
-      <c r="C96">
-        <v>1</v>
-      </c>
-      <c r="D96">
-        <v>0.32210350036620999</v>
-      </c>
-      <c r="E96" s="1">
-        <v>4.3399631977081299E-3</v>
-      </c>
-      <c r="F96" s="7">
-        <v>0.25033950805664001</v>
-      </c>
-      <c r="G96">
-        <v>0.12984275817870999</v>
-      </c>
-    </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>13</v>
-      </c>
-      <c r="B97">
-        <v>6.9167933755607498</v>
-      </c>
-      <c r="C97">
-        <v>100</v>
-      </c>
-      <c r="D97">
-        <v>1.6908645629882799</v>
-      </c>
-      <c r="E97" s="1">
-        <v>0.159744173288345</v>
-      </c>
-      <c r="F97" s="7">
-        <v>1.34897232055664</v>
-      </c>
-      <c r="G97">
-        <v>1.2818574905395499</v>
-      </c>
-    </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="G110" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="H110" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="I110" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="J110" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="K110" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="L110" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="M110" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="N110" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="O110" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="P110" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q110" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="R110" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="S110" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="G111" t="s">
-        <v>9</v>
-      </c>
-      <c r="H111" s="11">
-        <v>3.9895902707595199</v>
-      </c>
-      <c r="I111" s="11">
-        <v>4.02605646143118</v>
-      </c>
-      <c r="J111" s="11">
-        <v>4.0353076186722596</v>
-      </c>
-      <c r="K111" s="11">
-        <v>4.0050931003851096</v>
-      </c>
-      <c r="L111" s="11">
-        <v>104.206596222385</v>
-      </c>
-      <c r="M111" s="11">
-        <v>103.825935221908</v>
-      </c>
-      <c r="N111" s="11">
-        <v>100.11177985049</v>
-      </c>
-      <c r="O111" s="11">
-        <v>93.901651246207095</v>
-      </c>
-      <c r="P111">
-        <f>L111-H111</f>
-        <v>100.21700595162548</v>
-      </c>
-      <c r="Q111">
-        <f>M111-I111</f>
-        <v>99.799878760476815</v>
-      </c>
-      <c r="R111">
-        <f>N111-J111</f>
-        <v>96.076472231817732</v>
-      </c>
-      <c r="S111">
-        <f>O111-K111</f>
-        <v>89.896558145821984</v>
-      </c>
-    </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="G112" t="s">
-        <v>10</v>
-      </c>
-      <c r="H112" s="11">
-        <v>41.8466371823881</v>
-      </c>
-      <c r="I112" s="11">
-        <v>45.799138335569502</v>
-      </c>
-      <c r="J112" s="11">
-        <v>48.675797406364801</v>
-      </c>
-      <c r="K112" s="11">
-        <v>54.5115243820917</v>
-      </c>
-      <c r="L112" s="11">
-        <v>198.878516435623</v>
-      </c>
-      <c r="M112" s="11">
-        <v>193.56502606161001</v>
-      </c>
-      <c r="N112" s="11">
-        <v>204.52682309183899</v>
-      </c>
-      <c r="O112" s="11">
-        <v>207.255575950614</v>
+      <c r="K112" s="10">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="L112" s="10">
+        <v>104.699721246761</v>
+      </c>
+      <c r="M112" s="10">
+        <v>103.176413636536</v>
+      </c>
+      <c r="N112" s="10">
+        <v>100.929154780147</v>
+      </c>
+      <c r="O112" s="10">
+        <v>95.117645530865104</v>
       </c>
       <c r="P112">
-        <f t="shared" ref="P112:P117" si="15">L112-H112</f>
-        <v>157.03187925323491</v>
+        <f t="shared" si="16"/>
+        <v>100.68493520511052</v>
       </c>
       <c r="Q112">
-        <f t="shared" ref="Q112:Q117" si="16">M112-I112</f>
-        <v>147.76588772604052</v>
+        <f t="shared" si="17"/>
+        <v>99.013575153085824</v>
       </c>
       <c r="R112">
-        <f t="shared" ref="R112:R117" si="17">N112-J112</f>
-        <v>155.85102568547418</v>
+        <f t="shared" si="18"/>
+        <v>96.758430648757567</v>
       </c>
       <c r="S112">
-        <f t="shared" ref="S112:S117" si="18">O112-K112</f>
-        <v>152.74405156852231</v>
+        <f t="shared" si="19"/>
+        <v>91.040105773481287</v>
       </c>
     </row>
     <row r="113" spans="7:19" x14ac:dyDescent="0.25">
       <c r="G113" t="s">
-        <v>11</v>
-      </c>
-      <c r="H113" s="11">
-        <v>4.0147860416504804</v>
-      </c>
-      <c r="I113" s="11">
-        <v>4.1628384834501704</v>
-      </c>
-      <c r="J113" s="11">
-        <v>4.1707241313894299</v>
-      </c>
-      <c r="K113" s="11">
-        <v>4.0775397573838204</v>
-      </c>
-      <c r="L113" s="11">
-        <v>104.699721246761</v>
-      </c>
-      <c r="M113" s="11">
-        <v>103.176413636536</v>
-      </c>
-      <c r="N113" s="11">
-        <v>100.929154780147</v>
-      </c>
-      <c r="O113" s="11">
-        <v>95.117645530865104</v>
+        <v>12</v>
+      </c>
+      <c r="H113" s="10">
+        <v>38.3633321341607</v>
+      </c>
+      <c r="I113" s="10">
+        <v>42.259016332980003</v>
+      </c>
+      <c r="J113" s="10">
+        <v>44.808815805147901</v>
+      </c>
+      <c r="K113" s="10">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="L113" s="10">
+        <v>164.52485036118699</v>
+      </c>
+      <c r="M113" s="10">
+        <v>172.540658884236</v>
+      </c>
+      <c r="N113" s="10">
+        <v>183.230999074528</v>
+      </c>
+      <c r="O113" s="10">
+        <v>182.358312283896</v>
       </c>
       <c r="P113">
-        <f t="shared" si="15"/>
-        <v>100.68493520511052</v>
+        <f t="shared" si="16"/>
+        <v>126.16151822702629</v>
       </c>
       <c r="Q113">
-        <f t="shared" si="16"/>
-        <v>99.013575153085824</v>
+        <f t="shared" si="17"/>
+        <v>130.281642551256</v>
       </c>
       <c r="R113">
-        <f t="shared" si="17"/>
-        <v>96.758430648757567</v>
+        <f t="shared" si="18"/>
+        <v>138.4221832693801</v>
       </c>
       <c r="S113">
-        <f t="shared" si="18"/>
-        <v>91.040105773481287</v>
+        <f t="shared" si="19"/>
+        <v>135.16902791535711</v>
       </c>
     </row>
     <row r="114" spans="7:19" x14ac:dyDescent="0.25">
       <c r="G114" t="s">
-        <v>12</v>
-      </c>
-      <c r="H114" s="11">
-        <v>38.3633321341607</v>
-      </c>
-      <c r="I114" s="11">
-        <v>42.259016332980003</v>
-      </c>
-      <c r="J114" s="11">
-        <v>44.808815805147901</v>
-      </c>
-      <c r="K114" s="11">
-        <v>47.1892843685389</v>
-      </c>
-      <c r="L114" s="11">
-        <v>164.52485036118699</v>
-      </c>
-      <c r="M114" s="11">
-        <v>172.540658884236</v>
-      </c>
-      <c r="N114" s="11">
-        <v>183.230999074528</v>
-      </c>
-      <c r="O114" s="11">
-        <v>182.358312283896</v>
+        <v>1</v>
+      </c>
+      <c r="H114" s="10">
+        <v>7.9163517599320397</v>
+      </c>
+      <c r="I114" s="10">
+        <v>8.8410975673074592</v>
+      </c>
+      <c r="J114" s="10">
+        <v>9.8086684739508598</v>
+      </c>
+      <c r="K114" s="10">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="L114" s="10">
+        <v>103.10741371392299</v>
+      </c>
+      <c r="M114" s="10">
+        <v>113.343025767809</v>
+      </c>
+      <c r="N114" s="10">
+        <v>128.083347378882</v>
+      </c>
+      <c r="O114" s="10">
+        <v>139.43136468744001</v>
       </c>
       <c r="P114">
-        <f t="shared" si="15"/>
-        <v>126.16151822702629</v>
+        <f t="shared" si="16"/>
+        <v>95.191061953990953</v>
       </c>
       <c r="Q114">
-        <f t="shared" si="16"/>
-        <v>130.281642551256</v>
+        <f t="shared" si="17"/>
+        <v>104.50192820050154</v>
       </c>
       <c r="R114">
-        <f t="shared" si="17"/>
-        <v>138.4221832693801</v>
+        <f t="shared" si="18"/>
+        <v>118.27467890493114</v>
       </c>
       <c r="S114">
-        <f t="shared" si="18"/>
-        <v>135.16902791535711</v>
+        <f t="shared" si="19"/>
+        <v>128.22297576680302</v>
       </c>
     </row>
     <row r="115" spans="7:19" x14ac:dyDescent="0.25">
       <c r="G115" t="s">
-        <v>1</v>
-      </c>
-      <c r="H115" s="11">
-        <v>7.9163517599320397</v>
-      </c>
-      <c r="I115" s="11">
-        <v>8.8410975673074592</v>
-      </c>
-      <c r="J115" s="11">
-        <v>9.8086684739508598</v>
-      </c>
-      <c r="K115" s="11">
-        <v>11.208388920637001</v>
-      </c>
-      <c r="L115" s="11">
-        <v>103.10741371392299</v>
-      </c>
-      <c r="M115" s="11">
-        <v>113.343025767809</v>
-      </c>
-      <c r="N115" s="11">
-        <v>128.083347378882</v>
-      </c>
-      <c r="O115" s="11">
-        <v>139.43136468744001</v>
+        <v>2</v>
+      </c>
+      <c r="H115" s="10">
+        <v>4.0209035037549397</v>
+      </c>
+      <c r="I115" s="10">
+        <v>4.1352269590162702</v>
+      </c>
+      <c r="J115" s="10">
+        <v>4.0890994634011797</v>
+      </c>
+      <c r="K115" s="10">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="L115" s="10">
+        <v>103.38036423672099</v>
+      </c>
+      <c r="M115" s="10">
+        <v>103.99572480142</v>
+      </c>
+      <c r="N115" s="10">
+        <v>99.234147304171998</v>
+      </c>
+      <c r="O115" s="10">
+        <v>94.367099788090897</v>
       </c>
       <c r="P115">
-        <f t="shared" si="15"/>
-        <v>95.191061953990953</v>
+        <f t="shared" si="16"/>
+        <v>99.359460732966056</v>
       </c>
       <c r="Q115">
-        <f t="shared" si="16"/>
-        <v>104.50192820050154</v>
+        <f t="shared" si="17"/>
+        <v>99.860497842403731</v>
       </c>
       <c r="R115">
-        <f t="shared" si="17"/>
-        <v>118.27467890493114</v>
+        <f t="shared" si="18"/>
+        <v>95.145047840770815</v>
       </c>
       <c r="S115">
-        <f t="shared" si="18"/>
-        <v>128.22297576680302</v>
+        <f t="shared" si="19"/>
+        <v>90.259664086698052</v>
       </c>
     </row>
     <row r="116" spans="7:19" x14ac:dyDescent="0.25">
       <c r="G116" t="s">
-        <v>2</v>
-      </c>
-      <c r="H116" s="11">
-        <v>4.0209035037549397</v>
-      </c>
-      <c r="I116" s="11">
-        <v>4.1352269590162702</v>
-      </c>
-      <c r="J116" s="11">
-        <v>4.0890994634011797</v>
-      </c>
-      <c r="K116" s="11">
-        <v>4.1074357013928502</v>
-      </c>
-      <c r="L116" s="11">
-        <v>103.38036423672099</v>
-      </c>
-      <c r="M116" s="11">
-        <v>103.99572480142</v>
-      </c>
-      <c r="N116" s="11">
-        <v>99.234147304171998</v>
-      </c>
-      <c r="O116" s="11">
-        <v>94.367099788090897</v>
+        <v>13</v>
+      </c>
+      <c r="H116" s="10">
+        <v>6.9167933755607498</v>
+      </c>
+      <c r="I116" s="10">
+        <v>7.6918990911074498</v>
+      </c>
+      <c r="J116" s="10">
+        <v>8.6418529562595499</v>
+      </c>
+      <c r="K116" s="10">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="L116" s="10">
+        <v>101.70695238601699</v>
+      </c>
+      <c r="M116" s="10">
+        <v>110.026416640646</v>
+      </c>
+      <c r="N116" s="10">
+        <v>122.731095552444</v>
+      </c>
+      <c r="O116" s="10">
+        <v>138.09521327147601</v>
       </c>
       <c r="P116">
-        <f t="shared" si="15"/>
-        <v>99.359460732966056</v>
+        <f t="shared" si="16"/>
+        <v>94.79015901045625</v>
       </c>
       <c r="Q116">
-        <f t="shared" si="16"/>
-        <v>99.860497842403731</v>
+        <f t="shared" si="17"/>
+        <v>102.33451754953856</v>
       </c>
       <c r="R116">
-        <f t="shared" si="17"/>
-        <v>95.145047840770815</v>
+        <f t="shared" si="18"/>
+        <v>114.08924259618445</v>
       </c>
       <c r="S116">
-        <f t="shared" si="18"/>
-        <v>90.259664086698052</v>
-      </c>
-    </row>
-    <row r="117" spans="7:19" x14ac:dyDescent="0.25">
-      <c r="G117" t="s">
-        <v>13</v>
-      </c>
-      <c r="H117" s="11">
-        <v>6.9167933755607498</v>
-      </c>
-      <c r="I117" s="11">
-        <v>7.6918990911074498</v>
-      </c>
-      <c r="J117" s="11">
-        <v>8.6418529562595499</v>
-      </c>
-      <c r="K117" s="11">
-        <v>9.8390835440481492</v>
-      </c>
-      <c r="L117" s="11">
-        <v>101.70695238601699</v>
-      </c>
-      <c r="M117" s="11">
-        <v>110.026416640646</v>
-      </c>
-      <c r="N117" s="11">
-        <v>122.731095552444</v>
-      </c>
-      <c r="O117" s="11">
-        <v>138.09521327147601</v>
-      </c>
-      <c r="P117">
-        <f t="shared" si="15"/>
-        <v>94.79015901045625</v>
-      </c>
-      <c r="Q117">
-        <f t="shared" si="16"/>
-        <v>102.33451754953856</v>
-      </c>
-      <c r="R117">
-        <f t="shared" si="17"/>
-        <v>114.08924259618445</v>
-      </c>
-      <c r="S117">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>128.25612972742786</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="16">
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A57:F57"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F3:G3"/>
@@ -3525,7 +3607,6 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A11:B11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Add all visualizations and fine grain profiling
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4C3AB1-3950-41EB-8B79-F89D670EBEED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668D2FFF-2634-463C-AB29-AAEFC0C22C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="80">
   <si>
     <t>Functions</t>
   </si>
@@ -255,6 +255,27 @@
   </si>
   <si>
     <t>Baseline: 1</t>
+  </si>
+  <si>
+    <t>Baseline :</t>
+  </si>
+  <si>
+    <t>Baseline:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline: </t>
+  </si>
+  <si>
+    <t>M1: Internal Respone Time</t>
+  </si>
+  <si>
+    <t>M2: Internal Response Time</t>
+  </si>
+  <si>
+    <t>M4: Internal Response Time</t>
+  </si>
+  <si>
+    <t>M6: Internal Response Time</t>
   </si>
 </sst>
 </file>
@@ -865,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
-  <dimension ref="A1:S116"/>
+  <dimension ref="A1:S165"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -3409,7 +3430,7 @@
         <v>91.040105773481287</v>
       </c>
     </row>
-    <row r="113" spans="7:19" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="G113" t="s">
         <v>12</v>
       </c>
@@ -3454,7 +3475,7 @@
         <v>135.16902791535711</v>
       </c>
     </row>
-    <row r="114" spans="7:19" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="G114" t="s">
         <v>1</v>
       </c>
@@ -3499,7 +3520,7 @@
         <v>128.22297576680302</v>
       </c>
     </row>
-    <row r="115" spans="7:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="G115" t="s">
         <v>2</v>
       </c>
@@ -3544,7 +3565,7 @@
         <v>90.259664086698052</v>
       </c>
     </row>
-    <row r="116" spans="7:19" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
       <c r="G116" t="s">
         <v>13</v>
       </c>
@@ -3589,8 +3610,737 @@
         <v>128.25612972742786</v>
       </c>
     </row>
+    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A125" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B125" s="19"/>
+      <c r="C125" s="19"/>
+      <c r="D125" s="19"/>
+      <c r="E125" s="19"/>
+      <c r="F125" s="19"/>
+      <c r="G125" s="5"/>
+    </row>
+    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="D126" s="5"/>
+      <c r="F126" s="5"/>
+      <c r="G126" s="5"/>
+    </row>
+    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F127" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G127" s="17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>9</v>
+      </c>
+      <c r="B128">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="C128">
+        <v>1</v>
+      </c>
+      <c r="D128">
+        <v>1.7750263214111299</v>
+      </c>
+      <c r="E128" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F128" s="7"/>
+      <c r="G128">
+        <v>1.88845560695584</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>10</v>
+      </c>
+      <c r="B129">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="C129">
+        <v>1000</v>
+      </c>
+      <c r="D129">
+        <v>22.880792617797798</v>
+      </c>
+      <c r="E129" s="1">
+        <v>1.77403353154659</v>
+      </c>
+      <c r="F129" s="7"/>
+      <c r="G129">
+        <v>24.028556545575402</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>11</v>
+      </c>
+      <c r="B130">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="C130">
+        <v>1</v>
+      </c>
+      <c r="D130">
+        <v>0.46491622924804599</v>
+      </c>
+      <c r="E130" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F130" s="7"/>
+      <c r="G130">
+        <v>2.1100215528203101</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>12</v>
+      </c>
+      <c r="B131">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="C131">
+        <v>1000</v>
+      </c>
+      <c r="D131">
+        <v>15.479326248168899</v>
+      </c>
+      <c r="E131" s="1">
+        <v>1.77403353154659</v>
+      </c>
+      <c r="F131" s="7"/>
+      <c r="G131">
+        <v>21.906994919474698</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>1</v>
+      </c>
+      <c r="B132">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="C132">
+        <v>100</v>
+      </c>
+      <c r="D132">
+        <v>3.7736892700195299</v>
+      </c>
+      <c r="E132" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F132" s="7"/>
+      <c r="G132">
+        <v>3.5282435996756298</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>2</v>
+      </c>
+      <c r="B133">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="C133">
+        <v>1</v>
+      </c>
+      <c r="D133">
+        <v>0.19145011901855399</v>
+      </c>
+      <c r="E133" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F133" s="7"/>
+      <c r="G133">
+        <v>1.93604355925446</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>13</v>
+      </c>
+      <c r="B134">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="C134">
+        <v>100</v>
+      </c>
+      <c r="D134">
+        <v>3.9923191070556601</v>
+      </c>
+      <c r="E134" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F134" s="7"/>
+      <c r="G134">
+        <v>3.3641728812349001</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B135" s="1">
+        <v>18.626433459035201</v>
+      </c>
+      <c r="G135" s="1">
+        <v>10.456245141939799</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A137" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F137" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G137" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>9</v>
+      </c>
+      <c r="B138">
+        <v>4.0353076186722596</v>
+      </c>
+      <c r="C138">
+        <v>1</v>
+      </c>
+      <c r="D138">
+        <v>1.78432464599609</v>
+      </c>
+      <c r="E138" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F138" s="7"/>
+      <c r="G138">
+        <v>1.88845560695584</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>10</v>
+      </c>
+      <c r="B139">
+        <v>48.675797406364801</v>
+      </c>
+      <c r="C139">
+        <v>1000</v>
+      </c>
+      <c r="D139">
+        <v>20.764112472534102</v>
+      </c>
+      <c r="E139" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F139" s="7"/>
+      <c r="G139">
+        <v>24.028556545575402</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>11</v>
+      </c>
+      <c r="B140">
+        <v>4.1707241313894299</v>
+      </c>
+      <c r="C140">
+        <v>1</v>
+      </c>
+      <c r="D140">
+        <v>0.43320655822753901</v>
+      </c>
+      <c r="E140" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F140" s="7"/>
+      <c r="G140">
+        <v>2.1100215528203101</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>12</v>
+      </c>
+      <c r="B141">
+        <v>44.808815805147901</v>
+      </c>
+      <c r="C141">
+        <v>1000</v>
+      </c>
+      <c r="D141">
+        <v>14.152050018310501</v>
+      </c>
+      <c r="E141" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F141" s="7"/>
+      <c r="G141">
+        <v>21.906994919474698</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>1</v>
+      </c>
+      <c r="B142">
+        <v>9.8086684739508598</v>
+      </c>
+      <c r="C142">
+        <v>100</v>
+      </c>
+      <c r="D142">
+        <v>3.6182403564453098</v>
+      </c>
+      <c r="E142" s="1">
+        <v>0.170979648828506</v>
+      </c>
+      <c r="F142" s="7"/>
+      <c r="G142">
+        <v>3.5282435996756298</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>2</v>
+      </c>
+      <c r="B143">
+        <v>4.0890994634011797</v>
+      </c>
+      <c r="C143">
+        <v>1</v>
+      </c>
+      <c r="D143">
+        <v>0.30469894409179599</v>
+      </c>
+      <c r="E143" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F143" s="7"/>
+      <c r="G143">
+        <v>1.93604355925446</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>13</v>
+      </c>
+      <c r="B144">
+        <v>8.6418529562595499</v>
+      </c>
+      <c r="C144">
+        <v>100</v>
+      </c>
+      <c r="D144">
+        <v>3.2210350036621</v>
+      </c>
+      <c r="E144" s="1">
+        <v>0.170979648828506</v>
+      </c>
+      <c r="F144" s="7"/>
+      <c r="G144">
+        <v>3.3641728812349001</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B145" s="1">
+        <v>17.623530680131701</v>
+      </c>
+      <c r="G145" s="1">
+        <v>10.456245141939799</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D147" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E147" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F147" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G147" s="17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>9</v>
+      </c>
+      <c r="B148">
+        <v>4.02605646143118</v>
+      </c>
+      <c r="C148">
+        <v>1</v>
+      </c>
+      <c r="D148">
+        <v>1.7490386962890601</v>
+      </c>
+      <c r="E148" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F148" s="7"/>
+      <c r="G148">
+        <v>1.88845560695584</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>10</v>
+      </c>
+      <c r="B149">
+        <v>45.799138335569502</v>
+      </c>
+      <c r="C149">
+        <v>1000</v>
+      </c>
+      <c r="D149">
+        <v>19.1633701324462</v>
+      </c>
+      <c r="E149" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F149" s="7"/>
+      <c r="G149">
+        <v>24.028556545575402</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>11</v>
+      </c>
+      <c r="B150">
+        <v>4.1628384834501704</v>
+      </c>
+      <c r="C150">
+        <v>1</v>
+      </c>
+      <c r="D150">
+        <v>0.53834915161132801</v>
+      </c>
+      <c r="E150" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F150" s="7"/>
+      <c r="G150">
+        <v>2.1100215528203101</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>12</v>
+      </c>
+      <c r="B151">
+        <v>42.259016332980003</v>
+      </c>
+      <c r="C151">
+        <v>1000</v>
+      </c>
+      <c r="D151">
+        <v>12.4282836914062</v>
+      </c>
+      <c r="E151" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F151" s="7"/>
+      <c r="G151">
+        <v>21.906994919474698</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>1</v>
+      </c>
+      <c r="B152">
+        <v>8.8410975673074592</v>
+      </c>
+      <c r="C152">
+        <v>100</v>
+      </c>
+      <c r="D152">
+        <v>2.7823448181152299</v>
+      </c>
+      <c r="E152" s="1">
+        <v>0.16103312373161299</v>
+      </c>
+      <c r="F152" s="7"/>
+      <c r="G152">
+        <v>3.5282435996756298</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>2</v>
+      </c>
+      <c r="B153">
+        <v>4.1352269590162702</v>
+      </c>
+      <c r="C153">
+        <v>1</v>
+      </c>
+      <c r="D153">
+        <v>0.392913818359375</v>
+      </c>
+      <c r="E153" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F153" s="7"/>
+      <c r="G153">
+        <v>1.93604355925446</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>13</v>
+      </c>
+      <c r="B154">
+        <v>7.6918990911074498</v>
+      </c>
+      <c r="C154">
+        <v>100</v>
+      </c>
+      <c r="D154">
+        <v>2.16484069824218</v>
+      </c>
+      <c r="E154" s="1">
+        <v>0.16103312373161299</v>
+      </c>
+      <c r="F154" s="7"/>
+      <c r="G154">
+        <v>3.3641728812349001</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B155" s="1">
+        <v>16.466972683078801</v>
+      </c>
+      <c r="G155" s="1">
+        <v>10.456245141939799</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D157" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E157" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F157" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G157" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>9</v>
+      </c>
+      <c r="B158">
+        <v>3.9895902707595199</v>
+      </c>
+      <c r="C158">
+        <v>1</v>
+      </c>
+      <c r="D158">
+        <v>1.77168846130371</v>
+      </c>
+      <c r="E158" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F158" s="7"/>
+      <c r="G158">
+        <v>1.88845560695584</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>10</v>
+      </c>
+      <c r="B159">
+        <v>41.8466371823881</v>
+      </c>
+      <c r="C159">
+        <v>1000</v>
+      </c>
+      <c r="D159">
+        <v>16.952753067016602</v>
+      </c>
+      <c r="E159" s="1">
+        <v>1.54353864490985</v>
+      </c>
+      <c r="F159" s="7"/>
+      <c r="G159">
+        <v>24.028556545575402</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>11</v>
+      </c>
+      <c r="B160">
+        <v>4.0147860416504804</v>
+      </c>
+      <c r="C160">
+        <v>1</v>
+      </c>
+      <c r="D160">
+        <v>0.55480003356933505</v>
+      </c>
+      <c r="E160" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F160" s="7"/>
+      <c r="G160">
+        <v>2.1100215528203101</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>12</v>
+      </c>
+      <c r="B161">
+        <v>38.3633321341607</v>
+      </c>
+      <c r="C161">
+        <v>1000</v>
+      </c>
+      <c r="D161">
+        <v>11.2018585205078</v>
+      </c>
+      <c r="E161" s="1">
+        <v>1.54353864490985</v>
+      </c>
+      <c r="F161" s="7"/>
+      <c r="G161">
+        <v>21.906994919474698</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>1</v>
+      </c>
+      <c r="B162">
+        <v>7.9163517599320397</v>
+      </c>
+      <c r="C162">
+        <v>100</v>
+      </c>
+      <c r="D162">
+        <v>1.68442726135253</v>
+      </c>
+      <c r="E162" s="1">
+        <v>0.159744173288345</v>
+      </c>
+      <c r="F162" s="7"/>
+      <c r="G162">
+        <v>3.5282435996756298</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>2</v>
+      </c>
+      <c r="B163">
+        <v>4.0209035037549397</v>
+      </c>
+      <c r="C163">
+        <v>1</v>
+      </c>
+      <c r="D163">
+        <v>0.32210350036620999</v>
+      </c>
+      <c r="E163" s="1">
+        <v>4.3399631977081299E-3</v>
+      </c>
+      <c r="F163" s="7"/>
+      <c r="G163">
+        <v>1.93604355925446</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>13</v>
+      </c>
+      <c r="B164">
+        <v>6.9167933755607498</v>
+      </c>
+      <c r="C164">
+        <v>100</v>
+      </c>
+      <c r="D164">
+        <v>1.6908645629882799</v>
+      </c>
+      <c r="E164" s="1">
+        <v>0.159744173288345</v>
+      </c>
+      <c r="F164" s="7"/>
+      <c r="G164">
+        <v>3.3641728812349001</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B165" s="1">
+        <v>15.1045682929261</v>
+      </c>
+      <c r="G165" s="1">
+        <v>10.456245141939799</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="A125:F125"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="A40:B40"/>

</xml_diff>

<commit_message>
Add thesis draft latex
</commit_message>
<xml_diff>
--- a/Performance_Profiling/Response_Times_Measurement.xlsx
+++ b/Performance_Profiling/Response_Times_Measurement.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuSemesters\Semester Winter 2022_23\Bachelor Thesis\sharded-distributed-databases\Performance_Profiling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668D2FFF-2634-463C-AB29-AAEFC0C22C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E25AE6A-200C-409C-8662-F69765B57C73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="91">
   <si>
     <t>Functions</t>
   </si>
@@ -266,16 +266,49 @@
     <t xml:space="preserve">Baseline: </t>
   </si>
   <si>
-    <t>M1: Internal Respone Time</t>
-  </si>
-  <si>
-    <t>M2: Internal Response Time</t>
-  </si>
-  <si>
-    <t>M4: Internal Response Time</t>
-  </si>
-  <si>
-    <t>M6: Internal Response Time</t>
+    <t>Wait_Time + Other_Service Time</t>
+  </si>
+  <si>
+    <t>Service _Time_Sharding</t>
+  </si>
+  <si>
+    <t>M:6 - Service _Time</t>
+  </si>
+  <si>
+    <t>M:6 - DB Response Time</t>
+  </si>
+  <si>
+    <t>M:4 - DB Response Time</t>
+  </si>
+  <si>
+    <t>M:2 - DB Response Time</t>
+  </si>
+  <si>
+    <t>M:1 - DB Response Time</t>
+  </si>
+  <si>
+    <t>M:4 -Total Response Time</t>
+  </si>
+  <si>
+    <t>M:6 -Total Response Time</t>
+  </si>
+  <si>
+    <t>M:2 -Total Response Time</t>
+  </si>
+  <si>
+    <t>M:1 -Total Response Time</t>
+  </si>
+  <si>
+    <t>Load-Test Execution Report</t>
+  </si>
+  <si>
+    <t>M:4 - Service _Time</t>
+  </si>
+  <si>
+    <t>M:2 - Service _Time</t>
+  </si>
+  <si>
+    <t>M:1 - Service _Time</t>
   </si>
 </sst>
 </file>
@@ -285,7 +318,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +372,21 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -415,7 +463,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -538,8 +586,113 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -547,8 +700,9 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1"/>
@@ -567,10 +721,10 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="6" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -600,12 +754,37 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="14" xfId="4" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="13" xfId="6" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="15" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="16" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="17" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="19" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="20" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="20% - Accent5" xfId="5" builtinId="46"/>
     <cellStyle name="20% - Accent6" xfId="6" builtinId="50"/>
     <cellStyle name="40% - Accent4" xfId="4" builtinId="43"/>
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
+    <cellStyle name="Heading 1" xfId="7" builtinId="16"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Output" xfId="1" builtinId="21"/>
@@ -886,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2DFA73-0146-4B44-A73A-A03B2960D74C}">
-  <dimension ref="A1:S165"/>
+  <dimension ref="A1:S206"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
@@ -975,11 +1154,49 @@
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
+    <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
+      <c r="M8" s="34"/>
+      <c r="N8" s="34"/>
+      <c r="O8" s="34"/>
+      <c r="P8" s="35"/>
+    </row>
+    <row r="9" spans="1:16" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="36"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="37"/>
+      <c r="H9" s="37"/>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="38"/>
+    </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="18"/>
+      <c r="B11" s="19"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -1448,10 +1665,10 @@
       <c r="P20" s="15"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="19"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -1920,10 +2137,10 @@
       <c r="P34" s="15"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
+      <c r="A40" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B40" s="18"/>
+      <c r="B40" s="19"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
@@ -2403,30 +2620,22 @@
       <c r="G56" s="5"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="19" t="s">
+      <c r="A57" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B57" s="19"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
+      <c r="B57" s="18"/>
+      <c r="C57" s="18"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="18"/>
       <c r="G57" s="5"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="D58" s="5"/>
       <c r="F58" s="5"/>
       <c r="G58" s="5"/>
-      <c r="K58" t="s">
-        <v>9</v>
-      </c>
-      <c r="N58" s="3">
-        <v>0.52516379831418403</v>
-      </c>
-      <c r="O58" s="3">
-        <f t="shared" ref="O58:O64" si="15">N58-G90</f>
-        <v>0.19962707040891103</v>
-      </c>
+      <c r="N58" s="3"/>
+      <c r="O58" s="3"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
@@ -2450,16 +2659,7 @@
       <c r="G59" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="K59" t="s">
-        <v>10</v>
-      </c>
-      <c r="N59">
-        <v>32.977948012191398</v>
-      </c>
-      <c r="O59" s="3">
-        <f t="shared" si="15"/>
-        <v>19.1043947361294</v>
-      </c>
+      <c r="O59" s="3"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
@@ -2483,16 +2683,7 @@
       <c r="G60">
         <v>0.32553672790527299</v>
       </c>
-      <c r="K60" t="s">
-        <v>11</v>
-      </c>
-      <c r="N60">
-        <v>0.49840760395546102</v>
-      </c>
-      <c r="O60" s="3">
-        <f t="shared" si="15"/>
-        <v>0.33232522175331303</v>
-      </c>
+      <c r="O60" s="3"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
@@ -2516,16 +2707,7 @@
       <c r="G61">
         <v>13.873553276061999</v>
       </c>
-      <c r="K61" t="s">
-        <v>12</v>
-      </c>
-      <c r="N61">
-        <v>25.759887776849901</v>
-      </c>
-      <c r="O61" s="3">
-        <f t="shared" si="15"/>
-        <v>16.615271649835741</v>
-      </c>
+      <c r="O61" s="3"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
@@ -2549,16 +2731,7 @@
       <c r="G62">
         <v>0.16608238220214799</v>
       </c>
-      <c r="K62" t="s">
-        <v>1</v>
-      </c>
-      <c r="N62">
-        <v>3.52255095970304</v>
-      </c>
-      <c r="O62" s="3">
-        <f t="shared" si="15"/>
-        <v>2.1187900496688701</v>
-      </c>
+      <c r="O62" s="3"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
@@ -2582,16 +2755,8 @@
       <c r="G63">
         <v>9.1446161270141602</v>
       </c>
-      <c r="K63" t="s">
-        <v>2</v>
-      </c>
-      <c r="N63" s="3">
-        <v>0.49062787411620901</v>
-      </c>
-      <c r="O63" s="3">
-        <f t="shared" si="15"/>
-        <v>0.36078511593749901</v>
-      </c>
+      <c r="N63" s="3"/>
+      <c r="O63" s="3"/>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
@@ -2615,16 +2780,7 @@
       <c r="G64">
         <v>1.4037609100341699</v>
       </c>
-      <c r="K64" t="s">
-        <v>13</v>
-      </c>
-      <c r="N64">
-        <v>3.1790446098824598</v>
-      </c>
-      <c r="O64" s="3">
-        <f t="shared" si="15"/>
-        <v>1.89718711934291</v>
-      </c>
+      <c r="O64" s="3"/>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
@@ -3369,19 +3525,19 @@
         <v>207.255575950614</v>
       </c>
       <c r="P111">
-        <f t="shared" ref="P111:P116" si="16">L111-H111</f>
+        <f t="shared" ref="P111:P116" si="15">L111-H111</f>
         <v>157.03187925323491</v>
       </c>
       <c r="Q111">
-        <f t="shared" ref="Q111:Q116" si="17">M111-I111</f>
+        <f t="shared" ref="Q111:Q116" si="16">M111-I111</f>
         <v>147.76588772604052</v>
       </c>
       <c r="R111">
-        <f t="shared" ref="R111:R116" si="18">N111-J111</f>
+        <f t="shared" ref="R111:R116" si="17">N111-J111</f>
         <v>155.85102568547418</v>
       </c>
       <c r="S111">
-        <f t="shared" ref="S111:S116" si="19">O111-K111</f>
+        <f t="shared" ref="S111:S116" si="18">O111-K111</f>
         <v>152.74405156852231</v>
       </c>
     </row>
@@ -3414,19 +3570,19 @@
         <v>95.117645530865104</v>
       </c>
       <c r="P112">
+        <f t="shared" si="15"/>
+        <v>100.68493520511052</v>
+      </c>
+      <c r="Q112">
         <f t="shared" si="16"/>
-        <v>100.68493520511052</v>
-      </c>
-      <c r="Q112">
+        <v>99.013575153085824</v>
+      </c>
+      <c r="R112">
         <f t="shared" si="17"/>
-        <v>99.013575153085824</v>
-      </c>
-      <c r="R112">
+        <v>96.758430648757567</v>
+      </c>
+      <c r="S112">
         <f t="shared" si="18"/>
-        <v>96.758430648757567</v>
-      </c>
-      <c r="S112">
-        <f t="shared" si="19"/>
         <v>91.040105773481287</v>
       </c>
     </row>
@@ -3459,19 +3615,19 @@
         <v>182.358312283896</v>
       </c>
       <c r="P113">
+        <f t="shared" si="15"/>
+        <v>126.16151822702629</v>
+      </c>
+      <c r="Q113">
         <f t="shared" si="16"/>
-        <v>126.16151822702629</v>
-      </c>
-      <c r="Q113">
+        <v>130.281642551256</v>
+      </c>
+      <c r="R113">
         <f t="shared" si="17"/>
-        <v>130.281642551256</v>
-      </c>
-      <c r="R113">
+        <v>138.4221832693801</v>
+      </c>
+      <c r="S113">
         <f t="shared" si="18"/>
-        <v>138.4221832693801</v>
-      </c>
-      <c r="S113">
-        <f t="shared" si="19"/>
         <v>135.16902791535711</v>
       </c>
     </row>
@@ -3504,19 +3660,19 @@
         <v>139.43136468744001</v>
       </c>
       <c r="P114">
+        <f t="shared" si="15"/>
+        <v>95.191061953990953</v>
+      </c>
+      <c r="Q114">
         <f t="shared" si="16"/>
-        <v>95.191061953990953</v>
-      </c>
-      <c r="Q114">
+        <v>104.50192820050154</v>
+      </c>
+      <c r="R114">
         <f t="shared" si="17"/>
-        <v>104.50192820050154</v>
-      </c>
-      <c r="R114">
+        <v>118.27467890493114</v>
+      </c>
+      <c r="S114">
         <f t="shared" si="18"/>
-        <v>118.27467890493114</v>
-      </c>
-      <c r="S114">
-        <f t="shared" si="19"/>
         <v>128.22297576680302</v>
       </c>
     </row>
@@ -3549,19 +3705,19 @@
         <v>94.367099788090897</v>
       </c>
       <c r="P115">
+        <f t="shared" si="15"/>
+        <v>99.359460732966056</v>
+      </c>
+      <c r="Q115">
         <f t="shared" si="16"/>
-        <v>99.359460732966056</v>
-      </c>
-      <c r="Q115">
+        <v>99.860497842403731</v>
+      </c>
+      <c r="R115">
         <f t="shared" si="17"/>
-        <v>99.860497842403731</v>
-      </c>
-      <c r="R115">
+        <v>95.145047840770815</v>
+      </c>
+      <c r="S115">
         <f t="shared" si="18"/>
-        <v>95.145047840770815</v>
-      </c>
-      <c r="S115">
-        <f t="shared" si="19"/>
         <v>90.259664086698052</v>
       </c>
     </row>
@@ -3594,757 +3750,1234 @@
         <v>138.09521327147601</v>
       </c>
       <c r="P116">
+        <f t="shared" si="15"/>
+        <v>94.79015901045625</v>
+      </c>
+      <c r="Q116">
         <f t="shared" si="16"/>
-        <v>94.79015901045625</v>
-      </c>
-      <c r="Q116">
+        <v>102.33451754953856</v>
+      </c>
+      <c r="R116">
         <f t="shared" si="17"/>
-        <v>102.33451754953856</v>
-      </c>
-      <c r="R116">
+        <v>114.08924259618445</v>
+      </c>
+      <c r="S116">
         <f t="shared" si="18"/>
-        <v>114.08924259618445</v>
-      </c>
-      <c r="S116">
+        <v>128.25612972742786</v>
+      </c>
+    </row>
+    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A125" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="B125" s="18"/>
+      <c r="C125" s="18"/>
+      <c r="D125" s="18"/>
+      <c r="E125" s="18"/>
+      <c r="F125" s="18"/>
+      <c r="G125" s="18"/>
+    </row>
+    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="D127" s="5"/>
+      <c r="E127" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="F127" s="32"/>
+      <c r="G127" s="5"/>
+    </row>
+    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A128" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F128" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="G128" s="31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>9</v>
+      </c>
+      <c r="B129">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="C129">
+        <v>1</v>
+      </c>
+      <c r="D129">
+        <v>1.7750263214111299</v>
+      </c>
+      <c r="E129" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F129" s="7">
+        <f>B129-D129-E129</f>
+        <v>2.2256821122926898</v>
+      </c>
+      <c r="G129" s="29">
+        <v>2.9033422470092698</v>
+      </c>
+      <c r="I129">
+        <f>B129-D129</f>
+        <v>2.2300667789739794</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>10</v>
+      </c>
+      <c r="B130">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="C130">
+        <v>1000</v>
+      </c>
+      <c r="D130">
+        <v>22.880792617797798</v>
+      </c>
+      <c r="E130" s="1">
+        <v>1.77403353154659</v>
+      </c>
+      <c r="F130" s="7">
+        <f t="shared" ref="F130:F135" si="19">B130-D130-E130</f>
+        <v>29.856698232747313</v>
+      </c>
+      <c r="G130" s="29">
+        <v>26.091575622558501</v>
+      </c>
+      <c r="I130">
+        <f t="shared" ref="I130:I135" si="20">B130-D130</f>
+        <v>31.630731764293902</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>11</v>
+      </c>
+      <c r="B131">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="C131">
+        <v>1</v>
+      </c>
+      <c r="D131">
+        <v>0.46491622924804599</v>
+      </c>
+      <c r="E131" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F131" s="7">
         <f t="shared" si="19"/>
-        <v>128.25612972742786</v>
-      </c>
-    </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A125" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B125" s="19"/>
-      <c r="C125" s="19"/>
-      <c r="D125" s="19"/>
-      <c r="E125" s="19"/>
-      <c r="F125" s="19"/>
-      <c r="G125" s="5"/>
-    </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="D126" s="5"/>
-      <c r="F126" s="5"/>
-      <c r="G126" s="5"/>
-    </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A127" s="2" t="s">
+        <v>3.6082388614544847</v>
+      </c>
+      <c r="G131" s="29">
+        <v>1.69188976287841</v>
+      </c>
+      <c r="I131">
+        <f t="shared" si="20"/>
+        <v>3.6126235281357744</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>12</v>
+      </c>
+      <c r="B132">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="C132">
+        <v>1000</v>
+      </c>
+      <c r="D132">
+        <v>15.479326248168899</v>
+      </c>
+      <c r="E132" s="1">
+        <v>1.77403353154659</v>
+      </c>
+      <c r="F132" s="7">
+        <f t="shared" si="19"/>
+        <v>29.935924588823411</v>
+      </c>
+      <c r="G132" s="29">
+        <v>21.43235206604</v>
+      </c>
+      <c r="I132">
+        <f t="shared" si="20"/>
+        <v>31.709958120370001</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>1</v>
+      </c>
+      <c r="B133">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="C133">
+        <v>100</v>
+      </c>
+      <c r="D133">
+        <v>3.7736892700195299</v>
+      </c>
+      <c r="E133" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F133" s="7">
+        <f t="shared" si="19"/>
+        <v>7.2338375856598534</v>
+      </c>
+      <c r="G133" s="29">
+        <v>3.04076671600341</v>
+      </c>
+      <c r="I133">
+        <f t="shared" si="20"/>
+        <v>7.4346996506174712</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>2</v>
+      </c>
+      <c r="B134">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="C134">
+        <v>1</v>
+      </c>
+      <c r="D134">
+        <v>0.19145011901855399</v>
+      </c>
+      <c r="E134" s="1">
+        <v>4.3846666812896702E-3</v>
+      </c>
+      <c r="F134" s="7">
+        <f t="shared" si="19"/>
+        <v>3.9116009156930067</v>
+      </c>
+      <c r="G134" s="29">
+        <v>1.4133214950561499</v>
+      </c>
+      <c r="I134">
+        <f t="shared" si="20"/>
+        <v>3.9159855823742964</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>13</v>
+      </c>
+      <c r="B135">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="C135">
+        <v>100</v>
+      </c>
+      <c r="D135">
+        <v>3.9923191070556601</v>
+      </c>
+      <c r="E135" s="1">
+        <v>0.20086206495761799</v>
+      </c>
+      <c r="F135" s="7">
+        <f t="shared" si="19"/>
+        <v>5.6459023720348709</v>
+      </c>
+      <c r="G135" s="29">
+        <v>3.1214237213134699</v>
+      </c>
+      <c r="I135">
+        <f t="shared" si="20"/>
+        <v>5.8467644369924887</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B136" s="1">
+        <v>18.626433459035201</v>
+      </c>
+      <c r="G136" s="15">
+        <f>AVERAGE(G129:G135)</f>
+        <v>8.5278102329798884</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B137" s="1"/>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B138" s="1"/>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E139" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="F139" s="32"/>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A140" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B127" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C127" s="2" t="s">
+      <c r="B140" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C140" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D127" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F127" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G127" s="17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
+      <c r="D140" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F140" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="G140" s="31" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
         <v>9</v>
       </c>
-      <c r="B128">
-        <v>4.0050931003851096</v>
-      </c>
-      <c r="C128">
+      <c r="B141">
+        <v>4.0353076186722596</v>
+      </c>
+      <c r="C141">
         <v>1</v>
       </c>
-      <c r="D128">
-        <v>1.7750263214111299</v>
-      </c>
-      <c r="E128" s="1">
-        <v>4.3846666812896702E-3</v>
-      </c>
-      <c r="F128" s="7"/>
-      <c r="G128">
-        <v>1.88845560695584</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+      <c r="D141">
+        <v>1.78432464599609</v>
+      </c>
+      <c r="E141" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F141" s="7">
+        <f>B141-D141-E141</f>
+        <v>2.2466281083172674</v>
+      </c>
+      <c r="G141" s="29">
+        <v>2.9033422470092698</v>
+      </c>
+      <c r="I141">
+        <f>B141-D141</f>
+        <v>2.2509829726761694</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
         <v>10</v>
       </c>
-      <c r="B129">
-        <v>54.5115243820917</v>
-      </c>
-      <c r="C129">
+      <c r="B142">
+        <v>48.675797406364801</v>
+      </c>
+      <c r="C142">
         <v>1000</v>
       </c>
-      <c r="D129">
-        <v>22.880792617797798</v>
-      </c>
-      <c r="E129" s="1">
-        <v>1.77403353154659</v>
-      </c>
-      <c r="F129" s="7"/>
-      <c r="G129">
-        <v>24.028556545575402</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
+      <c r="D142">
+        <v>20.764112472534102</v>
+      </c>
+      <c r="E142" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F142" s="7">
+        <f t="shared" ref="F142:F147" si="21">B142-D142-E142</f>
+        <v>26.301605153609721</v>
+      </c>
+      <c r="G142" s="29">
+        <v>26.091575622558501</v>
+      </c>
+      <c r="I142">
+        <f t="shared" ref="I142:I147" si="22">B142-D142</f>
+        <v>27.911684933830699</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
         <v>11</v>
       </c>
-      <c r="B130">
-        <v>4.0775397573838204</v>
-      </c>
-      <c r="C130">
-        <v>1</v>
-      </c>
-      <c r="D130">
-        <v>0.46491622924804599</v>
-      </c>
-      <c r="E130" s="1">
-        <v>4.3846666812896702E-3</v>
-      </c>
-      <c r="F130" s="7"/>
-      <c r="G130">
-        <v>2.1100215528203101</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>12</v>
-      </c>
-      <c r="B131">
-        <v>47.1892843685389</v>
-      </c>
-      <c r="C131">
-        <v>1000</v>
-      </c>
-      <c r="D131">
-        <v>15.479326248168899</v>
-      </c>
-      <c r="E131" s="1">
-        <v>1.77403353154659</v>
-      </c>
-      <c r="F131" s="7"/>
-      <c r="G131">
-        <v>21.906994919474698</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>1</v>
-      </c>
-      <c r="B132">
-        <v>11.208388920637001</v>
-      </c>
-      <c r="C132">
-        <v>100</v>
-      </c>
-      <c r="D132">
-        <v>3.7736892700195299</v>
-      </c>
-      <c r="E132" s="1">
-        <v>0.20086206495761799</v>
-      </c>
-      <c r="F132" s="7"/>
-      <c r="G132">
-        <v>3.5282435996756298</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>2</v>
-      </c>
-      <c r="B133">
-        <v>4.1074357013928502</v>
-      </c>
-      <c r="C133">
-        <v>1</v>
-      </c>
-      <c r="D133">
-        <v>0.19145011901855399</v>
-      </c>
-      <c r="E133" s="1">
-        <v>4.3846666812896702E-3</v>
-      </c>
-      <c r="F133" s="7"/>
-      <c r="G133">
-        <v>1.93604355925446</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>13</v>
-      </c>
-      <c r="B134">
-        <v>9.8390835440481492</v>
-      </c>
-      <c r="C134">
-        <v>100</v>
-      </c>
-      <c r="D134">
-        <v>3.9923191070556601</v>
-      </c>
-      <c r="E134" s="1">
-        <v>0.20086206495761799</v>
-      </c>
-      <c r="F134" s="7"/>
-      <c r="G134">
-        <v>3.3641728812349001</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B135" s="1">
-        <v>18.626433459035201</v>
-      </c>
-      <c r="G135" s="1">
-        <v>10.456245141939799</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A137" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C137" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="E137" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F137" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G137" s="17" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>9</v>
-      </c>
-      <c r="B138">
-        <v>4.0353076186722596</v>
-      </c>
-      <c r="C138">
-        <v>1</v>
-      </c>
-      <c r="D138">
-        <v>1.78432464599609</v>
-      </c>
-      <c r="E138" s="1">
-        <v>4.3548643589019697E-3</v>
-      </c>
-      <c r="F138" s="7"/>
-      <c r="G138">
-        <v>1.88845560695584</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>10</v>
-      </c>
-      <c r="B139">
-        <v>48.675797406364801</v>
-      </c>
-      <c r="C139">
-        <v>1000</v>
-      </c>
-      <c r="D139">
-        <v>20.764112472534102</v>
-      </c>
-      <c r="E139" s="1">
-        <v>1.6100797802209801</v>
-      </c>
-      <c r="F139" s="7"/>
-      <c r="G139">
-        <v>24.028556545575402</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>11</v>
-      </c>
-      <c r="B140">
+      <c r="B143">
         <v>4.1707241313894299</v>
-      </c>
-      <c r="C140">
-        <v>1</v>
-      </c>
-      <c r="D140">
-        <v>0.43320655822753901</v>
-      </c>
-      <c r="E140" s="1">
-        <v>4.3548643589019697E-3</v>
-      </c>
-      <c r="F140" s="7"/>
-      <c r="G140">
-        <v>2.1100215528203101</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>12</v>
-      </c>
-      <c r="B141">
-        <v>44.808815805147901</v>
-      </c>
-      <c r="C141">
-        <v>1000</v>
-      </c>
-      <c r="D141">
-        <v>14.152050018310501</v>
-      </c>
-      <c r="E141" s="1">
-        <v>1.6100797802209801</v>
-      </c>
-      <c r="F141" s="7"/>
-      <c r="G141">
-        <v>21.906994919474698</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>1</v>
-      </c>
-      <c r="B142">
-        <v>9.8086684739508598</v>
-      </c>
-      <c r="C142">
-        <v>100</v>
-      </c>
-      <c r="D142">
-        <v>3.6182403564453098</v>
-      </c>
-      <c r="E142" s="1">
-        <v>0.170979648828506</v>
-      </c>
-      <c r="F142" s="7"/>
-      <c r="G142">
-        <v>3.5282435996756298</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>2</v>
-      </c>
-      <c r="B143">
-        <v>4.0890994634011797</v>
       </c>
       <c r="C143">
         <v>1</v>
       </c>
       <c r="D143">
-        <v>0.30469894409179599</v>
+        <v>0.43320655822753901</v>
       </c>
       <c r="E143" s="1">
         <v>4.3548643589019697E-3</v>
       </c>
-      <c r="F143" s="7"/>
-      <c r="G143">
-        <v>1.93604355925446</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F143" s="7">
+        <f t="shared" si="21"/>
+        <v>3.7331627088029888</v>
+      </c>
+      <c r="G143" s="29">
+        <v>1.69188976287841</v>
+      </c>
+      <c r="I143">
+        <f t="shared" si="22"/>
+        <v>3.7375175731618908</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>12</v>
+      </c>
+      <c r="B144">
+        <v>44.808815805147901</v>
+      </c>
+      <c r="C144">
+        <v>1000</v>
+      </c>
+      <c r="D144">
+        <v>14.152050018310501</v>
+      </c>
+      <c r="E144" s="1">
+        <v>1.6100797802209801</v>
+      </c>
+      <c r="F144" s="7">
+        <f t="shared" si="21"/>
+        <v>29.046686006616419</v>
+      </c>
+      <c r="G144" s="29">
+        <v>21.43235206604</v>
+      </c>
+      <c r="I144">
+        <f t="shared" si="22"/>
+        <v>30.656765786837401</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>1</v>
+      </c>
+      <c r="B145">
+        <v>9.8086684739508598</v>
+      </c>
+      <c r="C145">
+        <v>100</v>
+      </c>
+      <c r="D145">
+        <v>3.6182403564453098</v>
+      </c>
+      <c r="E145" s="1">
+        <v>0.170979648828506</v>
+      </c>
+      <c r="F145" s="7">
+        <f t="shared" si="21"/>
+        <v>6.0194484686770444</v>
+      </c>
+      <c r="G145" s="29">
+        <v>3.04076671600341</v>
+      </c>
+      <c r="I145">
+        <f t="shared" si="22"/>
+        <v>6.19042811750555</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>2</v>
+      </c>
+      <c r="B146">
+        <v>4.0890994634011797</v>
+      </c>
+      <c r="C146">
+        <v>1</v>
+      </c>
+      <c r="D146">
+        <v>0.30469894409179599</v>
+      </c>
+      <c r="E146" s="1">
+        <v>4.3548643589019697E-3</v>
+      </c>
+      <c r="F146" s="7">
+        <f t="shared" si="21"/>
+        <v>3.7800456549504817</v>
+      </c>
+      <c r="G146" s="29">
+        <v>1.4133214950561499</v>
+      </c>
+      <c r="I146">
+        <f t="shared" si="22"/>
+        <v>3.7844005193093837</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>13</v>
       </c>
-      <c r="B144">
+      <c r="B147">
         <v>8.6418529562595499</v>
       </c>
-      <c r="C144">
+      <c r="C147">
         <v>100</v>
       </c>
-      <c r="D144">
+      <c r="D147">
         <v>3.2210350036621</v>
       </c>
-      <c r="E144" s="1">
+      <c r="E147" s="1">
         <v>0.170979648828506</v>
       </c>
-      <c r="F144" s="7"/>
-      <c r="G144">
-        <v>3.3641728812349001</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B145" s="1">
+      <c r="F147" s="7">
+        <f t="shared" si="21"/>
+        <v>5.2498383037689438</v>
+      </c>
+      <c r="G147" s="29">
+        <v>3.1214237213134699</v>
+      </c>
+      <c r="I147">
+        <f t="shared" si="22"/>
+        <v>5.4208179525974494</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B148" s="1">
         <v>17.623530680131701</v>
       </c>
-      <c r="G145" s="1">
-        <v>10.456245141939799</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A147" s="2" t="s">
+      <c r="G148" s="15">
+        <f>AVERAGE(G141:G147)</f>
+        <v>8.5278102329798884</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B149" s="1"/>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B150" s="1"/>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E151" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="F151" s="32"/>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A152" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B147" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C147" s="2" t="s">
+      <c r="B152" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C152" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D147" s="2" t="s">
+      <c r="D152" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E147" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F147" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G147" s="17" t="s">
+      <c r="F152" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="G152" s="31" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
         <v>9</v>
       </c>
-      <c r="B148">
+      <c r="B153">
         <v>4.02605646143118</v>
-      </c>
-      <c r="C148">
-        <v>1</v>
-      </c>
-      <c r="D148">
-        <v>1.7490386962890601</v>
-      </c>
-      <c r="E148" s="1">
-        <v>3.89851629734039E-3</v>
-      </c>
-      <c r="F148" s="7"/>
-      <c r="G148">
-        <v>1.88845560695584</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>10</v>
-      </c>
-      <c r="B149">
-        <v>45.799138335569502</v>
-      </c>
-      <c r="C149">
-        <v>1000</v>
-      </c>
-      <c r="D149">
-        <v>19.1633701324462</v>
-      </c>
-      <c r="E149" s="1">
-        <v>1.62918865680694</v>
-      </c>
-      <c r="F149" s="7"/>
-      <c r="G149">
-        <v>24.028556545575402</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>11</v>
-      </c>
-      <c r="B150">
-        <v>4.1628384834501704</v>
-      </c>
-      <c r="C150">
-        <v>1</v>
-      </c>
-      <c r="D150">
-        <v>0.53834915161132801</v>
-      </c>
-      <c r="E150" s="1">
-        <v>3.89851629734039E-3</v>
-      </c>
-      <c r="F150" s="7"/>
-      <c r="G150">
-        <v>2.1100215528203101</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>12</v>
-      </c>
-      <c r="B151">
-        <v>42.259016332980003</v>
-      </c>
-      <c r="C151">
-        <v>1000</v>
-      </c>
-      <c r="D151">
-        <v>12.4282836914062</v>
-      </c>
-      <c r="E151" s="1">
-        <v>1.62918865680694</v>
-      </c>
-      <c r="F151" s="7"/>
-      <c r="G151">
-        <v>21.906994919474698</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>1</v>
-      </c>
-      <c r="B152">
-        <v>8.8410975673074592</v>
-      </c>
-      <c r="C152">
-        <v>100</v>
-      </c>
-      <c r="D152">
-        <v>2.7823448181152299</v>
-      </c>
-      <c r="E152" s="1">
-        <v>0.16103312373161299</v>
-      </c>
-      <c r="F152" s="7"/>
-      <c r="G152">
-        <v>3.5282435996756298</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A153" t="s">
-        <v>2</v>
-      </c>
-      <c r="B153">
-        <v>4.1352269590162702</v>
       </c>
       <c r="C153">
         <v>1</v>
       </c>
       <c r="D153">
-        <v>0.392913818359375</v>
+        <v>1.7490386962890601</v>
       </c>
       <c r="E153" s="1">
         <v>3.89851629734039E-3</v>
       </c>
-      <c r="F153" s="7"/>
-      <c r="G153">
-        <v>1.93604355925446</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F153" s="7">
+        <f>B153-D153-E153</f>
+        <v>2.2731192488447798</v>
+      </c>
+      <c r="G153" s="29">
+        <v>2.9033422470092698</v>
+      </c>
+      <c r="I153">
+        <f>B153-D153</f>
+        <v>2.2770177651421202</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B154">
-        <v>7.6918990911074498</v>
+        <v>45.799138335569502</v>
       </c>
       <c r="C154">
+        <v>1000</v>
+      </c>
+      <c r="D154">
+        <v>19.1633701324462</v>
+      </c>
+      <c r="E154" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F154" s="7">
+        <f t="shared" ref="F154:F159" si="23">B154-D154-E154</f>
+        <v>25.006579546316363</v>
+      </c>
+      <c r="G154" s="29">
+        <v>26.091575622558501</v>
+      </c>
+      <c r="I154">
+        <f t="shared" ref="I154:I159" si="24">B154-D154</f>
+        <v>26.635768203123302</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>11</v>
+      </c>
+      <c r="B155">
+        <v>4.1628384834501704</v>
+      </c>
+      <c r="C155">
+        <v>1</v>
+      </c>
+      <c r="D155">
+        <v>0.53834915161132801</v>
+      </c>
+      <c r="E155" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F155" s="7">
+        <f t="shared" si="23"/>
+        <v>3.6205908155415019</v>
+      </c>
+      <c r="G155" s="29">
+        <v>1.69188976287841</v>
+      </c>
+      <c r="I155">
+        <f t="shared" si="24"/>
+        <v>3.6244893318388423</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>12</v>
+      </c>
+      <c r="B156">
+        <v>42.259016332980003</v>
+      </c>
+      <c r="C156">
+        <v>1000</v>
+      </c>
+      <c r="D156">
+        <v>12.4282836914062</v>
+      </c>
+      <c r="E156" s="1">
+        <v>1.62918865680694</v>
+      </c>
+      <c r="F156" s="7">
+        <f t="shared" si="23"/>
+        <v>28.201543984766865</v>
+      </c>
+      <c r="G156" s="29">
+        <v>21.43235206604</v>
+      </c>
+      <c r="I156">
+        <f t="shared" si="24"/>
+        <v>29.830732641573803</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>1</v>
+      </c>
+      <c r="B157">
+        <v>8.8410975673074592</v>
+      </c>
+      <c r="C157">
         <v>100</v>
       </c>
-      <c r="D154">
-        <v>2.16484069824218</v>
-      </c>
-      <c r="E154" s="1">
+      <c r="D157">
+        <v>2.7823448181152299</v>
+      </c>
+      <c r="E157" s="1">
         <v>0.16103312373161299</v>
       </c>
-      <c r="F154" s="7"/>
-      <c r="G154">
-        <v>3.3641728812349001</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B155" s="1">
-        <v>16.466972683078801</v>
-      </c>
-      <c r="G155" s="1">
-        <v>10.456245141939799</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A157" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B157" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C157" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D157" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="E157" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F157" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G157" s="17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F157" s="7">
+        <f t="shared" si="23"/>
+        <v>5.8977196254606161</v>
+      </c>
+      <c r="G157" s="29">
+        <v>3.04076671600341</v>
+      </c>
+      <c r="I157">
+        <f t="shared" si="24"/>
+        <v>6.0587527491922293</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B158">
-        <v>3.9895902707595199</v>
+        <v>4.1352269590162702</v>
       </c>
       <c r="C158">
         <v>1</v>
       </c>
       <c r="D158">
+        <v>0.392913818359375</v>
+      </c>
+      <c r="E158" s="1">
+        <v>3.89851629734039E-3</v>
+      </c>
+      <c r="F158" s="7">
+        <f t="shared" si="23"/>
+        <v>3.7384146243595548</v>
+      </c>
+      <c r="G158" s="29">
+        <v>1.4133214950561499</v>
+      </c>
+      <c r="I158">
+        <f t="shared" si="24"/>
+        <v>3.7423131406568952</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>13</v>
+      </c>
+      <c r="B159">
+        <v>7.6918990911074498</v>
+      </c>
+      <c r="C159">
+        <v>100</v>
+      </c>
+      <c r="D159">
+        <v>2.16484069824218</v>
+      </c>
+      <c r="E159" s="1">
+        <v>0.16103312373161299</v>
+      </c>
+      <c r="F159" s="7">
+        <f t="shared" si="23"/>
+        <v>5.3660252691336563</v>
+      </c>
+      <c r="G159" s="29">
+        <v>3.1214237213134699</v>
+      </c>
+      <c r="I159">
+        <f t="shared" si="24"/>
+        <v>5.5270583928652695</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B160" s="1">
+        <v>16.466972683078801</v>
+      </c>
+      <c r="G160" s="15">
+        <f>AVERAGE(G153:G159)</f>
+        <v>8.5278102329798884</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B161" s="1"/>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B162" s="1"/>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E163" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="F163" s="32"/>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A164" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C164" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D164" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E164" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F164" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="G164" s="31" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>9</v>
+      </c>
+      <c r="B165">
+        <v>3.9895902707595199</v>
+      </c>
+      <c r="C165">
+        <v>1</v>
+      </c>
+      <c r="D165">
         <v>1.77168846130371</v>
       </c>
-      <c r="E158" s="1">
+      <c r="E165" s="1">
         <v>4.3399631977081299E-3</v>
       </c>
-      <c r="F158" s="7"/>
-      <c r="G158">
-        <v>1.88845560695584</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A159" t="s">
+      <c r="F165" s="7">
+        <f>B165-D165-E165</f>
+        <v>2.2135618462581017</v>
+      </c>
+      <c r="G165" s="29">
+        <v>2.9033422470092698</v>
+      </c>
+      <c r="I165">
+        <f>B165-D165</f>
+        <v>2.2179018094558098</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
         <v>10</v>
       </c>
-      <c r="B159">
+      <c r="B166">
         <v>41.8466371823881</v>
       </c>
-      <c r="C159">
+      <c r="C166">
         <v>1000</v>
       </c>
-      <c r="D159">
+      <c r="D166">
         <v>16.952753067016602</v>
       </c>
-      <c r="E159" s="1">
+      <c r="E166" s="1">
         <v>1.54353864490985</v>
       </c>
-      <c r="F159" s="7"/>
-      <c r="G159">
-        <v>24.028556545575402</v>
-      </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A160" t="s">
+      <c r="F166" s="7">
+        <f t="shared" ref="F166:F171" si="25">B166-D166-E166</f>
+        <v>23.350345470461647</v>
+      </c>
+      <c r="G166" s="29">
+        <v>26.091575622558501</v>
+      </c>
+      <c r="I166">
+        <f t="shared" ref="I166:I171" si="26">B166-D166</f>
+        <v>24.893884115371499</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
         <v>11</v>
       </c>
-      <c r="B160">
+      <c r="B167">
         <v>4.0147860416504804</v>
       </c>
-      <c r="C160">
+      <c r="C167">
         <v>1</v>
       </c>
-      <c r="D160">
+      <c r="D167">
         <v>0.55480003356933505</v>
       </c>
-      <c r="E160" s="1">
+      <c r="E167" s="1">
         <v>4.3399631977081299E-3</v>
       </c>
-      <c r="F160" s="7"/>
-      <c r="G160">
-        <v>2.1100215528203101</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A161" t="s">
+      <c r="F167" s="7">
+        <f t="shared" si="25"/>
+        <v>3.4556460448834372</v>
+      </c>
+      <c r="G167" s="29">
+        <v>1.69188976287841</v>
+      </c>
+      <c r="I167">
+        <f t="shared" si="26"/>
+        <v>3.4599860080811453</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
         <v>12</v>
       </c>
-      <c r="B161">
+      <c r="B168">
         <v>38.3633321341607</v>
       </c>
-      <c r="C161">
+      <c r="C168">
         <v>1000</v>
       </c>
-      <c r="D161">
+      <c r="D168">
         <v>11.2018585205078</v>
       </c>
-      <c r="E161" s="1">
+      <c r="E168" s="1">
         <v>1.54353864490985</v>
       </c>
-      <c r="F161" s="7"/>
-      <c r="G161">
-        <v>21.906994919474698</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A162" t="s">
+      <c r="F168" s="7">
+        <f t="shared" si="25"/>
+        <v>25.61793496874305</v>
+      </c>
+      <c r="G168" s="29">
+        <v>21.43235206604</v>
+      </c>
+      <c r="I168">
+        <f t="shared" si="26"/>
+        <v>27.161473613652902</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
         <v>1</v>
       </c>
-      <c r="B162">
+      <c r="B169">
         <v>7.9163517599320397</v>
       </c>
-      <c r="C162">
+      <c r="C169">
         <v>100</v>
       </c>
-      <c r="D162">
+      <c r="D169">
         <v>1.68442726135253</v>
       </c>
-      <c r="E162" s="1">
+      <c r="E169" s="1">
         <v>0.159744173288345</v>
       </c>
-      <c r="F162" s="7"/>
-      <c r="G162">
-        <v>3.5282435996756298</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A163" t="s">
+      <c r="F169" s="7">
+        <f t="shared" si="25"/>
+        <v>6.0721803252911641</v>
+      </c>
+      <c r="G169" s="29">
+        <v>3.04076671600341</v>
+      </c>
+      <c r="I169">
+        <f t="shared" si="26"/>
+        <v>6.2319244985795095</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
         <v>2</v>
       </c>
-      <c r="B163">
+      <c r="B170">
         <v>4.0209035037549397</v>
       </c>
-      <c r="C163">
+      <c r="C170">
         <v>1</v>
       </c>
-      <c r="D163">
+      <c r="D170">
         <v>0.32210350036620999</v>
       </c>
-      <c r="E163" s="1">
+      <c r="E170" s="1">
         <v>4.3399631977081299E-3</v>
       </c>
-      <c r="F163" s="7"/>
-      <c r="G163">
-        <v>1.93604355925446</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A164" t="s">
+      <c r="F170" s="7">
+        <f t="shared" si="25"/>
+        <v>3.6944600401910215</v>
+      </c>
+      <c r="G170" s="29">
+        <v>1.4133214950561499</v>
+      </c>
+      <c r="I170">
+        <f t="shared" si="26"/>
+        <v>3.6988000033887296</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
         <v>13</v>
       </c>
-      <c r="B164">
+      <c r="B171">
         <v>6.9167933755607498</v>
       </c>
-      <c r="C164">
+      <c r="C171">
         <v>100</v>
       </c>
-      <c r="D164">
+      <c r="D171">
         <v>1.6908645629882799</v>
       </c>
-      <c r="E164" s="1">
+      <c r="E171" s="1">
         <v>0.159744173288345</v>
       </c>
-      <c r="F164" s="7"/>
-      <c r="G164">
-        <v>3.3641728812349001</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B165" s="1">
+      <c r="F171" s="7">
+        <f t="shared" si="25"/>
+        <v>5.0661846392841241</v>
+      </c>
+      <c r="G171" s="29">
+        <v>3.1214237213134699</v>
+      </c>
+      <c r="I171">
+        <f t="shared" si="26"/>
+        <v>5.2259288125724694</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B172" s="1">
         <v>15.1045682929261</v>
       </c>
-      <c r="G165" s="1">
-        <v>10.456245141939799</v>
+      <c r="G172" s="15">
+        <f>AVERAGE(G165:G171)</f>
+        <v>8.5278102329798884</v>
+      </c>
+    </row>
+    <row r="178" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D178" s="1">
+        <v>2.2770177651421202</v>
+      </c>
+      <c r="E178">
+        <f>ROUND(D178,4)</f>
+        <v>2.2770000000000001</v>
+      </c>
+    </row>
+    <row r="179" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D179" s="1">
+        <v>26.635768203123302</v>
+      </c>
+      <c r="E179">
+        <f>ROUND(D179,4)</f>
+        <v>26.6358</v>
+      </c>
+    </row>
+    <row r="180" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D180" s="1">
+        <v>3.6244893318388423</v>
+      </c>
+      <c r="E180">
+        <f>ROUND(D180,4)</f>
+        <v>3.6244999999999998</v>
+      </c>
+    </row>
+    <row r="181" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D181" s="1">
+        <v>29.830732641573803</v>
+      </c>
+      <c r="E181">
+        <f>ROUND(D181,4)</f>
+        <v>29.8307</v>
+      </c>
+    </row>
+    <row r="182" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D182" s="1">
+        <v>6.0587527491922293</v>
+      </c>
+      <c r="E182">
+        <f>ROUND(D182,4)</f>
+        <v>6.0587999999999997</v>
+      </c>
+    </row>
+    <row r="183" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D183" s="1">
+        <v>3.7423131406568952</v>
+      </c>
+      <c r="E183">
+        <f>ROUND(D183,4)</f>
+        <v>3.7423000000000002</v>
+      </c>
+    </row>
+    <row r="184" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D184" s="1">
+        <v>5.5270583928652695</v>
+      </c>
+      <c r="E184">
+        <f>ROUND(D184,4)</f>
+        <v>5.5270999999999999</v>
+      </c>
+    </row>
+    <row r="190" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B190">
+        <v>4.0050931003851096</v>
+      </c>
+      <c r="C190">
+        <v>1.7750263214111299</v>
+      </c>
+      <c r="D190">
+        <v>2.2300667789739794</v>
+      </c>
+    </row>
+    <row r="191" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B191">
+        <v>54.5115243820917</v>
+      </c>
+      <c r="C191">
+        <v>22.880792617797798</v>
+      </c>
+      <c r="D191">
+        <v>31.630731764293902</v>
+      </c>
+    </row>
+    <row r="192" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B192">
+        <v>4.0775397573838204</v>
+      </c>
+      <c r="C192">
+        <v>0.46491622924804599</v>
+      </c>
+      <c r="D192">
+        <v>3.6126235281357744</v>
+      </c>
+    </row>
+    <row r="193" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B193">
+        <v>47.1892843685389</v>
+      </c>
+      <c r="C193">
+        <v>15.479326248168899</v>
+      </c>
+      <c r="D193">
+        <v>31.709958120370001</v>
+      </c>
+    </row>
+    <row r="194" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B194">
+        <v>11.208388920637001</v>
+      </c>
+      <c r="C194">
+        <v>3.7736892700195299</v>
+      </c>
+      <c r="D194">
+        <v>7.4346996506174712</v>
+      </c>
+    </row>
+    <row r="195" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B195">
+        <v>4.1074357013928502</v>
+      </c>
+      <c r="C195">
+        <v>0.19145011901855399</v>
+      </c>
+      <c r="D195">
+        <v>3.9159855823742964</v>
+      </c>
+    </row>
+    <row r="196" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B196">
+        <v>9.8390835440481492</v>
+      </c>
+      <c r="C196">
+        <v>3.9923191070556601</v>
+      </c>
+      <c r="D196">
+        <v>5.8467644369924887</v>
+      </c>
+    </row>
+    <row r="200" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B200">
+        <f>ROUND(B190, 4)</f>
+        <v>4.0050999999999997</v>
+      </c>
+      <c r="C200">
+        <f>ROUND(C190, 4)</f>
+        <v>1.7749999999999999</v>
+      </c>
+      <c r="D200">
+        <f>ROUND(D190, 4)</f>
+        <v>2.2301000000000002</v>
+      </c>
+    </row>
+    <row r="201" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B201">
+        <f t="shared" ref="B201:D206" si="27">ROUND(B191, 4)</f>
+        <v>54.511499999999998</v>
+      </c>
+      <c r="C201">
+        <f t="shared" si="27"/>
+        <v>22.880800000000001</v>
+      </c>
+      <c r="D201">
+        <f t="shared" si="27"/>
+        <v>31.630700000000001</v>
+      </c>
+    </row>
+    <row r="202" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B202">
+        <f t="shared" si="27"/>
+        <v>4.0774999999999997</v>
+      </c>
+      <c r="C202">
+        <f t="shared" si="27"/>
+        <v>0.46489999999999998</v>
+      </c>
+      <c r="D202">
+        <f t="shared" si="27"/>
+        <v>3.6126</v>
+      </c>
+    </row>
+    <row r="203" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B203">
+        <f t="shared" si="27"/>
+        <v>47.189300000000003</v>
+      </c>
+      <c r="C203">
+        <f t="shared" si="27"/>
+        <v>15.4793</v>
+      </c>
+      <c r="D203">
+        <f t="shared" si="27"/>
+        <v>31.71</v>
+      </c>
+    </row>
+    <row r="204" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B204">
+        <f t="shared" si="27"/>
+        <v>11.208399999999999</v>
+      </c>
+      <c r="C204">
+        <f t="shared" si="27"/>
+        <v>3.7736999999999998</v>
+      </c>
+      <c r="D204">
+        <f t="shared" si="27"/>
+        <v>7.4347000000000003</v>
+      </c>
+    </row>
+    <row r="205" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B205">
+        <f t="shared" si="27"/>
+        <v>4.1074000000000002</v>
+      </c>
+      <c r="C205">
+        <f t="shared" si="27"/>
+        <v>0.1915</v>
+      </c>
+      <c r="D205">
+        <f t="shared" si="27"/>
+        <v>3.9159999999999999</v>
+      </c>
+    </row>
+    <row r="206" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B206">
+        <f t="shared" si="27"/>
+        <v>9.8391000000000002</v>
+      </c>
+      <c r="C206">
+        <f t="shared" si="27"/>
+        <v>3.9923000000000002</v>
+      </c>
+      <c r="D206">
+        <f t="shared" si="27"/>
+        <v>5.8468</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A125:F125"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A57:F57"/>
+  <mergeCells count="22">
+    <mergeCell ref="A8:P9"/>
+    <mergeCell ref="E127:F127"/>
+    <mergeCell ref="E139:F139"/>
+    <mergeCell ref="E151:F151"/>
+    <mergeCell ref="E163:F163"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="F3:G3"/>
@@ -4357,6 +4990,11 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A125:G125"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>